<commit_message>
Finmodel tabs 3-4: single before/after block from Ukrainian cost to shelf, EUR and UAH
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
+++ b/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
@@ -18,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="23">
+  <numFmts count="24">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00&quot; ₴&quot;_-;\-* #,##0.00&quot; ₴&quot;_-;_-* \-??&quot; ₴&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$₴-422]_-;\-* #,##0.00\ [$₴-422]_-;_-* \-??\ [$₴-422]_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0000&quot; €&quot;"/>
@@ -40,10 +40,11 @@
     <numFmt numFmtId="182" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
     <numFmt numFmtId="183" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
     <numFmt numFmtId="184" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
-    <numFmt numFmtId="185" formatCode="+#,##0.00&quot; ₴&quot;;-#,##0.00&quot; ₴&quot;"/>
-    <numFmt numFmtId="186" formatCode="&quot;маржа &quot;0%"/>
+    <numFmt numFmtId="185" formatCode="&quot;€&quot;0.000"/>
+    <numFmt numFmtId="186" formatCode="+&quot;€&quot;0.000;-&quot;€&quot;0.000"/>
+    <numFmt numFmtId="187" formatCode="+#,##0.00;-#,##0.00"/>
   </numFmts>
-  <fonts count="56">
+  <fonts count="51">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -224,8 +225,83 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00172B46"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00172B46"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00008000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00172B46"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00172B46"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005E6D7E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00223A5E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B53A3A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005E6D7E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00223A5E"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005E6D7E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -242,107 +318,12 @@
     <font>
       <name val="Arial"/>
       <color rgb="005E6D7E"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00223A5E"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00172B46"/>
-      <sz val="17"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00172B46"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="003E8E96"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="0046538A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00223A5E"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00223A5E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00C4820A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00F9A50B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="008890B0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00008000"/>
+      <color rgb="00172B46"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00172B46"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00172B46"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00008000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="005E6D7E"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00008000"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -350,14 +331,8 @@
       <color rgb="005E6D7E"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="005E6D7E"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="30">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -484,12 +459,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE3A6"/>
+        <fgColor rgb="003E5A85"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003E5A85"/>
+        <fgColor rgb="005A74A0"/>
       </patternFill>
     </fill>
     <fill>
@@ -502,8 +477,13 @@
         <fgColor rgb="00FFF4D2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE3A6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="26">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -773,11 +753,6 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="medium">
-        <color rgb="00223A5E"/>
-      </bottom>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="00D5DCE8"/>
       </left>
@@ -791,6 +766,44 @@
         <color rgb="00D5DCE8"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00223A5E"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5DCE8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5DCE8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5DCE8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5DCE8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5DCE8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5DCE8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
@@ -801,7 +814,7 @@
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1242,123 +1255,134 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="185" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="35" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="36" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="37" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="39" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="38" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="35" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="37" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="39" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="38" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="37" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="35" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="35" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="37" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="39" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="38" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="186" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="187" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="47" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="35" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="34" fillId="25" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="34" fillId="25" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="37" fillId="26" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="38" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="48" fillId="29" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="49" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="50" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="51" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="185" fontId="49" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="185" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="48" fillId="29" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="48" fillId="29" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="53" fillId="28" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="53" fillId="28" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="53" fillId="28" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="48" fillId="29" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="48" fillId="29" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="186" fontId="48" fillId="29" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="38" fillId="25" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -6076,38 +6100,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N36"/>
+  <dimension ref="B2:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="3.5" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="3.5" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="3.5" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="3.5" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="3.5" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="3.5" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="2" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="2" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="151" t="inlineStr">
         <is>
-          <t>SIAS · закупка для полки 120 грн · 6 паллет</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
+          <t>SIAS · было → стало · от себестоимости в Украине до полки · 6 паллет</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="B3" s="152" t="str">
-        <f>"Запрос €"&amp;ROUND(L7,2)&amp;" за пачку → полка "&amp;ROUND(N12,2)&amp;" ₴ при марже "&amp;ROUND(J12/(F12/(1-F26-D26))*100,0)&amp;"%. Сейчас у SIAS €"&amp;MIN(D17:D22)&amp;"–€"&amp;MAX(D17:D22)&amp;" → снижение на "&amp;ROUND((1-L7/MIN(D17:D22))*100,0)&amp;"…"&amp;ROUND((1-L7/MAX(D17:D22))*100,0)&amp;"%."</f>
-        <v>Запрос €0.32 за пачку → полка 118.72 ₴ при марже 30%. Сейчас у SIAS €0.65–€0.75 → снижение на 51…57%.</v>
+        <f>"Чтобы полка стала "&amp;ROUND(C16,0)&amp;" ₴, закупка SIAS должна упасть с €"&amp;MIN(C7:C8)&amp;"–€"&amp;MAX(C7:C8)&amp;" до €"&amp;ROUND(C22,2)&amp;" за пачку (−"&amp;ROUND((1-C22/MIN(C7:C8))*100,0)&amp;"…"&amp;ROUND((1-C22/MAX(C7:C8))*100,0)&amp;"%). Маржа остаётся "&amp;ROUND(E16*100,0)&amp;"%."</f>
+        <v>Чтобы полка стала 120 ₴, закупка SIAS должна упасть с €0.65–€0.75 до €0.32 за пачку (−51…57%). Маржа остаётся 30%.</v>
       </c>
       <c r="C3" s="153" t="n"/>
       <c r="D3" s="153" t="n"/>
@@ -6121,708 +6147,659 @@
       <c r="L3" s="153" t="n"/>
       <c r="M3" s="153" t="n"/>
       <c r="N3" s="153" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="154" t="inlineStr">
-        <is>
-          <t>РАСЧЁТ ОДНОЙ ЛИНИЕЙ — от полки к закупочной цене</t>
-        </is>
-      </c>
-      <c r="C5" s="155" t="n"/>
+      <c r="O3" s="153" t="n"/>
+      <c r="P3" s="153" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="B5" s="154" t="inlineStr"/>
+      <c r="C5" s="154" t="inlineStr">
+        <is>
+          <t>Закупка SIAS</t>
+        </is>
+      </c>
       <c r="D5" s="155" t="n"/>
-      <c r="E5" s="155" t="n"/>
+      <c r="E5" s="154" t="inlineStr">
+        <is>
+          <t>Себестоимость в Украине (СС)</t>
+        </is>
+      </c>
       <c r="F5" s="155" t="n"/>
-      <c r="G5" s="155" t="n"/>
+      <c r="G5" s="154" t="inlineStr">
+        <is>
+          <t>Цена партнёру (магазину)</t>
+        </is>
+      </c>
       <c r="H5" s="155" t="n"/>
-      <c r="I5" s="155" t="n"/>
+      <c r="I5" s="154" t="inlineStr">
+        <is>
+          <t>Бонус сети</t>
+        </is>
+      </c>
       <c r="J5" s="155" t="n"/>
-      <c r="K5" s="155" t="n"/>
+      <c r="K5" s="154" t="inlineStr">
+        <is>
+          <t>Наша прибыль</t>
+        </is>
+      </c>
       <c r="L5" s="155" t="n"/>
-      <c r="M5" s="155" t="n"/>
+      <c r="M5" s="154" t="inlineStr">
+        <is>
+          <t>Наценка магазина</t>
+        </is>
+      </c>
       <c r="N5" s="155" t="n"/>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="156" t="inlineStr">
-        <is>
-          <t>Полка (цель)</t>
+      <c r="O5" s="154" t="inlineStr">
+        <is>
+          <t>ПОЛКА с НДС</t>
+        </is>
+      </c>
+      <c r="P5" s="155" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="154" t="inlineStr">
+        <is>
+          <t>Вариант</t>
+        </is>
+      </c>
+      <c r="C6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="D6" s="156" t="inlineStr">
         <is>
-          <t>Цена партнёру</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="E6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="F6" s="156" t="inlineStr">
         <is>
-          <t>Макс. себестоимость</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="G6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="H6" s="156" t="inlineStr">
         <is>
-          <t>Она же в €, без фин.</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="I6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="J6" s="156" t="inlineStr">
         <is>
-          <t>Предельная закупка</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="K6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="L6" s="156" t="inlineStr">
         <is>
-          <t>ЗАПРОС SIAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="B7" s="157">
-        <f>B26</f>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="M6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="N6" s="156" t="inlineStr">
+        <is>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="O6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="P6" s="156" t="inlineStr">
+        <is>
+          <t>₴</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="157" t="inlineStr">
+        <is>
+          <t>ДО · Vegetable, Spicy, Beef, Chicken</t>
+        </is>
+      </c>
+      <c r="C7" s="158" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D7" s="159">
+        <f>C7*K16</f>
+        <v>33.28</v>
+      </c>
+      <c r="E7" s="160">
+        <f>'Финмодель 6 паллет'!E13</f>
+        <v>1.134046875</v>
+      </c>
+      <c r="F7" s="161">
+        <f>E7*K16</f>
+        <v>58.063199999999995</v>
+      </c>
+      <c r="G7" s="162">
+        <f>H7/K16</f>
+        <v>2.520104166666666</v>
+      </c>
+      <c r="H7" s="161">
+        <f>F7/(1-G16-E16)</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="I7" s="162">
+        <f>J7/K16</f>
+        <v>0.6300260416666665</v>
+      </c>
+      <c r="J7" s="159">
+        <f>H7*G16</f>
+        <v>32.25733333333333</v>
+      </c>
+      <c r="K7" s="162">
+        <f>L7/K16</f>
+        <v>0.7560312499999997</v>
+      </c>
+      <c r="L7" s="159">
+        <f>H7-F7-J7</f>
+        <v>38.70879999999999</v>
+      </c>
+      <c r="M7" s="162">
+        <f>N7/K16</f>
+        <v>1.0080416666666663</v>
+      </c>
+      <c r="N7" s="159">
+        <f>H7*(I16-1)</f>
+        <v>51.61173333333331</v>
+      </c>
+      <c r="O7" s="162">
+        <f>P7/K16</f>
+        <v>3.5281458333333324</v>
+      </c>
+      <c r="P7" s="163">
+        <f>H7*I16</f>
+        <v>180.64106666666663</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="164" t="inlineStr">
+        <is>
+          <t>ДО · Gouda Cheese, Carbonara Spicy</t>
+        </is>
+      </c>
+      <c r="C8" s="158" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D8" s="165">
+        <f>C8*K16</f>
+        <v>38.400000000000006</v>
+      </c>
+      <c r="E8" s="160">
+        <f>'Финмодель 6 паллет'!E11</f>
+        <v>1.308515625</v>
+      </c>
+      <c r="F8" s="166">
+        <f>E8*K16</f>
+        <v>66.99600000000001</v>
+      </c>
+      <c r="G8" s="167">
+        <f>H8/K16</f>
+        <v>2.9078125000000004</v>
+      </c>
+      <c r="H8" s="166">
+        <f>F8/(1-G16-E16)</f>
+        <v>148.88000000000002</v>
+      </c>
+      <c r="I8" s="167">
+        <f>J8/K16</f>
+        <v>0.7269531250000001</v>
+      </c>
+      <c r="J8" s="165">
+        <f>H8*G16</f>
+        <v>37.220000000000006</v>
+      </c>
+      <c r="K8" s="167">
+        <f>L8/K16</f>
+        <v>0.8723437500000001</v>
+      </c>
+      <c r="L8" s="165">
+        <f>H8-F8-J8</f>
+        <v>44.66400000000001</v>
+      </c>
+      <c r="M8" s="167">
+        <f>N8/K16</f>
+        <v>1.163125</v>
+      </c>
+      <c r="N8" s="165">
+        <f>H8*(I16-1)</f>
+        <v>59.552</v>
+      </c>
+      <c r="O8" s="167">
+        <f>P8/K16</f>
+        <v>4.0709375</v>
+      </c>
+      <c r="P8" s="168">
+        <f>H8*I16</f>
+        <v>208.43200000000002</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="169" t="inlineStr">
+        <is>
+          <t>ПОСЛЕ · запрос SIAS (все 6 SKU)</t>
+        </is>
+      </c>
+      <c r="C9" s="170">
+        <f>C22</f>
+        <v>0.32</v>
+      </c>
+      <c r="D9" s="171">
+        <f>C9*K16</f>
+        <v>16.384</v>
+      </c>
+      <c r="E9" s="172">
+        <f>F9/K16</f>
+        <v>0.7453031249999998</v>
+      </c>
+      <c r="F9" s="173">
+        <f>(C9*K16+(E19+G19+I19)/(M19*O19)*K16+(C9+E19*K19/(M19*O19))*C19*K16+(C9+E19*K19/(M19*O19))*(1+C19)*O16*K16)*(1+M16)</f>
+        <v>38.15951999999999</v>
+      </c>
+      <c r="G9" s="174">
+        <f>H9/K16</f>
+        <v>1.6562291666666664</v>
+      </c>
+      <c r="H9" s="173">
+        <f>F9/(1-G16-E16)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="I9" s="174">
+        <f>J9/K16</f>
+        <v>0.4140572916666666</v>
+      </c>
+      <c r="J9" s="171">
+        <f>H9*G16</f>
+        <v>21.19973333333333</v>
+      </c>
+      <c r="K9" s="174">
+        <f>L9/K16</f>
+        <v>0.49686874999999997</v>
+      </c>
+      <c r="L9" s="171">
+        <f>H9-F9-J9</f>
+        <v>25.43968</v>
+      </c>
+      <c r="M9" s="174">
+        <f>N9/K16</f>
+        <v>0.6624916666666665</v>
+      </c>
+      <c r="N9" s="171">
+        <f>H9*(I16-1)</f>
+        <v>33.919573333333325</v>
+      </c>
+      <c r="O9" s="174">
+        <f>P9/K16</f>
+        <v>2.318720833333333</v>
+      </c>
+      <c r="P9" s="175">
+        <f>H9*I16</f>
+        <v>118.71850666666664</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="B10" s="176" t="inlineStr">
+        <is>
+          <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
+        </is>
+      </c>
+      <c r="C10" s="177">
+        <f>C9-C7</f>
+        <v>-0.33</v>
+      </c>
+      <c r="D10" s="178">
+        <f>D9-D7</f>
+        <v>-16.896</v>
+      </c>
+      <c r="E10" s="177">
+        <f>E9-E7</f>
+        <v>-0.38874375000000005</v>
+      </c>
+      <c r="F10" s="178">
+        <f>F9-F7</f>
+        <v>-19.90368</v>
+      </c>
+      <c r="G10" s="177">
+        <f>G9-G7</f>
+        <v>-0.8638749999999997</v>
+      </c>
+      <c r="H10" s="178">
+        <f>H9-H7</f>
+        <v>-44.23039999999999</v>
+      </c>
+      <c r="I10" s="177">
+        <f>I9-I7</f>
+        <v>-0.21596874999999993</v>
+      </c>
+      <c r="J10" s="178">
+        <f>J9-J7</f>
+        <v>-11.057599999999997</v>
+      </c>
+      <c r="K10" s="177">
+        <f>K9-K7</f>
+        <v>-0.25916249999999974</v>
+      </c>
+      <c r="L10" s="178">
+        <f>L9-L7</f>
+        <v>-13.26911999999999</v>
+      </c>
+      <c r="M10" s="177">
+        <f>M9-M7</f>
+        <v>-0.3455499999999998</v>
+      </c>
+      <c r="N10" s="178">
+        <f>N9-N7</f>
+        <v>-17.692159999999987</v>
+      </c>
+      <c r="O10" s="177">
+        <f>O9-O7</f>
+        <v>-1.2094249999999995</v>
+      </c>
+      <c r="P10" s="178">
+        <f>P9-P7</f>
+        <v>-61.92255999999999</v>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="179" t="inlineStr">
+        <is>
+          <t>Читайте по строке слева направо: закупка → себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="180" t="inlineStr">
+        <is>
+          <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 6 паллет»</t>
+        </is>
+      </c>
+      <c r="C13" s="181" t="n"/>
+      <c r="D13" s="181" t="n"/>
+      <c r="E13" s="181" t="n"/>
+      <c r="F13" s="181" t="n"/>
+      <c r="G13" s="181" t="n"/>
+      <c r="H13" s="181" t="n"/>
+      <c r="I13" s="181" t="n"/>
+      <c r="J13" s="181" t="n"/>
+      <c r="K13" s="181" t="n"/>
+      <c r="L13" s="181" t="n"/>
+      <c r="M13" s="181" t="n"/>
+      <c r="N13" s="181" t="n"/>
+      <c r="O13" s="181" t="n"/>
+      <c r="P13" s="181" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="C15" s="182" t="inlineStr">
+        <is>
+          <t>Полка, ₴</t>
+        </is>
+      </c>
+      <c r="E15" s="182" t="inlineStr">
+        <is>
+          <t>Наша маржа</t>
+        </is>
+      </c>
+      <c r="G15" s="182" t="inlineStr">
+        <is>
+          <t>Бонус сети</t>
+        </is>
+      </c>
+      <c r="I15" s="182" t="inlineStr">
+        <is>
+          <t>Множитель полки</t>
+        </is>
+      </c>
+      <c r="K15" s="182" t="inlineStr">
+        <is>
+          <t>Курс ₴/€</t>
+        </is>
+      </c>
+      <c r="M15" s="182" t="inlineStr">
+        <is>
+          <t>Финансирование</t>
+        </is>
+      </c>
+      <c r="O15" s="182" t="inlineStr">
+        <is>
+          <t>Импортный ПДВ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="183" t="inlineStr">
+        <is>
+          <t>Цель расчёта</t>
+        </is>
+      </c>
+      <c r="C16" s="184" t="n">
         <v>120</v>
       </c>
-      <c r="C7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="D7" s="157">
-        <f>B7/H26</f>
-        <v>85.71428571428572</v>
-      </c>
-      <c r="E7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="F7" s="157">
-        <f>D7*(1-F26-D26)</f>
-        <v>38.57142857142858</v>
-      </c>
-      <c r="G7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="H7" s="159">
-        <f>F7/J26/(1+L26)</f>
-        <v>0.7349738675958188</v>
-      </c>
-      <c r="I7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="J7" s="159">
-        <f>(H7-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+D28)*(1+B28))</f>
-        <v>0.3265407229965157</v>
-      </c>
-      <c r="K7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="L7" s="160">
-        <f>ROUNDDOWN(J7,2)</f>
-        <v>0.32</v>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="B8" s="161" t="str">
-        <f>"цель, с НДС"</f>
-        <v>цель, с НДС</v>
-      </c>
-      <c r="D8" s="161" t="str">
-        <f>"÷ множитель полки "&amp;H26</f>
-        <v>÷ множитель полки 1.4</v>
-      </c>
-      <c r="F8" s="161" t="str">
-        <f>"× "&amp;ROUND((1-F26-D26)*100,0)&amp;"% (100 − бонус − маржа)"</f>
-        <v>× 45% (100 − бонус − маржа)</v>
-      </c>
-      <c r="H8" s="161" t="str">
-        <f>"÷ курс "&amp;J26&amp;" и ÷ (1+"&amp;ROUND(L26*100,1)&amp;"% фин.)"</f>
-        <v>÷ курс 51.2 и ÷ (1+2.5% фин.)</v>
-      </c>
-      <c r="J8" s="161" t="str">
-        <f>"− расходы партии "&amp;ROUND(($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30),3)&amp;" €/пачку; ÷ "&amp;ROUND((1+D28)*(1+B28),2)&amp;" (ПДВ)"</f>
-        <v>− расходы партии 0.343 €/пачку; ÷ 1.2 (ПДВ)</v>
-      </c>
-      <c r="L8" s="161" t="str">
-        <f>"вниз до евроцента"</f>
-        <v>вниз до евроцента</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="154" t="inlineStr">
-        <is>
-          <t>ИЗ ЧЕГО СОСТОИТ ПОЛКА ПРИ ЗАПРОСЕ — ₴ за пачку и доля полки</t>
-        </is>
-      </c>
-      <c r="C10" s="155" t="n"/>
-      <c r="D10" s="155" t="n"/>
-      <c r="E10" s="155" t="n"/>
-      <c r="F10" s="155" t="n"/>
-      <c r="G10" s="155" t="n"/>
-      <c r="H10" s="155" t="n"/>
-      <c r="I10" s="155" t="n"/>
-      <c r="J10" s="155" t="n"/>
-      <c r="K10" s="155" t="n"/>
-      <c r="L10" s="155" t="n"/>
-      <c r="M10" s="155" t="n"/>
-      <c r="N10" s="155" t="n"/>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="156" t="inlineStr">
-        <is>
-          <t>Товар SIAS</t>
-        </is>
-      </c>
-      <c r="D11" s="156" t="inlineStr">
-        <is>
-          <t>Логистика, ПДВ, фін.</t>
-        </is>
-      </c>
-      <c r="F11" s="156" t="inlineStr">
-        <is>
-          <t>ИТОГО: себестоимость (СС)</t>
-        </is>
-      </c>
-      <c r="H11" s="156" t="inlineStr">
-        <is>
-          <t>Бонус сети</t>
-        </is>
-      </c>
-      <c r="J11" s="156" t="inlineStr">
-        <is>
-          <t>Наша прибыль</t>
-        </is>
-      </c>
-      <c r="L11" s="156" t="inlineStr">
-        <is>
-          <t>Наценка магазина</t>
-        </is>
-      </c>
-      <c r="N11" s="156" t="inlineStr">
-        <is>
-          <t>ИТОГО: ПОЛКА</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="B12" s="162">
-        <f>L7*J26</f>
-        <v>16.384</v>
-      </c>
-      <c r="C12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="D12" s="162">
-        <f>F12-B12</f>
-        <v>21.775519999999993</v>
-      </c>
-      <c r="E12" s="163" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="F12" s="157">
-        <f>(L7*J26+($F$28+$H$28+$J$28)/($B$30*$D$30)*J26+(L7+$F$28*$L$28/($B$30*$D$30))*$D$28*J26+(L7+$F$28*$L$28/($B$30*$D$30))*(1+$D$28)*$B$28*J26)*(1+L26)</f>
-        <v>38.15951999999999</v>
-      </c>
-      <c r="G12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="H12" s="162">
-        <f>F12/(1-F26-D26)*F26</f>
-        <v>21.19973333333333</v>
-      </c>
-      <c r="I12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="J12" s="162">
-        <f>F12/(1-F26-D26)-F12-H12</f>
-        <v>25.43968</v>
-      </c>
-      <c r="K12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="L12" s="162">
-        <f>F12/(1-F26-D26)*(H26-1)</f>
-        <v>33.919573333333325</v>
-      </c>
-      <c r="M12" s="163" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="N12" s="157">
-        <f>F12/(1-F26-D26)*H26</f>
-        <v>118.71850666666664</v>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="164">
-        <f>B12/$N$12</f>
-        <v>0.13800712677428112</v>
-      </c>
-      <c r="D13" s="165">
-        <f>D12/$N$12</f>
-        <v>0.18342144465429033</v>
-      </c>
-      <c r="F13" s="166">
-        <f>F12/$N$12</f>
-        <v>0.32142857142857145</v>
-      </c>
-      <c r="H13" s="167">
-        <f>H12/$N$12</f>
-        <v>0.17857142857142858</v>
-      </c>
-      <c r="J13" s="168">
-        <f>J12/$N$12</f>
-        <v>0.21428571428571433</v>
-      </c>
-      <c r="L13" s="169">
-        <f>L12/$N$12</f>
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="N13" s="166">
-        <f>N12/$N$12</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="154" t="inlineStr">
-        <is>
-          <t>ПО КАЖДОМУ SKU — цена закупки сейчас и в запросе</t>
-        </is>
-      </c>
-      <c r="C15" s="155" t="n"/>
-      <c r="D15" s="155" t="n"/>
-      <c r="E15" s="155" t="n"/>
-      <c r="F15" s="155" t="n"/>
-      <c r="G15" s="155" t="n"/>
-      <c r="H15" s="155" t="n"/>
-      <c r="I15" s="155" t="n"/>
-      <c r="J15" s="155" t="n"/>
-      <c r="K15" s="155" t="n"/>
-      <c r="L15" s="155" t="n"/>
-      <c r="M15" s="155" t="n"/>
-      <c r="N15" s="155" t="n"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="170" t="inlineStr">
-        <is>
-          <t>Продукт SIAS</t>
-        </is>
-      </c>
-      <c r="D16" s="170" t="inlineStr">
-        <is>
-          <t>Цена сейчас, €/уп.</t>
-        </is>
-      </c>
-      <c r="F16" s="170" t="inlineStr">
-        <is>
-          <t>Запрос, €/уп.</t>
-        </is>
-      </c>
-      <c r="H16" s="170" t="inlineStr">
-        <is>
-          <t>Снижение</t>
-        </is>
-      </c>
-      <c r="J16" s="170" t="inlineStr">
-        <is>
-          <t>Полка сейчас (маржа 30 %), ₴</t>
-        </is>
-      </c>
-      <c r="L16" s="170" t="inlineStr">
-        <is>
-          <t>Отрыв от цели 120, ₴</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="171" t="str">
-        <f>'Финмодель 6 паллет'!C11</f>
-        <v>Gouda Cheese 123 г</v>
-      </c>
-      <c r="D17" s="172" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F17" s="173">
-        <f>$L$7</f>
-        <v>0.32</v>
-      </c>
-      <c r="H17" s="174">
-        <f>1-F17/D17</f>
-        <v>0.5733333333333333</v>
-      </c>
-      <c r="J17" s="175">
-        <f>'Финмодель 6 паллет'!T11</f>
-        <v>208.43200000000002</v>
-      </c>
-      <c r="L17" s="176">
-        <f>J17-$B$26</f>
-        <v>88.43200000000002</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="177" t="str">
-        <f>'Финмодель 6 паллет'!C12</f>
-        <v>Carbonara Spicy 131 г</v>
-      </c>
-      <c r="D18" s="172" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F18" s="178">
-        <f>$L$7</f>
-        <v>0.32</v>
-      </c>
-      <c r="H18" s="179">
-        <f>1-F18/D18</f>
-        <v>0.5733333333333333</v>
-      </c>
-      <c r="J18" s="180">
-        <f>'Финмодель 6 паллет'!T12</f>
-        <v>208.43200000000002</v>
-      </c>
-      <c r="L18" s="181">
-        <f>J18-$B$26</f>
-        <v>88.43200000000002</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="171" t="str">
-        <f>'Финмодель 6 паллет'!C13</f>
-        <v>Vegetable Flavor 113 г</v>
-      </c>
-      <c r="D19" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F19" s="173">
-        <f>$L$7</f>
-        <v>0.32</v>
-      </c>
-      <c r="H19" s="174">
-        <f>1-F19/D19</f>
-        <v>0.5076923076923077</v>
-      </c>
-      <c r="J19" s="175">
-        <f>'Финмодель 6 паллет'!T13</f>
-        <v>180.64106666666663</v>
-      </c>
-      <c r="L19" s="176">
-        <f>J19-$B$26</f>
-        <v>60.64106666666663</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="177" t="str">
-        <f>'Финмодель 6 паллет'!C14</f>
-        <v>Spicy Flavor 112.5 г</v>
-      </c>
-      <c r="D20" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F20" s="178">
-        <f>$L$7</f>
-        <v>0.32</v>
-      </c>
-      <c r="H20" s="179">
-        <f>1-F20/D20</f>
-        <v>0.5076923076923077</v>
-      </c>
-      <c r="J20" s="180">
-        <f>'Финмодель 6 паллет'!T14</f>
-        <v>180.64106666666663</v>
-      </c>
-      <c r="L20" s="181">
-        <f>J20-$B$26</f>
-        <v>60.64106666666663</v>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="171" t="str">
-        <f>'Финмодель 6 паллет'!C15</f>
-        <v>Beef Flavor 113 г</v>
-      </c>
-      <c r="D21" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F21" s="173">
-        <f>$L$7</f>
-        <v>0.32</v>
-      </c>
-      <c r="H21" s="174">
-        <f>1-F21/D21</f>
-        <v>0.5076923076923077</v>
-      </c>
-      <c r="J21" s="175">
-        <f>'Финмодель 6 паллет'!T15</f>
-        <v>180.64106666666663</v>
-      </c>
-      <c r="L21" s="176">
-        <f>J21-$B$26</f>
-        <v>60.64106666666663</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="177" t="str">
-        <f>'Финмодель 6 паллет'!C16</f>
-        <v>Chicken Flavor 113 г</v>
-      </c>
-      <c r="D22" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F22" s="178">
-        <f>$L$7</f>
-        <v>0.32</v>
-      </c>
-      <c r="H22" s="179">
-        <f>1-F22/D22</f>
-        <v>0.5076923076923077</v>
-      </c>
-      <c r="J22" s="180">
-        <f>'Финмодель 6 паллет'!T16</f>
-        <v>180.64106666666663</v>
-      </c>
-      <c r="L22" s="181">
-        <f>J22-$B$26</f>
-        <v>60.64106666666663</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="154" t="inlineStr">
-        <is>
-          <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное — из вкладки «Финмодель 6 паллет», остальное — формулы</t>
-        </is>
-      </c>
-      <c r="C24" s="155" t="n"/>
-      <c r="D24" s="155" t="n"/>
-      <c r="E24" s="155" t="n"/>
-      <c r="F24" s="155" t="n"/>
-      <c r="G24" s="155" t="n"/>
-      <c r="H24" s="155" t="n"/>
-      <c r="I24" s="155" t="n"/>
-      <c r="J24" s="155" t="n"/>
-      <c r="K24" s="155" t="n"/>
-      <c r="L24" s="155" t="n"/>
-      <c r="M24" s="155" t="n"/>
-      <c r="N24" s="155" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="182" t="inlineStr">
-        <is>
-          <t>Полка, ₴</t>
-        </is>
-      </c>
-      <c r="D25" s="182" t="inlineStr">
-        <is>
-          <t>Наша маржа</t>
-        </is>
-      </c>
-      <c r="F25" s="182" t="inlineStr">
-        <is>
-          <t>Бонус сети</t>
-        </is>
-      </c>
-      <c r="H25" s="182" t="inlineStr">
-        <is>
-          <t>Множитель полки</t>
-        </is>
-      </c>
-      <c r="J25" s="182" t="inlineStr">
-        <is>
-          <t>Курс, ₴/€</t>
-        </is>
-      </c>
-      <c r="L25" s="182" t="inlineStr">
-        <is>
-          <t>Финансирование</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="183" t="n">
-        <v>120</v>
-      </c>
-      <c r="D26" s="184" t="n">
+      <c r="D16" s="185" t="n"/>
+      <c r="E16" s="186" t="n">
         <v>0.3</v>
       </c>
-      <c r="F26" s="185">
+      <c r="F16" s="185" t="n"/>
+      <c r="G16" s="187">
         <f>'Финмодель 6 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H26" s="186">
+      <c r="H16" s="188" t="n"/>
+      <c r="I16" s="189">
         <f>'Финмодель 6 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J26" s="187">
+      <c r="J16" s="188" t="n"/>
+      <c r="K16" s="190">
         <f>'Финмодель 6 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L26" s="184" t="n">
+      <c r="L16" s="188" t="n"/>
+      <c r="M16" s="186" t="n">
         <v>0.025</v>
       </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="B27" s="182" t="inlineStr">
-        <is>
-          <t>Импортный ПДВ</t>
-        </is>
-      </c>
-      <c r="D27" s="182" t="inlineStr">
+      <c r="N16" s="185" t="n"/>
+      <c r="O16" s="186" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P16" s="185" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="C18" s="182" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="F27" s="182" t="inlineStr">
+      <c r="E18" s="182" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="H27" s="182" t="inlineStr">
+      <c r="G18" s="182" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="J27" s="182" t="inlineStr">
-        <is>
-          <t>Прочие расходы, €</t>
-        </is>
-      </c>
-      <c r="L27" s="182" t="inlineStr">
+      <c r="I18" s="182" t="inlineStr">
+        <is>
+          <t>Прочие, €</t>
+        </is>
+      </c>
+      <c r="K18" s="182" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="184" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D28" s="184" t="n">
+      <c r="M18" s="182" t="inlineStr">
+        <is>
+          <t>Паллет в партии</t>
+        </is>
+      </c>
+      <c r="O18" s="182" t="inlineStr">
+        <is>
+          <t>Пачек на паллете</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="183" t="inlineStr">
+        <is>
+          <t>Расходы партии (Self-Cost_Sias)</t>
+        </is>
+      </c>
+      <c r="C19" s="186" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="188" t="n">
+      <c r="D19" s="185" t="n"/>
+      <c r="E19" s="191" t="n">
         <v>2600</v>
       </c>
-      <c r="H28" s="188" t="n">
+      <c r="F19" s="185" t="n"/>
+      <c r="G19" s="191" t="n">
         <v>288</v>
       </c>
-      <c r="J28" s="188" t="n">
+      <c r="H19" s="185" t="n"/>
+      <c r="I19" s="191" t="n">
         <v>42</v>
       </c>
-      <c r="L28" s="189" t="n">
+      <c r="J19" s="185" t="n"/>
+      <c r="K19" s="192" t="n">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="182" t="inlineStr">
-        <is>
-          <t>Паллет в партии</t>
-        </is>
-      </c>
-      <c r="D29" s="182" t="inlineStr">
-        <is>
-          <t>Пачек на паллете</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="188" t="n">
+      <c r="L19" s="185" t="n"/>
+      <c r="M19" s="191" t="n">
         <v>6</v>
       </c>
-      <c r="D30" s="188" t="n">
+      <c r="N19" s="185" t="n"/>
+      <c r="O19" s="191" t="n">
         <v>1600</v>
       </c>
-      <c r="F30" s="190" t="inlineStr">
-        <is>
-          <t>Источник чисел: Self-Cost_Sias (перевозка, брокер, прочие, ПДВ, фінансування, пачек на паллете).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="154" t="inlineStr">
-        <is>
-          <t>ЕСЛИ НАША МАРЖА ДРУГАЯ — запрос при той же полке</t>
-        </is>
-      </c>
-      <c r="C32" s="155" t="n"/>
-      <c r="D32" s="155" t="n"/>
-      <c r="E32" s="155" t="n"/>
-      <c r="F32" s="155" t="n"/>
-      <c r="G32" s="155" t="n"/>
-      <c r="H32" s="155" t="n"/>
-      <c r="I32" s="155" t="n"/>
-      <c r="J32" s="155" t="n"/>
-      <c r="K32" s="155" t="n"/>
-      <c r="L32" s="155" t="n"/>
-      <c r="M32" s="155" t="n"/>
-      <c r="N32" s="155" t="n"/>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="191" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D33" s="191" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F33" s="191" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H33" s="191" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J33" s="192" t="inlineStr">
-        <is>
-          <t>запрос, €/уп.: чем ниже наша маржа, тем выше допустимая закупка</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="B34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-B33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.25</v>
-      </c>
-      <c r="D34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-D33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.39</v>
-      </c>
-      <c r="F34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-F33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.46</v>
-      </c>
-      <c r="H34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-H33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.53</v>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="190" t="inlineStr">
-        <is>
-          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); импортный ПДВ входит в себестоимость, как в Self-Cost (если возмещается — допустимая закупка выше); без листинг-фи, промо и отсрочки; согласие SIAS не получено — цена для переговоров.</t>
+      <c r="P19" s="185" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="180" t="inlineStr">
+        <is>
+          <t>КАК ПОЛУЧЕН ЗАПРОС: из полки 120 ₴ обратно к закупке</t>
+        </is>
+      </c>
+      <c r="C21" s="181" t="n"/>
+      <c r="D21" s="181" t="n"/>
+      <c r="E21" s="181" t="n"/>
+      <c r="F21" s="181" t="n"/>
+      <c r="G21" s="181" t="n"/>
+      <c r="H21" s="181" t="n"/>
+      <c r="I21" s="181" t="n"/>
+      <c r="J21" s="181" t="n"/>
+      <c r="K21" s="181" t="n"/>
+      <c r="L21" s="181" t="n"/>
+      <c r="M21" s="181" t="n"/>
+      <c r="N21" s="181" t="n"/>
+      <c r="O21" s="181" t="n"/>
+      <c r="P21" s="181" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="193" t="inlineStr">
+        <is>
+          <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
+        </is>
+      </c>
+      <c r="C22" s="194">
+        <f>ROUNDDOWN(((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16)),2)</f>
+        <v>0.32</v>
+      </c>
+      <c r="D22" s="195" t="n"/>
+      <c r="E22" s="196" t="inlineStr">
+        <is>
+          <t>Формула: (полка ÷ множитель × (1 − бонус − маржа) ÷ курс ÷ (1 + фин.) − расходы партии на пачку) ÷ (1 + ПДВ)(1 + пошлина), округлено вниз</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="197" t="inlineStr">
+        <is>
+          <t>Предельная закупка до округления, €/уп.</t>
+        </is>
+      </c>
+      <c r="C23" s="198">
+        <f>((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16))</f>
+        <v>0.3265407229965157</v>
+      </c>
+      <c r="D23" s="199" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="200" t="inlineStr">
+        <is>
+          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); импортный ПДВ входит в себестоимость, как в Self-Cost; без листинг-фи, промо и отсрочки; согласие SIAS не получено — цена для переговоров.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B5:N5"/>
-    <mergeCell ref="B36:N36"/>
-    <mergeCell ref="J33:N34"/>
-    <mergeCell ref="B24:N24"/>
-    <mergeCell ref="B32:N32"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="B10:N10"/>
-    <mergeCell ref="F30:N30"/>
+  <mergeCells count="44">
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="B11:P11"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="B24:P24"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E22:P22"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="B3:P3"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B21:P21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
@@ -6836,38 +6813,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N36"/>
+  <dimension ref="B2:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="3.5" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="3.5" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="3.5" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="3.5" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="3.5" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="3.5" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="2" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="2" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="151" t="inlineStr">
         <is>
-          <t>SIAS · закупка для полки 120 грн · 33 паллеты (Full Truck)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
+          <t>SIAS · было → стало · от себестоимости в Украине до полки · 33 паллеты (Full Truck)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="B3" s="152" t="str">
-        <f>"Запрос €"&amp;ROUND(L7,2)&amp;" за пачку → полка "&amp;ROUND(N12,2)&amp;" ₴ при марже "&amp;ROUND(J12/(F12/(1-F26-D26))*100,0)&amp;"%. Сейчас у SIAS €"&amp;MIN(D17:D22)&amp;"–€"&amp;MAX(D17:D22)&amp;" → снижение на "&amp;ROUND((1-L7/MIN(D17:D22))*100,0)&amp;"…"&amp;ROUND((1-L7/MAX(D17:D22))*100,0)&amp;"%."</f>
-        <v>Запрос €0.54 за пачку → полка 119.86 ₴ при марже 30%. Сейчас у SIAS €0.65–€0.75 → снижение на 17…28%.</v>
+        <f>"Чтобы полка стала "&amp;ROUND(C16,0)&amp;" ₴, закупка SIAS должна упасть с €"&amp;MIN(C7:C8)&amp;"–€"&amp;MAX(C7:C8)&amp;" до €"&amp;ROUND(C22,2)&amp;" за пачку (−"&amp;ROUND((1-C22/MIN(C7:C8))*100,0)&amp;"…"&amp;ROUND((1-C22/MAX(C7:C8))*100,0)&amp;"%). Маржа остаётся "&amp;ROUND(E16*100,0)&amp;"%."</f>
+        <v>Чтобы полка стала 120 ₴, закупка SIAS должна упасть с €0.65–€0.75 до €0.54 за пачку (−17…28%). Маржа остаётся 30%.</v>
       </c>
       <c r="C3" s="153" t="n"/>
       <c r="D3" s="153" t="n"/>
@@ -6881,708 +6860,659 @@
       <c r="L3" s="153" t="n"/>
       <c r="M3" s="153" t="n"/>
       <c r="N3" s="153" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="154" t="inlineStr">
-        <is>
-          <t>РАСЧЁТ ОДНОЙ ЛИНИЕЙ — от полки к закупочной цене</t>
-        </is>
-      </c>
-      <c r="C5" s="155" t="n"/>
+      <c r="O3" s="153" t="n"/>
+      <c r="P3" s="153" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="B5" s="154" t="inlineStr"/>
+      <c r="C5" s="154" t="inlineStr">
+        <is>
+          <t>Закупка SIAS</t>
+        </is>
+      </c>
       <c r="D5" s="155" t="n"/>
-      <c r="E5" s="155" t="n"/>
+      <c r="E5" s="154" t="inlineStr">
+        <is>
+          <t>Себестоимость в Украине (СС)</t>
+        </is>
+      </c>
       <c r="F5" s="155" t="n"/>
-      <c r="G5" s="155" t="n"/>
+      <c r="G5" s="154" t="inlineStr">
+        <is>
+          <t>Цена партнёру (магазину)</t>
+        </is>
+      </c>
       <c r="H5" s="155" t="n"/>
-      <c r="I5" s="155" t="n"/>
+      <c r="I5" s="154" t="inlineStr">
+        <is>
+          <t>Бонус сети</t>
+        </is>
+      </c>
       <c r="J5" s="155" t="n"/>
-      <c r="K5" s="155" t="n"/>
+      <c r="K5" s="154" t="inlineStr">
+        <is>
+          <t>Наша прибыль</t>
+        </is>
+      </c>
       <c r="L5" s="155" t="n"/>
-      <c r="M5" s="155" t="n"/>
+      <c r="M5" s="154" t="inlineStr">
+        <is>
+          <t>Наценка магазина</t>
+        </is>
+      </c>
       <c r="N5" s="155" t="n"/>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="156" t="inlineStr">
-        <is>
-          <t>Полка (цель)</t>
+      <c r="O5" s="154" t="inlineStr">
+        <is>
+          <t>ПОЛКА с НДС</t>
+        </is>
+      </c>
+      <c r="P5" s="155" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="154" t="inlineStr">
+        <is>
+          <t>Вариант</t>
+        </is>
+      </c>
+      <c r="C6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="D6" s="156" t="inlineStr">
         <is>
-          <t>Цена партнёру</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="E6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="F6" s="156" t="inlineStr">
         <is>
-          <t>Макс. себестоимость</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="G6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="H6" s="156" t="inlineStr">
         <is>
-          <t>Она же в €, без фин.</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="I6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="J6" s="156" t="inlineStr">
         <is>
-          <t>Предельная закупка</t>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="K6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
         </is>
       </c>
       <c r="L6" s="156" t="inlineStr">
         <is>
-          <t>ЗАПРОС SIAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="B7" s="157">
-        <f>B26</f>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="M6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="N6" s="156" t="inlineStr">
+        <is>
+          <t>₴</t>
+        </is>
+      </c>
+      <c r="O6" s="156" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="P6" s="156" t="inlineStr">
+        <is>
+          <t>₴</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="157" t="inlineStr">
+        <is>
+          <t>ДО · Vegetable, Spicy, Beef, Chicken</t>
+        </is>
+      </c>
+      <c r="C7" s="158" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D7" s="159">
+        <f>C7*K16</f>
+        <v>33.28</v>
+      </c>
+      <c r="E7" s="160">
+        <f>'Финмодель 33 паллет'!E13</f>
+        <v>0.882380333698031</v>
+      </c>
+      <c r="F7" s="161">
+        <f>E7*K16</f>
+        <v>45.17787308533919</v>
+      </c>
+      <c r="G7" s="162">
+        <f>H7/K16</f>
+        <v>1.9608451859956246</v>
+      </c>
+      <c r="H7" s="161">
+        <f>F7/(1-G16-E16)</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="I7" s="162">
+        <f>J7/K16</f>
+        <v>0.49021129649890616</v>
+      </c>
+      <c r="J7" s="159">
+        <f>H7*G16</f>
+        <v>25.098818380743996</v>
+      </c>
+      <c r="K7" s="162">
+        <f>L7/K16</f>
+        <v>0.5882535557986873</v>
+      </c>
+      <c r="L7" s="159">
+        <f>H7-F7-J7</f>
+        <v>30.118582056892794</v>
+      </c>
+      <c r="M7" s="162">
+        <f>N7/K16</f>
+        <v>0.7843380743982498</v>
+      </c>
+      <c r="N7" s="159">
+        <f>H7*(I16-1)</f>
+        <v>40.15810940919039</v>
+      </c>
+      <c r="O7" s="162">
+        <f>P7/K16</f>
+        <v>2.745183260393874</v>
+      </c>
+      <c r="P7" s="163">
+        <f>H7*I16</f>
+        <v>140.55338293216636</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="164" t="inlineStr">
+        <is>
+          <t>ДО · Gouda Cheese, Carbonara Spicy</t>
+        </is>
+      </c>
+      <c r="C8" s="158" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D8" s="165">
+        <f>C8*K16</f>
+        <v>38.400000000000006</v>
+      </c>
+      <c r="E8" s="160">
+        <f>'Финмодель 33 паллет'!E11</f>
+        <v>1.018131154266958</v>
+      </c>
+      <c r="F8" s="166">
+        <f>E8*K16</f>
+        <v>52.12831509846825</v>
+      </c>
+      <c r="G8" s="167">
+        <f>H8/K16</f>
+        <v>2.2625136761487954</v>
+      </c>
+      <c r="H8" s="166">
+        <f>F8/(1-G16-E16)</f>
+        <v>115.84070021881833</v>
+      </c>
+      <c r="I8" s="167">
+        <f>J8/K16</f>
+        <v>0.5656284190371988</v>
+      </c>
+      <c r="J8" s="165">
+        <f>H8*G16</f>
+        <v>28.96017505470458</v>
+      </c>
+      <c r="K8" s="167">
+        <f>L8/K16</f>
+        <v>0.6787541028446387</v>
+      </c>
+      <c r="L8" s="165">
+        <f>H8-F8-J8</f>
+        <v>34.7522100656455</v>
+      </c>
+      <c r="M8" s="167">
+        <f>N8/K16</f>
+        <v>0.905005470459518</v>
+      </c>
+      <c r="N8" s="165">
+        <f>H8*(I16-1)</f>
+        <v>46.33628008752732</v>
+      </c>
+      <c r="O8" s="167">
+        <f>P8/K16</f>
+        <v>3.1675191466083135</v>
+      </c>
+      <c r="P8" s="168">
+        <f>H8*I16</f>
+        <v>162.17698030634565</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="169" t="inlineStr">
+        <is>
+          <t>ПОСЛЕ · запрос SIAS (все 6 SKU)</t>
+        </is>
+      </c>
+      <c r="C9" s="170">
+        <f>C22</f>
+        <v>0.54</v>
+      </c>
+      <c r="D9" s="171">
+        <f>C9*K16</f>
+        <v>27.648000000000003</v>
+      </c>
+      <c r="E9" s="172">
+        <f>F9/K16</f>
+        <v>0.7524897727272728</v>
+      </c>
+      <c r="F9" s="173">
+        <f>(C9*K16+(E19+G19+I19)/(M19*O19)*K16+(C9+E19*K19/(M19*O19))*C19*K16+(C9+E19*K19/(M19*O19))*(1+C19)*O16*K16)*(1+M16)</f>
+        <v>38.52747636363637</v>
+      </c>
+      <c r="G9" s="174">
+        <f>H9/K16</f>
+        <v>1.672199494949495</v>
+      </c>
+      <c r="H9" s="173">
+        <f>F9/(1-G16-E16)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="I9" s="174">
+        <f>J9/K16</f>
+        <v>0.41804987373737373</v>
+      </c>
+      <c r="J9" s="171">
+        <f>H9*G16</f>
+        <v>21.404153535353537</v>
+      </c>
+      <c r="K9" s="174">
+        <f>L9/K16</f>
+        <v>0.5016598484848485</v>
+      </c>
+      <c r="L9" s="171">
+        <f>H9-F9-J9</f>
+        <v>25.684984242424242</v>
+      </c>
+      <c r="M9" s="174">
+        <f>N9/K16</f>
+        <v>0.6688797979797979</v>
+      </c>
+      <c r="N9" s="171">
+        <f>H9*(I16-1)</f>
+        <v>34.246645656565654</v>
+      </c>
+      <c r="O9" s="174">
+        <f>P9/K16</f>
+        <v>2.3410792929292925</v>
+      </c>
+      <c r="P9" s="175">
+        <f>H9*I16</f>
+        <v>119.8632597979798</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="B10" s="176" t="inlineStr">
+        <is>
+          <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
+        </is>
+      </c>
+      <c r="C10" s="177">
+        <f>C9-C7</f>
+        <v>-0.10999999999999999</v>
+      </c>
+      <c r="D10" s="178">
+        <f>D9-D7</f>
+        <v>-5.631999999999998</v>
+      </c>
+      <c r="E10" s="177">
+        <f>E9-E7</f>
+        <v>-0.12989056097075824</v>
+      </c>
+      <c r="F10" s="178">
+        <f>F9-F7</f>
+        <v>-6.650396721702826</v>
+      </c>
+      <c r="G10" s="177">
+        <f>G9-G7</f>
+        <v>-0.2886456910461297</v>
+      </c>
+      <c r="H10" s="178">
+        <f>H9-H7</f>
+        <v>-14.778659381561837</v>
+      </c>
+      <c r="I10" s="177">
+        <f>I9-I7</f>
+        <v>-0.07216142276153242</v>
+      </c>
+      <c r="J10" s="178">
+        <f>J9-J7</f>
+        <v>-3.6946648453904594</v>
+      </c>
+      <c r="K10" s="177">
+        <f>K9-K7</f>
+        <v>-0.08659370731383886</v>
+      </c>
+      <c r="L10" s="178">
+        <f>L9-L7</f>
+        <v>-4.433597814468552</v>
+      </c>
+      <c r="M10" s="177">
+        <f>M9-M7</f>
+        <v>-0.11545827641845186</v>
+      </c>
+      <c r="N10" s="178">
+        <f>N9-N7</f>
+        <v>-5.911463752624734</v>
+      </c>
+      <c r="O10" s="177">
+        <f>O9-O7</f>
+        <v>-0.40410396746458144</v>
+      </c>
+      <c r="P10" s="178">
+        <f>P9-P7</f>
+        <v>-20.690123134186564</v>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="179" t="inlineStr">
+        <is>
+          <t>Читайте по строке слева направо: закупка → себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="180" t="inlineStr">
+        <is>
+          <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 33 паллет»</t>
+        </is>
+      </c>
+      <c r="C13" s="181" t="n"/>
+      <c r="D13" s="181" t="n"/>
+      <c r="E13" s="181" t="n"/>
+      <c r="F13" s="181" t="n"/>
+      <c r="G13" s="181" t="n"/>
+      <c r="H13" s="181" t="n"/>
+      <c r="I13" s="181" t="n"/>
+      <c r="J13" s="181" t="n"/>
+      <c r="K13" s="181" t="n"/>
+      <c r="L13" s="181" t="n"/>
+      <c r="M13" s="181" t="n"/>
+      <c r="N13" s="181" t="n"/>
+      <c r="O13" s="181" t="n"/>
+      <c r="P13" s="181" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="C15" s="182" t="inlineStr">
+        <is>
+          <t>Полка, ₴</t>
+        </is>
+      </c>
+      <c r="E15" s="182" t="inlineStr">
+        <is>
+          <t>Наша маржа</t>
+        </is>
+      </c>
+      <c r="G15" s="182" t="inlineStr">
+        <is>
+          <t>Бонус сети</t>
+        </is>
+      </c>
+      <c r="I15" s="182" t="inlineStr">
+        <is>
+          <t>Множитель полки</t>
+        </is>
+      </c>
+      <c r="K15" s="182" t="inlineStr">
+        <is>
+          <t>Курс ₴/€</t>
+        </is>
+      </c>
+      <c r="M15" s="182" t="inlineStr">
+        <is>
+          <t>Финансирование</t>
+        </is>
+      </c>
+      <c r="O15" s="182" t="inlineStr">
+        <is>
+          <t>Импортный ПДВ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="183" t="inlineStr">
+        <is>
+          <t>Цель расчёта</t>
+        </is>
+      </c>
+      <c r="C16" s="184" t="n">
         <v>120</v>
       </c>
-      <c r="C7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="D7" s="157">
-        <f>B7/H26</f>
-        <v>85.71428571428572</v>
-      </c>
-      <c r="E7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="F7" s="157">
-        <f>D7*(1-F26-D26)</f>
-        <v>38.57142857142858</v>
-      </c>
-      <c r="G7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="H7" s="159">
-        <f>F7/J26/(1+L26)</f>
-        <v>0.7349738675958188</v>
-      </c>
-      <c r="I7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="J7" s="159">
-        <f>(H7-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+D28)*(1+B28))</f>
-        <v>0.5406979199662126</v>
-      </c>
-      <c r="K7" s="158" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="L7" s="160">
-        <f>ROUNDDOWN(J7,2)</f>
-        <v>0.54</v>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="B8" s="161" t="str">
-        <f>"цель, с НДС"</f>
-        <v>цель, с НДС</v>
-      </c>
-      <c r="D8" s="161" t="str">
-        <f>"÷ множитель полки "&amp;H26</f>
-        <v>÷ множитель полки 1.4</v>
-      </c>
-      <c r="F8" s="161" t="str">
-        <f>"× "&amp;ROUND((1-F26-D26)*100,0)&amp;"% (100 − бонус − маржа)"</f>
-        <v>× 45% (100 − бонус − маржа)</v>
-      </c>
-      <c r="H8" s="161" t="str">
-        <f>"÷ курс "&amp;J26&amp;" и ÷ (1+"&amp;ROUND(L26*100,1)&amp;"% фин.)"</f>
-        <v>÷ курс 51.2 и ÷ (1+2.5% фин.)</v>
-      </c>
-      <c r="J8" s="161" t="str">
-        <f>"− расходы партии "&amp;ROUND(($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30),3)&amp;" €/пачку; ÷ "&amp;ROUND((1+D28)*(1+B28),2)&amp;" (ПДВ)"</f>
-        <v>− расходы партии 0.086 €/пачку; ÷ 1.2 (ПДВ)</v>
-      </c>
-      <c r="L8" s="161" t="str">
-        <f>"вниз до евроцента"</f>
-        <v>вниз до евроцента</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="154" t="inlineStr">
-        <is>
-          <t>ИЗ ЧЕГО СОСТОИТ ПОЛКА ПРИ ЗАПРОСЕ — ₴ за пачку и доля полки</t>
-        </is>
-      </c>
-      <c r="C10" s="155" t="n"/>
-      <c r="D10" s="155" t="n"/>
-      <c r="E10" s="155" t="n"/>
-      <c r="F10" s="155" t="n"/>
-      <c r="G10" s="155" t="n"/>
-      <c r="H10" s="155" t="n"/>
-      <c r="I10" s="155" t="n"/>
-      <c r="J10" s="155" t="n"/>
-      <c r="K10" s="155" t="n"/>
-      <c r="L10" s="155" t="n"/>
-      <c r="M10" s="155" t="n"/>
-      <c r="N10" s="155" t="n"/>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="156" t="inlineStr">
-        <is>
-          <t>Товар SIAS</t>
-        </is>
-      </c>
-      <c r="D11" s="156" t="inlineStr">
-        <is>
-          <t>Логистика, ПДВ, фін.</t>
-        </is>
-      </c>
-      <c r="F11" s="156" t="inlineStr">
-        <is>
-          <t>ИТОГО: себестоимость (СС)</t>
-        </is>
-      </c>
-      <c r="H11" s="156" t="inlineStr">
-        <is>
-          <t>Бонус сети</t>
-        </is>
-      </c>
-      <c r="J11" s="156" t="inlineStr">
-        <is>
-          <t>Наша прибыль</t>
-        </is>
-      </c>
-      <c r="L11" s="156" t="inlineStr">
-        <is>
-          <t>Наценка магазина</t>
-        </is>
-      </c>
-      <c r="N11" s="156" t="inlineStr">
-        <is>
-          <t>ИТОГО: ПОЛКА</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="B12" s="162">
-        <f>L7*J26</f>
-        <v>27.648000000000003</v>
-      </c>
-      <c r="C12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="D12" s="162">
-        <f>F12-B12</f>
-        <v>10.879476363636364</v>
-      </c>
-      <c r="E12" s="163" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="F12" s="157">
-        <f>(L7*J26+($F$28+$H$28+$J$28)/($B$30*$D$30)*J26+(L7+$F$28*$L$28/($B$30*$D$30))*$D$28*J26+(L7+$F$28*$L$28/($B$30*$D$30))*(1+$D$28)*$B$28*J26)*(1+L26)</f>
-        <v>38.52747636363637</v>
-      </c>
-      <c r="G12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="H12" s="162">
-        <f>F12/(1-F26-D26)*F26</f>
-        <v>21.404153535353537</v>
-      </c>
-      <c r="I12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="J12" s="162">
-        <f>F12/(1-F26-D26)-F12-H12</f>
-        <v>25.684984242424242</v>
-      </c>
-      <c r="K12" s="163" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="L12" s="162">
-        <f>F12/(1-F26-D26)*(H26-1)</f>
-        <v>34.246645656565654</v>
-      </c>
-      <c r="M12" s="163" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="N12" s="157">
-        <f>F12/(1-F26-D26)*H26</f>
-        <v>119.8632597979798</v>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="164">
-        <f>B12/$N$12</f>
-        <v>0.2306628406952936</v>
-      </c>
-      <c r="D13" s="165">
-        <f>D12/$N$12</f>
-        <v>0.09076573073327787</v>
-      </c>
-      <c r="F13" s="166">
-        <f>F12/$N$12</f>
-        <v>0.32142857142857145</v>
-      </c>
-      <c r="H13" s="167">
-        <f>H12/$N$12</f>
-        <v>0.17857142857142858</v>
-      </c>
-      <c r="J13" s="168">
-        <f>J12/$N$12</f>
-        <v>0.2142857142857143</v>
-      </c>
-      <c r="L13" s="169">
-        <f>L12/$N$12</f>
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="N13" s="166">
-        <f>N12/$N$12</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="154" t="inlineStr">
-        <is>
-          <t>ПО КАЖДОМУ SKU — цена закупки сейчас и в запросе</t>
-        </is>
-      </c>
-      <c r="C15" s="155" t="n"/>
-      <c r="D15" s="155" t="n"/>
-      <c r="E15" s="155" t="n"/>
-      <c r="F15" s="155" t="n"/>
-      <c r="G15" s="155" t="n"/>
-      <c r="H15" s="155" t="n"/>
-      <c r="I15" s="155" t="n"/>
-      <c r="J15" s="155" t="n"/>
-      <c r="K15" s="155" t="n"/>
-      <c r="L15" s="155" t="n"/>
-      <c r="M15" s="155" t="n"/>
-      <c r="N15" s="155" t="n"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="170" t="inlineStr">
-        <is>
-          <t>Продукт SIAS</t>
-        </is>
-      </c>
-      <c r="D16" s="170" t="inlineStr">
-        <is>
-          <t>Цена сейчас, €/уп.</t>
-        </is>
-      </c>
-      <c r="F16" s="170" t="inlineStr">
-        <is>
-          <t>Запрос, €/уп.</t>
-        </is>
-      </c>
-      <c r="H16" s="170" t="inlineStr">
-        <is>
-          <t>Снижение</t>
-        </is>
-      </c>
-      <c r="J16" s="170" t="inlineStr">
-        <is>
-          <t>Полка сейчас (маржа 30 %), ₴</t>
-        </is>
-      </c>
-      <c r="L16" s="170" t="inlineStr">
-        <is>
-          <t>Отрыв от цели 120, ₴</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="171" t="str">
-        <f>'Финмодель 33 паллет'!C11</f>
-        <v>Gouda Cheese 123 г</v>
-      </c>
-      <c r="D17" s="172" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F17" s="173">
-        <f>$L$7</f>
-        <v>0.54</v>
-      </c>
-      <c r="H17" s="174">
-        <f>1-F17/D17</f>
-        <v>0.2799999999999999</v>
-      </c>
-      <c r="J17" s="175">
-        <f>'Финмодель 33 паллет'!T11</f>
-        <v>162.17698030634565</v>
-      </c>
-      <c r="L17" s="176">
-        <f>J17-$B$26</f>
-        <v>42.176980306345655</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="177" t="str">
-        <f>'Финмодель 33 паллет'!C12</f>
-        <v>Carbonara Spicy 131 г</v>
-      </c>
-      <c r="D18" s="172" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F18" s="178">
-        <f>$L$7</f>
-        <v>0.54</v>
-      </c>
-      <c r="H18" s="179">
-        <f>1-F18/D18</f>
-        <v>0.2799999999999999</v>
-      </c>
-      <c r="J18" s="180">
-        <f>'Финмодель 33 паллет'!T12</f>
-        <v>162.17698030634565</v>
-      </c>
-      <c r="L18" s="181">
-        <f>J18-$B$26</f>
-        <v>42.176980306345655</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="171" t="str">
-        <f>'Финмодель 33 паллет'!C13</f>
-        <v>Vegetable Flavor 113 г</v>
-      </c>
-      <c r="D19" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F19" s="173">
-        <f>$L$7</f>
-        <v>0.54</v>
-      </c>
-      <c r="H19" s="174">
-        <f>1-F19/D19</f>
-        <v>0.16923076923076918</v>
-      </c>
-      <c r="J19" s="175">
-        <f>'Финмодель 33 паллет'!T13</f>
-        <v>140.55338293216636</v>
-      </c>
-      <c r="L19" s="176">
-        <f>J19-$B$26</f>
-        <v>20.553382932166357</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="177" t="str">
-        <f>'Финмодель 33 паллет'!C14</f>
-        <v>Spicy Flavor 112.5 г</v>
-      </c>
-      <c r="D20" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F20" s="178">
-        <f>$L$7</f>
-        <v>0.54</v>
-      </c>
-      <c r="H20" s="179">
-        <f>1-F20/D20</f>
-        <v>0.16923076923076918</v>
-      </c>
-      <c r="J20" s="180">
-        <f>'Финмодель 33 паллет'!T14</f>
-        <v>140.55338293216636</v>
-      </c>
-      <c r="L20" s="181">
-        <f>J20-$B$26</f>
-        <v>20.553382932166357</v>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="171" t="str">
-        <f>'Финмодель 33 паллет'!C15</f>
-        <v>Beef Flavor 113 г</v>
-      </c>
-      <c r="D21" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F21" s="173">
-        <f>$L$7</f>
-        <v>0.54</v>
-      </c>
-      <c r="H21" s="174">
-        <f>1-F21/D21</f>
-        <v>0.16923076923076918</v>
-      </c>
-      <c r="J21" s="175">
-        <f>'Финмодель 33 паллет'!T15</f>
-        <v>140.55338293216636</v>
-      </c>
-      <c r="L21" s="176">
-        <f>J21-$B$26</f>
-        <v>20.553382932166357</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="177" t="str">
-        <f>'Финмодель 33 паллет'!C16</f>
-        <v>Chicken Flavor 113 г</v>
-      </c>
-      <c r="D22" s="172" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F22" s="178">
-        <f>$L$7</f>
-        <v>0.54</v>
-      </c>
-      <c r="H22" s="179">
-        <f>1-F22/D22</f>
-        <v>0.16923076923076918</v>
-      </c>
-      <c r="J22" s="180">
-        <f>'Финмодель 33 паллет'!T16</f>
-        <v>140.55338293216636</v>
-      </c>
-      <c r="L22" s="181">
-        <f>J22-$B$26</f>
-        <v>20.553382932166357</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="154" t="inlineStr">
-        <is>
-          <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное — из вкладки «Финмодель 33 паллет», остальное — формулы</t>
-        </is>
-      </c>
-      <c r="C24" s="155" t="n"/>
-      <c r="D24" s="155" t="n"/>
-      <c r="E24" s="155" t="n"/>
-      <c r="F24" s="155" t="n"/>
-      <c r="G24" s="155" t="n"/>
-      <c r="H24" s="155" t="n"/>
-      <c r="I24" s="155" t="n"/>
-      <c r="J24" s="155" t="n"/>
-      <c r="K24" s="155" t="n"/>
-      <c r="L24" s="155" t="n"/>
-      <c r="M24" s="155" t="n"/>
-      <c r="N24" s="155" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="182" t="inlineStr">
-        <is>
-          <t>Полка, ₴</t>
-        </is>
-      </c>
-      <c r="D25" s="182" t="inlineStr">
-        <is>
-          <t>Наша маржа</t>
-        </is>
-      </c>
-      <c r="F25" s="182" t="inlineStr">
-        <is>
-          <t>Бонус сети</t>
-        </is>
-      </c>
-      <c r="H25" s="182" t="inlineStr">
-        <is>
-          <t>Множитель полки</t>
-        </is>
-      </c>
-      <c r="J25" s="182" t="inlineStr">
-        <is>
-          <t>Курс, ₴/€</t>
-        </is>
-      </c>
-      <c r="L25" s="182" t="inlineStr">
-        <is>
-          <t>Финансирование</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="183" t="n">
-        <v>120</v>
-      </c>
-      <c r="D26" s="184" t="n">
+      <c r="D16" s="185" t="n"/>
+      <c r="E16" s="186" t="n">
         <v>0.3</v>
       </c>
-      <c r="F26" s="185">
+      <c r="F16" s="185" t="n"/>
+      <c r="G16" s="187">
         <f>'Финмодель 33 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H26" s="186">
+      <c r="H16" s="188" t="n"/>
+      <c r="I16" s="189">
         <f>'Финмодель 33 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J26" s="187">
+      <c r="J16" s="188" t="n"/>
+      <c r="K16" s="190">
         <f>'Финмодель 33 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L26" s="184" t="n">
+      <c r="L16" s="188" t="n"/>
+      <c r="M16" s="186" t="n">
         <v>0.025</v>
       </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="B27" s="182" t="inlineStr">
-        <is>
-          <t>Импортный ПДВ</t>
-        </is>
-      </c>
-      <c r="D27" s="182" t="inlineStr">
+      <c r="N16" s="185" t="n"/>
+      <c r="O16" s="186" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P16" s="185" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="C18" s="182" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="F27" s="182" t="inlineStr">
+      <c r="E18" s="182" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="H27" s="182" t="inlineStr">
+      <c r="G18" s="182" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="J27" s="182" t="inlineStr">
-        <is>
-          <t>Прочие расходы, €</t>
-        </is>
-      </c>
-      <c r="L27" s="182" t="inlineStr">
+      <c r="I18" s="182" t="inlineStr">
+        <is>
+          <t>Прочие, €</t>
+        </is>
+      </c>
+      <c r="K18" s="182" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="184" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D28" s="184" t="n">
+      <c r="M18" s="182" t="inlineStr">
+        <is>
+          <t>Паллет в партии</t>
+        </is>
+      </c>
+      <c r="O18" s="182" t="inlineStr">
+        <is>
+          <t>Пачек на паллете</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="183" t="inlineStr">
+        <is>
+          <t>Расходы партии (Self-Cost_Sias)</t>
+        </is>
+      </c>
+      <c r="C19" s="186" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="188" t="n">
+      <c r="D19" s="185" t="n"/>
+      <c r="E19" s="191" t="n">
         <v>3700</v>
       </c>
-      <c r="H28" s="188" t="n">
+      <c r="F19" s="185" t="n"/>
+      <c r="G19" s="191" t="n">
         <v>288</v>
       </c>
-      <c r="J28" s="188" t="n">
+      <c r="H19" s="185" t="n"/>
+      <c r="I19" s="191" t="n">
         <v>42</v>
       </c>
-      <c r="L28" s="189" t="n">
+      <c r="J19" s="185" t="n"/>
+      <c r="K19" s="192" t="n">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="182" t="inlineStr">
-        <is>
-          <t>Паллет в партии</t>
-        </is>
-      </c>
-      <c r="D29" s="182" t="inlineStr">
-        <is>
-          <t>Пачек на паллете</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="188" t="n">
+      <c r="L19" s="185" t="n"/>
+      <c r="M19" s="191" t="n">
         <v>33</v>
       </c>
-      <c r="D30" s="188" t="n">
+      <c r="N19" s="185" t="n"/>
+      <c r="O19" s="191" t="n">
         <v>1600</v>
       </c>
-      <c r="F30" s="190" t="inlineStr">
-        <is>
-          <t>Источник чисел: Self-Cost_Sias (перевозка, брокер, прочие, ПДВ, фінансування, пачек на паллете).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="154" t="inlineStr">
-        <is>
-          <t>ЕСЛИ НАША МАРЖА ДРУГАЯ — запрос при той же полке</t>
-        </is>
-      </c>
-      <c r="C32" s="155" t="n"/>
-      <c r="D32" s="155" t="n"/>
-      <c r="E32" s="155" t="n"/>
-      <c r="F32" s="155" t="n"/>
-      <c r="G32" s="155" t="n"/>
-      <c r="H32" s="155" t="n"/>
-      <c r="I32" s="155" t="n"/>
-      <c r="J32" s="155" t="n"/>
-      <c r="K32" s="155" t="n"/>
-      <c r="L32" s="155" t="n"/>
-      <c r="M32" s="155" t="n"/>
-      <c r="N32" s="155" t="n"/>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="191" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D33" s="191" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F33" s="191" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H33" s="191" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J33" s="192" t="inlineStr">
-        <is>
-          <t>запрос, €/уп.: чем ниже наша маржа, тем выше допустимая закупка</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="B34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-B33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.47</v>
-      </c>
-      <c r="D34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-D33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.6</v>
-      </c>
-      <c r="F34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-F33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.67</v>
-      </c>
-      <c r="H34" s="193">
-        <f>ROUNDDOWN((($B$26/$H$26*(1-$F$26-H33))/$J$26/(1+$L$26)-($F$28+$H$28+$J$28+$F$28*$L$28*($D$28+$B$28*(1+$D$28)))/($B$30*$D$30))/((1+$D$28)*(1+$B$28)),2)</f>
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="190" t="inlineStr">
-        <is>
-          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); импортный ПДВ входит в себестоимость, как в Self-Cost (если возмещается — допустимая закупка выше); без листинг-фи, промо и отсрочки; согласие SIAS не получено — цена для переговоров.</t>
+      <c r="P19" s="185" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="180" t="inlineStr">
+        <is>
+          <t>КАК ПОЛУЧЕН ЗАПРОС: из полки 120 ₴ обратно к закупке</t>
+        </is>
+      </c>
+      <c r="C21" s="181" t="n"/>
+      <c r="D21" s="181" t="n"/>
+      <c r="E21" s="181" t="n"/>
+      <c r="F21" s="181" t="n"/>
+      <c r="G21" s="181" t="n"/>
+      <c r="H21" s="181" t="n"/>
+      <c r="I21" s="181" t="n"/>
+      <c r="J21" s="181" t="n"/>
+      <c r="K21" s="181" t="n"/>
+      <c r="L21" s="181" t="n"/>
+      <c r="M21" s="181" t="n"/>
+      <c r="N21" s="181" t="n"/>
+      <c r="O21" s="181" t="n"/>
+      <c r="P21" s="181" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="193" t="inlineStr">
+        <is>
+          <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
+        </is>
+      </c>
+      <c r="C22" s="194">
+        <f>ROUNDDOWN(((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16)),2)</f>
+        <v>0.54</v>
+      </c>
+      <c r="D22" s="195" t="n"/>
+      <c r="E22" s="196" t="inlineStr">
+        <is>
+          <t>Формула: (полка ÷ множитель × (1 − бонус − маржа) ÷ курс ÷ (1 + фин.) − расходы партии на пачку) ÷ (1 + ПДВ)(1 + пошлина), округлено вниз</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="197" t="inlineStr">
+        <is>
+          <t>Предельная закупка до округления, €/уп.</t>
+        </is>
+      </c>
+      <c r="C23" s="198">
+        <f>((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16))</f>
+        <v>0.5406979199662126</v>
+      </c>
+      <c r="D23" s="199" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="200" t="inlineStr">
+        <is>
+          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); импортный ПДВ входит в себестоимость, как в Self-Cost; без листинг-фи, промо и отсрочки; согласие SIAS не получено — цена для переговоров.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B5:N5"/>
-    <mergeCell ref="B36:N36"/>
-    <mergeCell ref="J33:N34"/>
-    <mergeCell ref="B24:N24"/>
-    <mergeCell ref="B32:N32"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="B10:N10"/>
-    <mergeCell ref="F30:N30"/>
+  <mergeCells count="44">
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="B11:P11"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="B24:P24"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E22:P22"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="B3:P3"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B21:P21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Finmodel tabs 3-4: hide batch cost inputs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
+++ b/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
@@ -6625,7 +6625,7 @@
       </c>
       <c r="P16" s="185" t="n"/>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" hidden="1" ht="22" customHeight="1">
       <c r="C18" s="182" t="inlineStr">
         <is>
           <t>Пошлина</t>
@@ -6662,7 +6662,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" hidden="1" ht="22" customHeight="1">
       <c r="B19" s="183" t="inlineStr">
         <is>
           <t>Расходы партии (Self-Cost_Sias)</t>
@@ -6731,7 +6731,7 @@
       <c r="D22" s="195" t="n"/>
       <c r="E22" s="196" t="inlineStr">
         <is>
-          <t>Формула: (полка ÷ множитель × (1 − бонус − маржа) ÷ курс ÷ (1 + фин.) − расходы партии на пачку) ÷ (1 + ПДВ)(1 + пошлина), округлено вниз</t>
+          <t>Считаем от полки 120 ₴ назад: цена партнёру → допустимая себестоимость → предельная закупка, округлено вниз до евроцента.</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="P16" s="185" t="n"/>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" hidden="1" ht="22" customHeight="1">
       <c r="C18" s="182" t="inlineStr">
         <is>
           <t>Пошлина</t>
@@ -7375,7 +7375,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" hidden="1" ht="22" customHeight="1">
       <c r="B19" s="183" t="inlineStr">
         <is>
           <t>Расходы партии (Self-Cost_Sias)</t>
@@ -7444,7 +7444,7 @@
       <c r="D22" s="195" t="n"/>
       <c r="E22" s="196" t="inlineStr">
         <is>
-          <t>Формула: (полка ÷ множитель × (1 − бонус − маржа) ÷ курс ÷ (1 + фин.) − расходы партии на пачку) ÷ (1 + ПДВ)(1 + пошлина), округлено вниз</t>
+          <t>Считаем от полки 120 ₴ назад: цена партнёру → допустимая себестоимость → предельная закупка, округлено вниз до евроцента.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finmodel tabs 3-4: start from cost price figure, cost calculation hidden
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
+++ b/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
@@ -236,31 +236,25 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00172B46"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="00008000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00172B46"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00172B46"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00172B46"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00172B46"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -300,6 +294,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00008000"/>
       <sz val="11"/>
     </font>
@@ -311,9 +311,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00172B46"/>
-      <sz val="14"/>
+      <i val="1"/>
+      <color rgb="005E6D7E"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -322,14 +322,14 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00172B46"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="005E6D7E"/>
-      <sz val="8"/>
+      <color rgb="00172B46"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="31">
@@ -474,12 +474,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF4D2"/>
+        <fgColor rgb="00FCE3A6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE3A6"/>
+        <fgColor rgb="00FFF4D2"/>
       </patternFill>
     </fill>
   </fills>
@@ -814,7 +814,7 @@
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="197">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1265,87 +1265,78 @@
     <xf numFmtId="0" fontId="33" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="34" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="35" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="36" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="38" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="36" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="37" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="39" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="38" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="35" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="37" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="38" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="39" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="36" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="38" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="37" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="37" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="38" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="35" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="35" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="35" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="36" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="37" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="37" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="39" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="186" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="38" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="187" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="187" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="173" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1358,31 +1349,28 @@
     <xf numFmtId="2" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="34" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="47" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="35" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="49" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="50" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="4" fontId="50" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -6100,26 +6088,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:P24"/>
+  <dimension ref="B2:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="2" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="2" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6130,10 +6116,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="B3" s="152" t="str">
-        <f>"Чтобы полка стала "&amp;ROUND(C16,0)&amp;" ₴, закупка SIAS должна упасть с €"&amp;MIN(C7:C8)&amp;"–€"&amp;MAX(C7:C8)&amp;" до €"&amp;ROUND(C22,2)&amp;" за пачку (−"&amp;ROUND((1-C22/MIN(C7:C8))*100,0)&amp;"…"&amp;ROUND((1-C22/MAX(C7:C8))*100,0)&amp;"%). Маржа остаётся "&amp;ROUND(E16*100,0)&amp;"%."</f>
-        <v>Чтобы полка стала 120 ₴, закупка SIAS должна упасть с €0.65–€0.75 до €0.32 за пачку (−51…57%). Маржа остаётся 30%.</v>
+        <f>"Полка "&amp;ROUND(C14,0)&amp;" ₴ достижима при себестоимости "&amp;ROUND(D9,2)&amp;" ₴ (сейчас "&amp;ROUND(D7,2)&amp;"–"&amp;ROUND(D8,2)&amp;" ₴). Для этого закупка SIAS должна быть €"&amp;ROUND(C21,2)&amp;" вместо €"&amp;MIN(C20,E20)&amp;"–€"&amp;MAX(C20,E20)&amp;" (−"&amp;ROUND((1-C21/MIN(C20,E20))*100,0)&amp;"…"&amp;ROUND((1-C21/MAX(C20,E20))*100,0)&amp;"%)."</f>
+        <v>Полка 120 ₴ достижима при себестоимости 38.16 ₴ (сейчас 58.06–67 ₴). Для этого закупка SIAS должна быть €0.32 вместо €0.65–€0.75 (−51…57%).</v>
       </c>
       <c r="C3" s="153" t="n"/>
       <c r="D3" s="153" t="n"/>
@@ -6147,53 +6133,45 @@
       <c r="L3" s="153" t="n"/>
       <c r="M3" s="153" t="n"/>
       <c r="N3" s="153" t="n"/>
-      <c r="O3" s="153" t="n"/>
-      <c r="P3" s="153" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="154" t="inlineStr"/>
       <c r="C5" s="154" t="inlineStr">
         <is>
-          <t>Закупка SIAS</t>
+          <t>Себестоимость в Украине (СС)</t>
         </is>
       </c>
       <c r="D5" s="155" t="n"/>
       <c r="E5" s="154" t="inlineStr">
         <is>
-          <t>Себестоимость в Украине (СС)</t>
+          <t>Цена партнёру (магазину)</t>
         </is>
       </c>
       <c r="F5" s="155" t="n"/>
       <c r="G5" s="154" t="inlineStr">
         <is>
-          <t>Цена партнёру (магазину)</t>
+          <t>Бонус сети</t>
         </is>
       </c>
       <c r="H5" s="155" t="n"/>
       <c r="I5" s="154" t="inlineStr">
         <is>
-          <t>Бонус сети</t>
+          <t>Наша прибыль</t>
         </is>
       </c>
       <c r="J5" s="155" t="n"/>
       <c r="K5" s="154" t="inlineStr">
         <is>
-          <t>Наша прибыль</t>
+          <t>Наценка магазина</t>
         </is>
       </c>
       <c r="L5" s="155" t="n"/>
       <c r="M5" s="154" t="inlineStr">
         <is>
-          <t>Наценка магазина</t>
+          <t>ПОЛКА с НДС</t>
         </is>
       </c>
       <c r="N5" s="155" t="n"/>
-      <c r="O5" s="154" t="inlineStr">
-        <is>
-          <t>ПОЛКА с НДС</t>
-        </is>
-      </c>
-      <c r="P5" s="155" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="B6" s="154" t="inlineStr">
@@ -6261,545 +6239,496 @@
           <t>₴</t>
         </is>
       </c>
-      <c r="O6" s="156" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="P6" s="156" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="157" t="inlineStr">
-        <is>
-          <t>ДО · Vegetable, Spicy, Beef, Chicken</t>
-        </is>
-      </c>
-      <c r="C7" s="158" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D7" s="159">
-        <f>C7*K16</f>
-        <v>33.28</v>
-      </c>
-      <c r="E7" s="160">
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="157" t="str">
+        <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
+        <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
+      </c>
+      <c r="C7" s="158">
         <f>'Финмодель 6 паллет'!E13</f>
         <v>1.134046875</v>
       </c>
-      <c r="F7" s="161">
-        <f>E7*K16</f>
+      <c r="D7" s="159">
+        <f>C7*K14</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="G7" s="162">
-        <f>H7/K16</f>
+      <c r="E7" s="160">
+        <f>F7/K14</f>
         <v>2.520104166666666</v>
       </c>
+      <c r="F7" s="159">
+        <f>D7/(1-G14-E14)</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="G7" s="160">
+        <f>H7/K14</f>
+        <v>0.6300260416666665</v>
+      </c>
       <c r="H7" s="161">
-        <f>F7/(1-G16-E16)</f>
-        <v>129.0293333333333</v>
-      </c>
-      <c r="I7" s="162">
-        <f>J7/K16</f>
-        <v>0.6300260416666665</v>
-      </c>
-      <c r="J7" s="159">
-        <f>H7*G16</f>
+        <f>F7*G14</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="K7" s="162">
-        <f>L7/K16</f>
+      <c r="I7" s="160">
+        <f>J7/K14</f>
         <v>0.7560312499999997</v>
       </c>
-      <c r="L7" s="159">
-        <f>H7-F7-J7</f>
+      <c r="J7" s="161">
+        <f>F7-D7-H7</f>
         <v>38.70879999999999</v>
       </c>
-      <c r="M7" s="162">
-        <f>N7/K16</f>
+      <c r="K7" s="160">
+        <f>L7/K14</f>
         <v>1.0080416666666663</v>
       </c>
-      <c r="N7" s="159">
-        <f>H7*(I16-1)</f>
+      <c r="L7" s="161">
+        <f>F7*(I14-1)</f>
         <v>51.61173333333331</v>
       </c>
-      <c r="O7" s="162">
-        <f>P7/K16</f>
+      <c r="M7" s="160">
+        <f>N7/K14</f>
         <v>3.5281458333333324</v>
       </c>
-      <c r="P7" s="163">
-        <f>H7*I16</f>
+      <c r="N7" s="162">
+        <f>F7*I14</f>
         <v>180.64106666666663</v>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="164" t="inlineStr">
-        <is>
-          <t>ДО · Gouda Cheese, Carbonara Spicy</t>
-        </is>
-      </c>
-      <c r="C8" s="158" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D8" s="165">
-        <f>C8*K16</f>
-        <v>38.400000000000006</v>
-      </c>
-      <c r="E8" s="160">
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="163" t="str">
+        <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
+        <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
+      </c>
+      <c r="C8" s="158">
         <f>'Финмодель 6 паллет'!E11</f>
         <v>1.308515625</v>
       </c>
-      <c r="F8" s="166">
-        <f>E8*K16</f>
+      <c r="D8" s="164">
+        <f>C8*K14</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="G8" s="167">
-        <f>H8/K16</f>
+      <c r="E8" s="165">
+        <f>F8/K14</f>
         <v>2.9078125000000004</v>
       </c>
+      <c r="F8" s="164">
+        <f>D8/(1-G14-E14)</f>
+        <v>148.88000000000002</v>
+      </c>
+      <c r="G8" s="165">
+        <f>H8/K14</f>
+        <v>0.7269531250000001</v>
+      </c>
       <c r="H8" s="166">
-        <f>F8/(1-G16-E16)</f>
-        <v>148.88000000000002</v>
-      </c>
-      <c r="I8" s="167">
-        <f>J8/K16</f>
-        <v>0.7269531250000001</v>
-      </c>
-      <c r="J8" s="165">
-        <f>H8*G16</f>
+        <f>F8*G14</f>
         <v>37.220000000000006</v>
       </c>
-      <c r="K8" s="167">
-        <f>L8/K16</f>
+      <c r="I8" s="165">
+        <f>J8/K14</f>
         <v>0.8723437500000001</v>
       </c>
-      <c r="L8" s="165">
-        <f>H8-F8-J8</f>
+      <c r="J8" s="166">
+        <f>F8-D8-H8</f>
         <v>44.66400000000001</v>
       </c>
-      <c r="M8" s="167">
-        <f>N8/K16</f>
+      <c r="K8" s="165">
+        <f>L8/K14</f>
         <v>1.163125</v>
       </c>
-      <c r="N8" s="165">
-        <f>H8*(I16-1)</f>
+      <c r="L8" s="166">
+        <f>F8*(I14-1)</f>
         <v>59.552</v>
       </c>
-      <c r="O8" s="167">
-        <f>P8/K16</f>
+      <c r="M8" s="165">
+        <f>N8/K14</f>
         <v>4.0709375</v>
       </c>
-      <c r="P8" s="168">
-        <f>H8*I16</f>
+      <c r="N8" s="167">
+        <f>F8*I14</f>
         <v>208.43200000000002</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="169" t="inlineStr">
-        <is>
-          <t>ПОСЛЕ · запрос SIAS (все 6 SKU)</t>
-        </is>
-      </c>
-      <c r="C9" s="170">
-        <f>C22</f>
-        <v>0.32</v>
-      </c>
-      <c r="D9" s="171">
-        <f>C9*K16</f>
-        <v>16.384</v>
-      </c>
-      <c r="E9" s="172">
-        <f>F9/K16</f>
+    <row r="9" ht="32" customHeight="1">
+      <c r="B9" s="168" t="str">
+        <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
+        <v>ПОСЛЕ · запрос SIAS €0.32 (все 6 SKU)</v>
+      </c>
+      <c r="C9" s="169">
+        <f>D9/K14</f>
         <v>0.7453031249999998</v>
       </c>
-      <c r="F9" s="173">
-        <f>(C9*K16+(E19+G19+I19)/(M19*O19)*K16+(C9+E19*K19/(M19*O19))*C19*K16+(C9+E19*K19/(M19*O19))*(1+C19)*O16*K16)*(1+M16)</f>
+      <c r="D9" s="170">
+        <f>C23</f>
         <v>38.15951999999999</v>
       </c>
-      <c r="G9" s="174">
-        <f>H9/K16</f>
+      <c r="E9" s="169">
+        <f>F9/K14</f>
         <v>1.6562291666666664</v>
       </c>
-      <c r="H9" s="173">
-        <f>F9/(1-G16-E16)</f>
+      <c r="F9" s="170">
+        <f>D9/(1-G14-E14)</f>
         <v>84.79893333333332</v>
       </c>
-      <c r="I9" s="174">
-        <f>J9/K16</f>
+      <c r="G9" s="169">
+        <f>H9/K14</f>
         <v>0.4140572916666666</v>
       </c>
+      <c r="H9" s="171">
+        <f>F9*G14</f>
+        <v>21.19973333333333</v>
+      </c>
+      <c r="I9" s="169">
+        <f>J9/K14</f>
+        <v>0.49686874999999997</v>
+      </c>
       <c r="J9" s="171">
-        <f>H9*G16</f>
-        <v>21.19973333333333</v>
-      </c>
-      <c r="K9" s="174">
-        <f>L9/K16</f>
-        <v>0.49686874999999997</v>
+        <f>F9-D9-H9</f>
+        <v>25.43968</v>
+      </c>
+      <c r="K9" s="169">
+        <f>L9/K14</f>
+        <v>0.6624916666666665</v>
       </c>
       <c r="L9" s="171">
-        <f>H9-F9-J9</f>
-        <v>25.43968</v>
-      </c>
-      <c r="M9" s="174">
-        <f>N9/K16</f>
-        <v>0.6624916666666665</v>
-      </c>
-      <c r="N9" s="171">
-        <f>H9*(I16-1)</f>
+        <f>F9*(I14-1)</f>
         <v>33.919573333333325</v>
       </c>
-      <c r="O9" s="174">
-        <f>P9/K16</f>
+      <c r="M9" s="169">
+        <f>N9/K14</f>
         <v>2.318720833333333</v>
       </c>
-      <c r="P9" s="175">
-        <f>H9*I16</f>
+      <c r="N9" s="172">
+        <f>F9*I14</f>
         <v>118.71850666666664</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="176" t="inlineStr">
+      <c r="B10" s="173" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="177">
+      <c r="C10" s="174">
         <f>C9-C7</f>
-        <v>-0.33</v>
-      </c>
-      <c r="D10" s="178">
+        <v>-0.38874375000000005</v>
+      </c>
+      <c r="D10" s="175">
         <f>D9-D7</f>
-        <v>-16.896</v>
-      </c>
-      <c r="E10" s="177">
+        <v>-19.90368</v>
+      </c>
+      <c r="E10" s="174">
         <f>E9-E7</f>
-        <v>-0.38874375000000005</v>
-      </c>
-      <c r="F10" s="178">
+        <v>-0.8638749999999997</v>
+      </c>
+      <c r="F10" s="175">
         <f>F9-F7</f>
-        <v>-19.90368</v>
-      </c>
-      <c r="G10" s="177">
+        <v>-44.23039999999999</v>
+      </c>
+      <c r="G10" s="174">
         <f>G9-G7</f>
-        <v>-0.8638749999999997</v>
-      </c>
-      <c r="H10" s="178">
+        <v>-0.21596874999999993</v>
+      </c>
+      <c r="H10" s="175">
         <f>H9-H7</f>
-        <v>-44.23039999999999</v>
-      </c>
-      <c r="I10" s="177">
+        <v>-11.057599999999997</v>
+      </c>
+      <c r="I10" s="174">
         <f>I9-I7</f>
-        <v>-0.21596874999999993</v>
-      </c>
-      <c r="J10" s="178">
+        <v>-0.25916249999999974</v>
+      </c>
+      <c r="J10" s="175">
         <f>J9-J7</f>
-        <v>-11.057599999999997</v>
-      </c>
-      <c r="K10" s="177">
+        <v>-13.26911999999999</v>
+      </c>
+      <c r="K10" s="174">
         <f>K9-K7</f>
-        <v>-0.25916249999999974</v>
-      </c>
-      <c r="L10" s="178">
+        <v>-0.3455499999999998</v>
+      </c>
+      <c r="L10" s="175">
         <f>L9-L7</f>
-        <v>-13.26911999999999</v>
-      </c>
-      <c r="M10" s="177">
+        <v>-17.692159999999987</v>
+      </c>
+      <c r="M10" s="174">
         <f>M9-M7</f>
-        <v>-0.3455499999999998</v>
-      </c>
-      <c r="N10" s="178">
+        <v>-1.2094249999999995</v>
+      </c>
+      <c r="N10" s="175">
         <f>N9-N7</f>
-        <v>-17.692159999999987</v>
-      </c>
-      <c r="O10" s="177">
-        <f>O9-O7</f>
-        <v>-1.2094249999999995</v>
-      </c>
-      <c r="P10" s="178">
-        <f>P9-P7</f>
         <v>-61.92255999999999</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="179" t="inlineStr">
-        <is>
-          <t>Читайте по строке слева направо: закупка → себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="180" t="inlineStr">
+      <c r="B11" s="176" t="inlineStr">
+        <is>
+          <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="177" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 6 паллет»</t>
         </is>
       </c>
-      <c r="C13" s="181" t="n"/>
-      <c r="D13" s="181" t="n"/>
-      <c r="E13" s="181" t="n"/>
-      <c r="F13" s="181" t="n"/>
-      <c r="G13" s="181" t="n"/>
-      <c r="H13" s="181" t="n"/>
-      <c r="I13" s="181" t="n"/>
-      <c r="J13" s="181" t="n"/>
-      <c r="K13" s="181" t="n"/>
-      <c r="L13" s="181" t="n"/>
-      <c r="M13" s="181" t="n"/>
-      <c r="N13" s="181" t="n"/>
-      <c r="O13" s="181" t="n"/>
-      <c r="P13" s="181" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="C15" s="182" t="inlineStr">
+      <c r="C12" s="178" t="n"/>
+      <c r="D12" s="178" t="n"/>
+      <c r="E12" s="178" t="n"/>
+      <c r="F12" s="178" t="n"/>
+      <c r="G12" s="178" t="n"/>
+      <c r="H12" s="178" t="n"/>
+      <c r="I12" s="178" t="n"/>
+      <c r="J12" s="178" t="n"/>
+      <c r="K12" s="178" t="n"/>
+      <c r="L12" s="178" t="n"/>
+      <c r="M12" s="178" t="n"/>
+      <c r="N12" s="178" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="C13" s="179" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E15" s="182" t="inlineStr">
+      <c r="E13" s="179" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G15" s="182" t="inlineStr">
+      <c r="G13" s="179" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I15" s="182" t="inlineStr">
+      <c r="I13" s="179" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K15" s="182" t="inlineStr">
+      <c r="K13" s="179" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
-      <c r="M15" s="182" t="inlineStr">
-        <is>
-          <t>Финансирование</t>
-        </is>
-      </c>
-      <c r="O15" s="182" t="inlineStr">
-        <is>
-          <t>Импортный ПДВ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="183" t="inlineStr">
-        <is>
-          <t>Цель расчёта</t>
-        </is>
-      </c>
-      <c r="C16" s="184" t="n">
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="180" t="inlineStr">
+        <is>
+          <t>Цель расчёта и условия модели</t>
+        </is>
+      </c>
+      <c r="C14" s="181" t="n">
         <v>120</v>
       </c>
-      <c r="D16" s="185" t="n"/>
-      <c r="E16" s="186" t="n">
+      <c r="D14" s="182" t="n"/>
+      <c r="E14" s="183" t="n">
         <v>0.3</v>
       </c>
-      <c r="F16" s="185" t="n"/>
-      <c r="G16" s="187">
+      <c r="F14" s="182" t="n"/>
+      <c r="G14" s="184">
         <f>'Финмодель 6 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H16" s="188" t="n"/>
-      <c r="I16" s="189">
+      <c r="H14" s="185" t="n"/>
+      <c r="I14" s="186">
         <f>'Финмодель 6 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J16" s="188" t="n"/>
-      <c r="K16" s="190">
+      <c r="J14" s="185" t="n"/>
+      <c r="K14" s="187">
         <f>'Финмодель 6 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L16" s="188" t="n"/>
-      <c r="M16" s="186" t="n">
+      <c r="L14" s="185" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="188" t="inlineStr">
+        <is>
+          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1">
+      <c r="C16" s="179" t="inlineStr">
+        <is>
+          <t>Импортный ПДВ</t>
+        </is>
+      </c>
+      <c r="E16" s="179" t="inlineStr">
+        <is>
+          <t>Финансирование</t>
+        </is>
+      </c>
+      <c r="G16" s="179" t="inlineStr">
+        <is>
+          <t>Пошлина</t>
+        </is>
+      </c>
+      <c r="I16" s="179" t="inlineStr">
+        <is>
+          <t>Перевозка партии, €</t>
+        </is>
+      </c>
+      <c r="K16" s="179" t="inlineStr">
+        <is>
+          <t>Брокер, €</t>
+        </is>
+      </c>
+      <c r="M16" s="179" t="inlineStr">
+        <is>
+          <t>Прочие, €</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" hidden="1">
+      <c r="C17" s="183" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="182" t="n"/>
+      <c r="E17" s="183" t="n">
         <v>0.025</v>
       </c>
-      <c r="N16" s="185" t="n"/>
-      <c r="O16" s="186" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P16" s="185" t="n"/>
-    </row>
-    <row r="18" hidden="1" ht="22" customHeight="1">
-      <c r="C18" s="182" t="inlineStr">
-        <is>
-          <t>Пошлина</t>
-        </is>
-      </c>
-      <c r="E18" s="182" t="inlineStr">
-        <is>
-          <t>Перевозка партии, €</t>
-        </is>
-      </c>
-      <c r="G18" s="182" t="inlineStr">
-        <is>
-          <t>Брокер, €</t>
-        </is>
-      </c>
-      <c r="I18" s="182" t="inlineStr">
-        <is>
-          <t>Прочие, €</t>
-        </is>
-      </c>
-      <c r="K18" s="182" t="inlineStr">
+      <c r="F17" s="182" t="n"/>
+      <c r="G17" s="183" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="182" t="n"/>
+      <c r="I17" s="189" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J17" s="182" t="n"/>
+      <c r="K17" s="189" t="n">
+        <v>288</v>
+      </c>
+      <c r="L17" s="182" t="n"/>
+      <c r="M17" s="189" t="n">
+        <v>42</v>
+      </c>
+      <c r="N17" s="182" t="n"/>
+    </row>
+    <row r="18" hidden="1">
+      <c r="C18" s="179" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="M18" s="182" t="inlineStr">
+      <c r="E18" s="179" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="O18" s="182" t="inlineStr">
+      <c r="G18" s="179" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
-    <row r="19" hidden="1" ht="22" customHeight="1">
-      <c r="B19" s="183" t="inlineStr">
-        <is>
-          <t>Расходы партии (Self-Cost_Sias)</t>
-        </is>
-      </c>
-      <c r="C19" s="186" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="185" t="n"/>
-      <c r="E19" s="191" t="n">
-        <v>2600</v>
-      </c>
-      <c r="F19" s="185" t="n"/>
-      <c r="G19" s="191" t="n">
-        <v>288</v>
-      </c>
-      <c r="H19" s="185" t="n"/>
-      <c r="I19" s="191" t="n">
-        <v>42</v>
-      </c>
-      <c r="J19" s="185" t="n"/>
-      <c r="K19" s="192" t="n">
+    <row r="19" hidden="1">
+      <c r="C19" s="190" t="n">
         <v>0.7</v>
       </c>
-      <c r="L19" s="185" t="n"/>
-      <c r="M19" s="191" t="n">
+      <c r="D19" s="182" t="n"/>
+      <c r="E19" s="189" t="n">
         <v>6</v>
       </c>
-      <c r="N19" s="185" t="n"/>
-      <c r="O19" s="191" t="n">
+      <c r="F19" s="182" t="n"/>
+      <c r="G19" s="189" t="n">
         <v>1600</v>
       </c>
-      <c r="P19" s="185" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="180" t="inlineStr">
-        <is>
-          <t>КАК ПОЛУЧЕН ЗАПРОС: из полки 120 ₴ обратно к закупке</t>
-        </is>
-      </c>
-      <c r="C21" s="181" t="n"/>
-      <c r="D21" s="181" t="n"/>
-      <c r="E21" s="181" t="n"/>
-      <c r="F21" s="181" t="n"/>
-      <c r="G21" s="181" t="n"/>
-      <c r="H21" s="181" t="n"/>
-      <c r="I21" s="181" t="n"/>
-      <c r="J21" s="181" t="n"/>
-      <c r="K21" s="181" t="n"/>
-      <c r="L21" s="181" t="n"/>
-      <c r="M21" s="181" t="n"/>
-      <c r="N21" s="181" t="n"/>
-      <c r="O21" s="181" t="n"/>
-      <c r="P21" s="181" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="193" t="inlineStr">
+      <c r="H19" s="182" t="n"/>
+    </row>
+    <row r="20" hidden="1">
+      <c r="B20" s="191" t="inlineStr">
+        <is>
+          <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
+        </is>
+      </c>
+      <c r="C20" s="190" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E20" s="190" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="21" hidden="1">
+      <c r="B21" s="191" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
+      <c r="C21" s="192">
+        <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
+        <v>0.32</v>
+      </c>
+      <c r="D21" s="193" t="n"/>
+    </row>
+    <row r="22" hidden="1">
+      <c r="B22" s="191" t="inlineStr">
+        <is>
+          <t>Предельная закупка до округления, €/уп.</t>
+        </is>
+      </c>
       <c r="C22" s="194">
-        <f>ROUNDDOWN(((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16)),2)</f>
-        <v>0.32</v>
+        <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
+        <v>0.3265407229965157</v>
       </c>
       <c r="D22" s="195" t="n"/>
-      <c r="E22" s="196" t="inlineStr">
-        <is>
-          <t>Считаем от полки 120 ₴ назад: цена партнёру → допустимая себестоимость → предельная закупка, округлено вниз до евроцента.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="197" t="inlineStr">
-        <is>
-          <t>Предельная закупка до округления, €/уп.</t>
-        </is>
-      </c>
-      <c r="C23" s="198">
-        <f>((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16))</f>
-        <v>0.3265407229965157</v>
-      </c>
-      <c r="D23" s="199" t="n"/>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="B24" s="200" t="inlineStr">
-        <is>
-          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); импортный ПДВ входит в себестоимость, как в Self-Cost; без листинг-фи, промо и отсрочки; согласие SIAS не получено — цена для переговоров.</t>
-        </is>
-      </c>
+    </row>
+    <row r="23" hidden="1">
+      <c r="B23" s="191" t="inlineStr">
+        <is>
+          <t>Себестоимость в Украине при запросе, ₴/уп.</t>
+        </is>
+      </c>
+      <c r="C23" s="196">
+        <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
+        <v>38.15951999999999</v>
+      </c>
+      <c r="D23" s="195" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="42">
     <mergeCell ref="K16:L16"/>
-    <mergeCell ref="B11:P11"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="K15:L15"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="K5:L5"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="C14:D14"/>
     <mergeCell ref="M5:N5"/>
-    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="I16:J16"/>
-    <mergeCell ref="O5:P5"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="G19:H19"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="G13:H13"/>
     <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="B3:N3"/>
     <mergeCell ref="M16:N16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="B24:P24"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="B12:N12"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E22:P22"/>
     <mergeCell ref="I5:J5"/>
-    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="B11:N11"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="K17:L17"/>
     <mergeCell ref="C23:D23"/>
+    <mergeCell ref="M17:N17"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:H16"/>
-    <mergeCell ref="B3:P3"/>
     <mergeCell ref="C19:D19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="I13:J13"/>
     <mergeCell ref="C18:D18"/>
+    <mergeCell ref="K13:L13"/>
     <mergeCell ref="E18:F18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="B21:P21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
@@ -6813,26 +6742,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:P24"/>
+  <dimension ref="B2:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="2" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="2" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6843,10 +6770,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="B3" s="152" t="str">
-        <f>"Чтобы полка стала "&amp;ROUND(C16,0)&amp;" ₴, закупка SIAS должна упасть с €"&amp;MIN(C7:C8)&amp;"–€"&amp;MAX(C7:C8)&amp;" до €"&amp;ROUND(C22,2)&amp;" за пачку (−"&amp;ROUND((1-C22/MIN(C7:C8))*100,0)&amp;"…"&amp;ROUND((1-C22/MAX(C7:C8))*100,0)&amp;"%). Маржа остаётся "&amp;ROUND(E16*100,0)&amp;"%."</f>
-        <v>Чтобы полка стала 120 ₴, закупка SIAS должна упасть с €0.65–€0.75 до €0.54 за пачку (−17…28%). Маржа остаётся 30%.</v>
+        <f>"Полка "&amp;ROUND(C14,0)&amp;" ₴ достижима при себестоимости "&amp;ROUND(D9,2)&amp;" ₴ (сейчас "&amp;ROUND(D7,2)&amp;"–"&amp;ROUND(D8,2)&amp;" ₴). Для этого закупка SIAS должна быть €"&amp;ROUND(C21,2)&amp;" вместо €"&amp;MIN(C20,E20)&amp;"–€"&amp;MAX(C20,E20)&amp;" (−"&amp;ROUND((1-C21/MIN(C20,E20))*100,0)&amp;"…"&amp;ROUND((1-C21/MAX(C20,E20))*100,0)&amp;"%)."</f>
+        <v>Полка 120 ₴ достижима при себестоимости 38.53 ₴ (сейчас 45.18–52.13 ₴). Для этого закупка SIAS должна быть €0.54 вместо €0.65–€0.75 (−17…28%).</v>
       </c>
       <c r="C3" s="153" t="n"/>
       <c r="D3" s="153" t="n"/>
@@ -6860,53 +6787,45 @@
       <c r="L3" s="153" t="n"/>
       <c r="M3" s="153" t="n"/>
       <c r="N3" s="153" t="n"/>
-      <c r="O3" s="153" t="n"/>
-      <c r="P3" s="153" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="154" t="inlineStr"/>
       <c r="C5" s="154" t="inlineStr">
         <is>
-          <t>Закупка SIAS</t>
+          <t>Себестоимость в Украине (СС)</t>
         </is>
       </c>
       <c r="D5" s="155" t="n"/>
       <c r="E5" s="154" t="inlineStr">
         <is>
-          <t>Себестоимость в Украине (СС)</t>
+          <t>Цена партнёру (магазину)</t>
         </is>
       </c>
       <c r="F5" s="155" t="n"/>
       <c r="G5" s="154" t="inlineStr">
         <is>
-          <t>Цена партнёру (магазину)</t>
+          <t>Бонус сети</t>
         </is>
       </c>
       <c r="H5" s="155" t="n"/>
       <c r="I5" s="154" t="inlineStr">
         <is>
-          <t>Бонус сети</t>
+          <t>Наша прибыль</t>
         </is>
       </c>
       <c r="J5" s="155" t="n"/>
       <c r="K5" s="154" t="inlineStr">
         <is>
-          <t>Наша прибыль</t>
+          <t>Наценка магазина</t>
         </is>
       </c>
       <c r="L5" s="155" t="n"/>
       <c r="M5" s="154" t="inlineStr">
         <is>
-          <t>Наценка магазина</t>
+          <t>ПОЛКА с НДС</t>
         </is>
       </c>
       <c r="N5" s="155" t="n"/>
-      <c r="O5" s="154" t="inlineStr">
-        <is>
-          <t>ПОЛКА с НДС</t>
-        </is>
-      </c>
-      <c r="P5" s="155" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="B6" s="154" t="inlineStr">
@@ -6974,545 +6893,496 @@
           <t>₴</t>
         </is>
       </c>
-      <c r="O6" s="156" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="P6" s="156" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="157" t="inlineStr">
-        <is>
-          <t>ДО · Vegetable, Spicy, Beef, Chicken</t>
-        </is>
-      </c>
-      <c r="C7" s="158" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D7" s="159">
-        <f>C7*K16</f>
-        <v>33.28</v>
-      </c>
-      <c r="E7" s="160">
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="157" t="str">
+        <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
+        <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
+      </c>
+      <c r="C7" s="158">
         <f>'Финмодель 33 паллет'!E13</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="F7" s="161">
-        <f>E7*K16</f>
+      <c r="D7" s="159">
+        <f>C7*K14</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="G7" s="162">
-        <f>H7/K16</f>
+      <c r="E7" s="160">
+        <f>F7/K14</f>
         <v>1.9608451859956246</v>
       </c>
+      <c r="F7" s="159">
+        <f>D7/(1-G14-E14)</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="G7" s="160">
+        <f>H7/K14</f>
+        <v>0.49021129649890616</v>
+      </c>
       <c r="H7" s="161">
-        <f>F7/(1-G16-E16)</f>
-        <v>100.39527352297598</v>
-      </c>
-      <c r="I7" s="162">
-        <f>J7/K16</f>
-        <v>0.49021129649890616</v>
-      </c>
-      <c r="J7" s="159">
-        <f>H7*G16</f>
+        <f>F7*G14</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="K7" s="162">
-        <f>L7/K16</f>
+      <c r="I7" s="160">
+        <f>J7/K14</f>
         <v>0.5882535557986873</v>
       </c>
-      <c r="L7" s="159">
-        <f>H7-F7-J7</f>
+      <c r="J7" s="161">
+        <f>F7-D7-H7</f>
         <v>30.118582056892794</v>
       </c>
-      <c r="M7" s="162">
-        <f>N7/K16</f>
+      <c r="K7" s="160">
+        <f>L7/K14</f>
         <v>0.7843380743982498</v>
       </c>
-      <c r="N7" s="159">
-        <f>H7*(I16-1)</f>
+      <c r="L7" s="161">
+        <f>F7*(I14-1)</f>
         <v>40.15810940919039</v>
       </c>
-      <c r="O7" s="162">
-        <f>P7/K16</f>
+      <c r="M7" s="160">
+        <f>N7/K14</f>
         <v>2.745183260393874</v>
       </c>
-      <c r="P7" s="163">
-        <f>H7*I16</f>
+      <c r="N7" s="162">
+        <f>F7*I14</f>
         <v>140.55338293216636</v>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="164" t="inlineStr">
-        <is>
-          <t>ДО · Gouda Cheese, Carbonara Spicy</t>
-        </is>
-      </c>
-      <c r="C8" s="158" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D8" s="165">
-        <f>C8*K16</f>
-        <v>38.400000000000006</v>
-      </c>
-      <c r="E8" s="160">
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="163" t="str">
+        <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
+        <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
+      </c>
+      <c r="C8" s="158">
         <f>'Финмодель 33 паллет'!E11</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="F8" s="166">
-        <f>E8*K16</f>
+      <c r="D8" s="164">
+        <f>C8*K14</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="G8" s="167">
-        <f>H8/K16</f>
+      <c r="E8" s="165">
+        <f>F8/K14</f>
         <v>2.2625136761487954</v>
       </c>
+      <c r="F8" s="164">
+        <f>D8/(1-G14-E14)</f>
+        <v>115.84070021881833</v>
+      </c>
+      <c r="G8" s="165">
+        <f>H8/K14</f>
+        <v>0.5656284190371988</v>
+      </c>
       <c r="H8" s="166">
-        <f>F8/(1-G16-E16)</f>
-        <v>115.84070021881833</v>
-      </c>
-      <c r="I8" s="167">
-        <f>J8/K16</f>
-        <v>0.5656284190371988</v>
-      </c>
-      <c r="J8" s="165">
-        <f>H8*G16</f>
+        <f>F8*G14</f>
         <v>28.96017505470458</v>
       </c>
-      <c r="K8" s="167">
-        <f>L8/K16</f>
+      <c r="I8" s="165">
+        <f>J8/K14</f>
         <v>0.6787541028446387</v>
       </c>
-      <c r="L8" s="165">
-        <f>H8-F8-J8</f>
+      <c r="J8" s="166">
+        <f>F8-D8-H8</f>
         <v>34.7522100656455</v>
       </c>
-      <c r="M8" s="167">
-        <f>N8/K16</f>
+      <c r="K8" s="165">
+        <f>L8/K14</f>
         <v>0.905005470459518</v>
       </c>
-      <c r="N8" s="165">
-        <f>H8*(I16-1)</f>
+      <c r="L8" s="166">
+        <f>F8*(I14-1)</f>
         <v>46.33628008752732</v>
       </c>
-      <c r="O8" s="167">
-        <f>P8/K16</f>
+      <c r="M8" s="165">
+        <f>N8/K14</f>
         <v>3.1675191466083135</v>
       </c>
-      <c r="P8" s="168">
-        <f>H8*I16</f>
+      <c r="N8" s="167">
+        <f>F8*I14</f>
         <v>162.17698030634565</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="169" t="inlineStr">
-        <is>
-          <t>ПОСЛЕ · запрос SIAS (все 6 SKU)</t>
-        </is>
-      </c>
-      <c r="C9" s="170">
-        <f>C22</f>
-        <v>0.54</v>
-      </c>
-      <c r="D9" s="171">
-        <f>C9*K16</f>
-        <v>27.648000000000003</v>
-      </c>
-      <c r="E9" s="172">
-        <f>F9/K16</f>
+    <row r="9" ht="32" customHeight="1">
+      <c r="B9" s="168" t="str">
+        <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
+        <v>ПОСЛЕ · запрос SIAS €0.54 (все 6 SKU)</v>
+      </c>
+      <c r="C9" s="169">
+        <f>D9/K14</f>
         <v>0.7524897727272728</v>
       </c>
-      <c r="F9" s="173">
-        <f>(C9*K16+(E19+G19+I19)/(M19*O19)*K16+(C9+E19*K19/(M19*O19))*C19*K16+(C9+E19*K19/(M19*O19))*(1+C19)*O16*K16)*(1+M16)</f>
+      <c r="D9" s="170">
+        <f>C23</f>
         <v>38.52747636363637</v>
       </c>
-      <c r="G9" s="174">
-        <f>H9/K16</f>
+      <c r="E9" s="169">
+        <f>F9/K14</f>
         <v>1.672199494949495</v>
       </c>
-      <c r="H9" s="173">
-        <f>F9/(1-G16-E16)</f>
+      <c r="F9" s="170">
+        <f>D9/(1-G14-E14)</f>
         <v>85.61661414141415</v>
       </c>
-      <c r="I9" s="174">
-        <f>J9/K16</f>
+      <c r="G9" s="169">
+        <f>H9/K14</f>
         <v>0.41804987373737373</v>
       </c>
+      <c r="H9" s="171">
+        <f>F9*G14</f>
+        <v>21.404153535353537</v>
+      </c>
+      <c r="I9" s="169">
+        <f>J9/K14</f>
+        <v>0.5016598484848485</v>
+      </c>
       <c r="J9" s="171">
-        <f>H9*G16</f>
-        <v>21.404153535353537</v>
-      </c>
-      <c r="K9" s="174">
-        <f>L9/K16</f>
-        <v>0.5016598484848485</v>
+        <f>F9-D9-H9</f>
+        <v>25.684984242424242</v>
+      </c>
+      <c r="K9" s="169">
+        <f>L9/K14</f>
+        <v>0.6688797979797979</v>
       </c>
       <c r="L9" s="171">
-        <f>H9-F9-J9</f>
-        <v>25.684984242424242</v>
-      </c>
-      <c r="M9" s="174">
-        <f>N9/K16</f>
-        <v>0.6688797979797979</v>
-      </c>
-      <c r="N9" s="171">
-        <f>H9*(I16-1)</f>
+        <f>F9*(I14-1)</f>
         <v>34.246645656565654</v>
       </c>
-      <c r="O9" s="174">
-        <f>P9/K16</f>
+      <c r="M9" s="169">
+        <f>N9/K14</f>
         <v>2.3410792929292925</v>
       </c>
-      <c r="P9" s="175">
-        <f>H9*I16</f>
+      <c r="N9" s="172">
+        <f>F9*I14</f>
         <v>119.8632597979798</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="176" t="inlineStr">
+      <c r="B10" s="173" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="177">
+      <c r="C10" s="174">
         <f>C9-C7</f>
-        <v>-0.10999999999999999</v>
-      </c>
-      <c r="D10" s="178">
+        <v>-0.12989056097075824</v>
+      </c>
+      <c r="D10" s="175">
         <f>D9-D7</f>
-        <v>-5.631999999999998</v>
-      </c>
-      <c r="E10" s="177">
+        <v>-6.650396721702826</v>
+      </c>
+      <c r="E10" s="174">
         <f>E9-E7</f>
-        <v>-0.12989056097075824</v>
-      </c>
-      <c r="F10" s="178">
+        <v>-0.2886456910461297</v>
+      </c>
+      <c r="F10" s="175">
         <f>F9-F7</f>
-        <v>-6.650396721702826</v>
-      </c>
-      <c r="G10" s="177">
+        <v>-14.778659381561837</v>
+      </c>
+      <c r="G10" s="174">
         <f>G9-G7</f>
-        <v>-0.2886456910461297</v>
-      </c>
-      <c r="H10" s="178">
+        <v>-0.07216142276153242</v>
+      </c>
+      <c r="H10" s="175">
         <f>H9-H7</f>
-        <v>-14.778659381561837</v>
-      </c>
-      <c r="I10" s="177">
+        <v>-3.6946648453904594</v>
+      </c>
+      <c r="I10" s="174">
         <f>I9-I7</f>
-        <v>-0.07216142276153242</v>
-      </c>
-      <c r="J10" s="178">
+        <v>-0.08659370731383886</v>
+      </c>
+      <c r="J10" s="175">
         <f>J9-J7</f>
-        <v>-3.6946648453904594</v>
-      </c>
-      <c r="K10" s="177">
+        <v>-4.433597814468552</v>
+      </c>
+      <c r="K10" s="174">
         <f>K9-K7</f>
-        <v>-0.08659370731383886</v>
-      </c>
-      <c r="L10" s="178">
+        <v>-0.11545827641845186</v>
+      </c>
+      <c r="L10" s="175">
         <f>L9-L7</f>
-        <v>-4.433597814468552</v>
-      </c>
-      <c r="M10" s="177">
+        <v>-5.911463752624734</v>
+      </c>
+      <c r="M10" s="174">
         <f>M9-M7</f>
-        <v>-0.11545827641845186</v>
-      </c>
-      <c r="N10" s="178">
+        <v>-0.40410396746458144</v>
+      </c>
+      <c r="N10" s="175">
         <f>N9-N7</f>
-        <v>-5.911463752624734</v>
-      </c>
-      <c r="O10" s="177">
-        <f>O9-O7</f>
-        <v>-0.40410396746458144</v>
-      </c>
-      <c r="P10" s="178">
-        <f>P9-P7</f>
         <v>-20.690123134186564</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="179" t="inlineStr">
-        <is>
-          <t>Читайте по строке слева направо: закупка → себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="180" t="inlineStr">
+      <c r="B11" s="176" t="inlineStr">
+        <is>
+          <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="177" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 33 паллет»</t>
         </is>
       </c>
-      <c r="C13" s="181" t="n"/>
-      <c r="D13" s="181" t="n"/>
-      <c r="E13" s="181" t="n"/>
-      <c r="F13" s="181" t="n"/>
-      <c r="G13" s="181" t="n"/>
-      <c r="H13" s="181" t="n"/>
-      <c r="I13" s="181" t="n"/>
-      <c r="J13" s="181" t="n"/>
-      <c r="K13" s="181" t="n"/>
-      <c r="L13" s="181" t="n"/>
-      <c r="M13" s="181" t="n"/>
-      <c r="N13" s="181" t="n"/>
-      <c r="O13" s="181" t="n"/>
-      <c r="P13" s="181" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="C15" s="182" t="inlineStr">
+      <c r="C12" s="178" t="n"/>
+      <c r="D12" s="178" t="n"/>
+      <c r="E12" s="178" t="n"/>
+      <c r="F12" s="178" t="n"/>
+      <c r="G12" s="178" t="n"/>
+      <c r="H12" s="178" t="n"/>
+      <c r="I12" s="178" t="n"/>
+      <c r="J12" s="178" t="n"/>
+      <c r="K12" s="178" t="n"/>
+      <c r="L12" s="178" t="n"/>
+      <c r="M12" s="178" t="n"/>
+      <c r="N12" s="178" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="C13" s="179" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E15" s="182" t="inlineStr">
+      <c r="E13" s="179" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G15" s="182" t="inlineStr">
+      <c r="G13" s="179" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I15" s="182" t="inlineStr">
+      <c r="I13" s="179" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K15" s="182" t="inlineStr">
+      <c r="K13" s="179" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
-      <c r="M15" s="182" t="inlineStr">
-        <is>
-          <t>Финансирование</t>
-        </is>
-      </c>
-      <c r="O15" s="182" t="inlineStr">
-        <is>
-          <t>Импортный ПДВ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="183" t="inlineStr">
-        <is>
-          <t>Цель расчёта</t>
-        </is>
-      </c>
-      <c r="C16" s="184" t="n">
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="180" t="inlineStr">
+        <is>
+          <t>Цель расчёта и условия модели</t>
+        </is>
+      </c>
+      <c r="C14" s="181" t="n">
         <v>120</v>
       </c>
-      <c r="D16" s="185" t="n"/>
-      <c r="E16" s="186" t="n">
+      <c r="D14" s="182" t="n"/>
+      <c r="E14" s="183" t="n">
         <v>0.3</v>
       </c>
-      <c r="F16" s="185" t="n"/>
-      <c r="G16" s="187">
+      <c r="F14" s="182" t="n"/>
+      <c r="G14" s="184">
         <f>'Финмодель 33 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H16" s="188" t="n"/>
-      <c r="I16" s="189">
+      <c r="H14" s="185" t="n"/>
+      <c r="I14" s="186">
         <f>'Финмодель 33 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J16" s="188" t="n"/>
-      <c r="K16" s="190">
+      <c r="J14" s="185" t="n"/>
+      <c r="K14" s="187">
         <f>'Финмодель 33 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L16" s="188" t="n"/>
-      <c r="M16" s="186" t="n">
+      <c r="L14" s="185" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="188" t="inlineStr">
+        <is>
+          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1">
+      <c r="C16" s="179" t="inlineStr">
+        <is>
+          <t>Импортный ПДВ</t>
+        </is>
+      </c>
+      <c r="E16" s="179" t="inlineStr">
+        <is>
+          <t>Финансирование</t>
+        </is>
+      </c>
+      <c r="G16" s="179" t="inlineStr">
+        <is>
+          <t>Пошлина</t>
+        </is>
+      </c>
+      <c r="I16" s="179" t="inlineStr">
+        <is>
+          <t>Перевозка партии, €</t>
+        </is>
+      </c>
+      <c r="K16" s="179" t="inlineStr">
+        <is>
+          <t>Брокер, €</t>
+        </is>
+      </c>
+      <c r="M16" s="179" t="inlineStr">
+        <is>
+          <t>Прочие, €</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" hidden="1">
+      <c r="C17" s="183" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="182" t="n"/>
+      <c r="E17" s="183" t="n">
         <v>0.025</v>
       </c>
-      <c r="N16" s="185" t="n"/>
-      <c r="O16" s="186" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P16" s="185" t="n"/>
-    </row>
-    <row r="18" hidden="1" ht="22" customHeight="1">
-      <c r="C18" s="182" t="inlineStr">
-        <is>
-          <t>Пошлина</t>
-        </is>
-      </c>
-      <c r="E18" s="182" t="inlineStr">
-        <is>
-          <t>Перевозка партии, €</t>
-        </is>
-      </c>
-      <c r="G18" s="182" t="inlineStr">
-        <is>
-          <t>Брокер, €</t>
-        </is>
-      </c>
-      <c r="I18" s="182" t="inlineStr">
-        <is>
-          <t>Прочие, €</t>
-        </is>
-      </c>
-      <c r="K18" s="182" t="inlineStr">
+      <c r="F17" s="182" t="n"/>
+      <c r="G17" s="183" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="182" t="n"/>
+      <c r="I17" s="189" t="n">
+        <v>3700</v>
+      </c>
+      <c r="J17" s="182" t="n"/>
+      <c r="K17" s="189" t="n">
+        <v>288</v>
+      </c>
+      <c r="L17" s="182" t="n"/>
+      <c r="M17" s="189" t="n">
+        <v>42</v>
+      </c>
+      <c r="N17" s="182" t="n"/>
+    </row>
+    <row r="18" hidden="1">
+      <c r="C18" s="179" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="M18" s="182" t="inlineStr">
+      <c r="E18" s="179" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="O18" s="182" t="inlineStr">
+      <c r="G18" s="179" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
-    <row r="19" hidden="1" ht="22" customHeight="1">
-      <c r="B19" s="183" t="inlineStr">
-        <is>
-          <t>Расходы партии (Self-Cost_Sias)</t>
-        </is>
-      </c>
-      <c r="C19" s="186" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="185" t="n"/>
-      <c r="E19" s="191" t="n">
-        <v>3700</v>
-      </c>
-      <c r="F19" s="185" t="n"/>
-      <c r="G19" s="191" t="n">
-        <v>288</v>
-      </c>
-      <c r="H19" s="185" t="n"/>
-      <c r="I19" s="191" t="n">
-        <v>42</v>
-      </c>
-      <c r="J19" s="185" t="n"/>
-      <c r="K19" s="192" t="n">
+    <row r="19" hidden="1">
+      <c r="C19" s="190" t="n">
         <v>0.7</v>
       </c>
-      <c r="L19" s="185" t="n"/>
-      <c r="M19" s="191" t="n">
+      <c r="D19" s="182" t="n"/>
+      <c r="E19" s="189" t="n">
         <v>33</v>
       </c>
-      <c r="N19" s="185" t="n"/>
-      <c r="O19" s="191" t="n">
+      <c r="F19" s="182" t="n"/>
+      <c r="G19" s="189" t="n">
         <v>1600</v>
       </c>
-      <c r="P19" s="185" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="180" t="inlineStr">
-        <is>
-          <t>КАК ПОЛУЧЕН ЗАПРОС: из полки 120 ₴ обратно к закупке</t>
-        </is>
-      </c>
-      <c r="C21" s="181" t="n"/>
-      <c r="D21" s="181" t="n"/>
-      <c r="E21" s="181" t="n"/>
-      <c r="F21" s="181" t="n"/>
-      <c r="G21" s="181" t="n"/>
-      <c r="H21" s="181" t="n"/>
-      <c r="I21" s="181" t="n"/>
-      <c r="J21" s="181" t="n"/>
-      <c r="K21" s="181" t="n"/>
-      <c r="L21" s="181" t="n"/>
-      <c r="M21" s="181" t="n"/>
-      <c r="N21" s="181" t="n"/>
-      <c r="O21" s="181" t="n"/>
-      <c r="P21" s="181" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="193" t="inlineStr">
+      <c r="H19" s="182" t="n"/>
+    </row>
+    <row r="20" hidden="1">
+      <c r="B20" s="191" t="inlineStr">
+        <is>
+          <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
+        </is>
+      </c>
+      <c r="C20" s="190" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E20" s="190" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="21" hidden="1">
+      <c r="B21" s="191" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
+      <c r="C21" s="192">
+        <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
+        <v>0.54</v>
+      </c>
+      <c r="D21" s="193" t="n"/>
+    </row>
+    <row r="22" hidden="1">
+      <c r="B22" s="191" t="inlineStr">
+        <is>
+          <t>Предельная закупка до округления, €/уп.</t>
+        </is>
+      </c>
       <c r="C22" s="194">
-        <f>ROUNDDOWN(((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16)),2)</f>
-        <v>0.54</v>
+        <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
+        <v>0.5406979199662126</v>
       </c>
       <c r="D22" s="195" t="n"/>
-      <c r="E22" s="196" t="inlineStr">
-        <is>
-          <t>Считаем от полки 120 ₴ назад: цена партнёру → допустимая себестоимость → предельная закупка, округлено вниз до евроцента.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="197" t="inlineStr">
-        <is>
-          <t>Предельная закупка до округления, €/уп.</t>
-        </is>
-      </c>
-      <c r="C23" s="198">
-        <f>((C16/I16*(1-G16-E16))/K16/(1+M16)-(E19+G19+I19+E19*K19*(C19+O16*(1+C19)))/(M19*O19))/((1+C19)*(1+O16))</f>
-        <v>0.5406979199662126</v>
-      </c>
-      <c r="D23" s="199" t="n"/>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="B24" s="200" t="inlineStr">
-        <is>
-          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); импортный ПДВ входит в себестоимость, как в Self-Cost; без листинг-фи, промо и отсрочки; согласие SIAS не получено — цена для переговоров.</t>
-        </is>
-      </c>
+    </row>
+    <row r="23" hidden="1">
+      <c r="B23" s="191" t="inlineStr">
+        <is>
+          <t>Себестоимость в Украине при запросе, ₴/уп.</t>
+        </is>
+      </c>
+      <c r="C23" s="196">
+        <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
+        <v>38.52747636363637</v>
+      </c>
+      <c r="D23" s="195" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="42">
     <mergeCell ref="K16:L16"/>
-    <mergeCell ref="B11:P11"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="K15:L15"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="K5:L5"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="C14:D14"/>
     <mergeCell ref="M5:N5"/>
-    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="I16:J16"/>
-    <mergeCell ref="O5:P5"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="G19:H19"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="G13:H13"/>
     <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="B3:N3"/>
     <mergeCell ref="M16:N16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="B24:P24"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="B12:N12"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E22:P22"/>
     <mergeCell ref="I5:J5"/>
-    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="B11:N11"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="K17:L17"/>
     <mergeCell ref="C23:D23"/>
+    <mergeCell ref="M17:N17"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:H16"/>
-    <mergeCell ref="B3:P3"/>
     <mergeCell ref="C19:D19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="I13:J13"/>
     <mergeCell ref="C18:D18"/>
+    <mergeCell ref="K13:L13"/>
     <mergeCell ref="E18:F18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="B21:P21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Finmodel: remove empty dark leftover blocks on tabs 1-2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
+++ b/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
@@ -814,7 +814,7 @@
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="197">
+  <cellXfs count="198">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1175,6 +1175,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="left" vertical="center"/>
@@ -1762,10 +1765,8 @@
       <c r="I2" s="123" t="n"/>
       <c r="J2" s="123" t="n"/>
       <c r="K2" s="122" t="n"/>
-      <c r="L2" s="7" t="n"/>
-      <c r="M2" s="121" t="n"/>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="121" t="n"/>
+      <c r="L2" s="124" t="n"/>
+      <c r="N2" s="124" t="n"/>
     </row>
     <row r="3" ht="37.5" customHeight="1">
       <c r="B3" s="1" t="inlineStr">
@@ -1788,10 +1789,8 @@
       <c r="I3" s="120" t="n"/>
       <c r="J3" s="120" t="n"/>
       <c r="K3" s="121" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="121" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="121" t="n"/>
+      <c r="L3" s="124" t="n"/>
+      <c r="N3" s="124" t="n"/>
     </row>
     <row r="4" ht="37.5" customHeight="1">
       <c r="B4" s="1" t="inlineStr">
@@ -1814,10 +1813,8 @@
       <c r="I4" s="120" t="n"/>
       <c r="J4" s="120" t="n"/>
       <c r="K4" s="121" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="121" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="121" t="n"/>
+      <c r="L4" s="124" t="n"/>
+      <c r="N4" s="124" t="n"/>
     </row>
     <row r="5" ht="61.5" customHeight="1">
       <c r="B5" s="1" t="inlineStr">
@@ -1840,10 +1837,8 @@
       <c r="I5" s="120" t="n"/>
       <c r="J5" s="120" t="n"/>
       <c r="K5" s="121" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="121" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="121" t="n"/>
+      <c r="L5" s="124" t="n"/>
+      <c r="N5" s="124" t="n"/>
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="B6" s="1" t="inlineStr">
@@ -1866,8 +1861,7 @@
       <c r="I6" s="120" t="n"/>
       <c r="J6" s="120" t="n"/>
       <c r="K6" s="121" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="121" t="n"/>
+      <c r="L6" s="124" t="n"/>
     </row>
     <row r="7" ht="27.75" customHeight="1">
       <c r="B7" s="1" t="inlineStr">
@@ -1892,8 +1886,7 @@
       <c r="I7" s="120" t="n"/>
       <c r="J7" s="120" t="n"/>
       <c r="K7" s="121" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="121" t="n"/>
+      <c r="L7" s="124" t="n"/>
     </row>
     <row r="8" ht="30" customFormat="1" customHeight="1" s="21">
       <c r="B8" s="80" t="inlineStr">
@@ -1901,12 +1894,12 @@
           <t>Частка ціни для собівартості</t>
         </is>
       </c>
-      <c r="C8" s="124" t="n"/>
+      <c r="C8" s="125" t="n"/>
       <c r="D8" s="24">
         <f>IF(AND(COUNT(D3:D6)=4,D3&gt;0,D4&gt;=0,D5&gt;=0,D4+D5&lt;1,D6&gt;0),1-D4-D5,NA())</f>
         <v>0.4</v>
       </c>
-      <c r="E8" s="125" t="inlineStr">
+      <c r="E8" s="126" t="inlineStr">
         <is>
           <t>100% − бонус − маржа. За поточних умов: 100% − 25% − 35% = 40%.</t>
         </is>
@@ -1958,34 +1951,34 @@
         </is>
       </c>
       <c r="O9" s="121" t="n"/>
-      <c r="P9" s="126" t="n">
+      <c r="P9" s="127" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q9" s="127" t="n"/>
-      <c r="R9" s="127" t="n"/>
-      <c r="S9" s="127" t="n"/>
-      <c r="T9" s="128" t="n"/>
-      <c r="U9" s="129" t="n">
+      <c r="Q9" s="128" t="n"/>
+      <c r="R9" s="128" t="n"/>
+      <c r="S9" s="128" t="n"/>
+      <c r="T9" s="129" t="n"/>
+      <c r="U9" s="130" t="n">
         <v>0.25</v>
       </c>
-      <c r="V9" s="127" t="n"/>
-      <c r="W9" s="127" t="n"/>
-      <c r="X9" s="127" t="n"/>
-      <c r="Y9" s="128" t="n"/>
-      <c r="Z9" s="126" t="n">
+      <c r="V9" s="128" t="n"/>
+      <c r="W9" s="128" t="n"/>
+      <c r="X9" s="128" t="n"/>
+      <c r="Y9" s="129" t="n"/>
+      <c r="Z9" s="127" t="n">
         <v>0.2</v>
       </c>
-      <c r="AA9" s="127" t="n"/>
-      <c r="AB9" s="127" t="n"/>
-      <c r="AC9" s="127" t="n"/>
-      <c r="AD9" s="128" t="n"/>
-      <c r="AE9" s="129" t="n">
+      <c r="AA9" s="128" t="n"/>
+      <c r="AB9" s="128" t="n"/>
+      <c r="AC9" s="128" t="n"/>
+      <c r="AD9" s="129" t="n"/>
+      <c r="AE9" s="130" t="n">
         <v>0.15</v>
       </c>
-      <c r="AF9" s="127" t="n"/>
-      <c r="AG9" s="127" t="n"/>
-      <c r="AH9" s="127" t="n"/>
-      <c r="AI9" s="128" t="n"/>
+      <c r="AF9" s="128" t="n"/>
+      <c r="AG9" s="128" t="n"/>
+      <c r="AH9" s="128" t="n"/>
+      <c r="AI9" s="129" t="n"/>
     </row>
     <row r="10" ht="41.4" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -2181,22 +2174,22 @@
       <c r="D11" s="8" t="n">
         <v>123</v>
       </c>
-      <c r="E11" s="130" t="n">
+      <c r="E11" s="131" t="n">
         <v>1.308515625</v>
       </c>
-      <c r="F11" s="131">
+      <c r="F11" s="132">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($D$8)),E11*$D$3,NA())</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="G11" s="132">
+      <c r="G11" s="133">
         <f>F11/$D$8</f>
         <v>167.49</v>
       </c>
-      <c r="H11" s="133">
+      <c r="H11" s="134">
         <f>G11*$D$4</f>
         <v>41.8725</v>
       </c>
-      <c r="I11" s="134">
+      <c r="I11" s="135">
         <f>G11-F11-H11</f>
         <v>58.6215</v>
       </c>
@@ -2204,35 +2197,35 @@
         <f>I11/G11</f>
         <v>0.35</v>
       </c>
-      <c r="K11" s="135">
+      <c r="K11" s="136">
         <f>G11*$D$6</f>
         <v>234.486</v>
       </c>
-      <c r="L11" s="136">
+      <c r="L11" s="137">
         <f>F11/(1-$D$4)</f>
         <v>89.32800000000002</v>
       </c>
-      <c r="M11" s="136">
+      <c r="M11" s="137">
         <f>L11*$D$6</f>
         <v>125.05920000000002</v>
       </c>
-      <c r="N11" s="137">
+      <c r="N11" s="138">
         <f>G11-F11</f>
         <v>100.494</v>
       </c>
-      <c r="O11" s="138">
+      <c r="O11" s="139">
         <f>N11-H11</f>
         <v>58.6215</v>
       </c>
-      <c r="P11" s="139">
+      <c r="P11" s="140">
         <f>$F11/(1-$D$4-$P$9)</f>
         <v>148.88000000000002</v>
       </c>
-      <c r="Q11" s="140">
+      <c r="Q11" s="141">
         <f>P11*$D$4</f>
         <v>37.220000000000006</v>
       </c>
-      <c r="R11" s="141">
+      <c r="R11" s="142">
         <f>P11-$F11-Q11</f>
         <v>44.66400000000001</v>
       </c>
@@ -2240,19 +2233,19 @@
         <f>R11/P11</f>
         <v>0.3</v>
       </c>
-      <c r="T11" s="139">
+      <c r="T11" s="140">
         <f>P11*$D$6</f>
         <v>208.43200000000002</v>
       </c>
-      <c r="U11" s="139">
+      <c r="U11" s="140">
         <f>$F11/(1-$D$4-$U$9)</f>
         <v>133.99200000000002</v>
       </c>
-      <c r="V11" s="140">
+      <c r="V11" s="141">
         <f>U11*$D$4</f>
         <v>33.498000000000005</v>
       </c>
-      <c r="W11" s="141">
+      <c r="W11" s="142">
         <f>U11-$F11-V11</f>
         <v>33.498000000000005</v>
       </c>
@@ -2260,19 +2253,19 @@
         <f>W11/U11</f>
         <v>0.25</v>
       </c>
-      <c r="Y11" s="139">
+      <c r="Y11" s="140">
         <f>U11*$D$6</f>
         <v>187.58880000000002</v>
       </c>
-      <c r="Z11" s="139">
+      <c r="Z11" s="140">
         <f>$F11/(1-$D$4-$Z$9)</f>
         <v>121.81090909090909</v>
       </c>
-      <c r="AA11" s="140">
+      <c r="AA11" s="141">
         <f>Z11*$D$4</f>
         <v>30.452727272727273</v>
       </c>
-      <c r="AB11" s="141">
+      <c r="AB11" s="142">
         <f>Z11-$F11-AA11</f>
         <v>24.36218181818181</v>
       </c>
@@ -2280,19 +2273,19 @@
         <f>AB11/Z11</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD11" s="139">
+      <c r="AD11" s="140">
         <f>Z11*$D$6</f>
         <v>170.5352727272727</v>
       </c>
-      <c r="AE11" s="139">
+      <c r="AE11" s="140">
         <f>$F11/(1-$D$4-$AE$9)</f>
         <v>111.66000000000003</v>
       </c>
-      <c r="AF11" s="140">
+      <c r="AF11" s="141">
         <f>AE11*$D$4</f>
         <v>27.915000000000006</v>
       </c>
-      <c r="AG11" s="141">
+      <c r="AG11" s="142">
         <f>AE11-$F11-AF11</f>
         <v>16.74900000000001</v>
       </c>
@@ -2300,7 +2293,7 @@
         <f>AG11/AE11</f>
         <v>0.15000000000000005</v>
       </c>
-      <c r="AI11" s="139">
+      <c r="AI11" s="140">
         <f>AE11*$D$6</f>
         <v>156.324</v>
       </c>
@@ -2322,22 +2315,22 @@
       <c r="D12" s="8" t="n">
         <v>131</v>
       </c>
-      <c r="E12" s="130" t="n">
+      <c r="E12" s="131" t="n">
         <v>1.308515625</v>
       </c>
-      <c r="F12" s="131">
+      <c r="F12" s="132">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($D$8)),E12*$D$3,NA())</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="G12" s="132">
+      <c r="G12" s="133">
         <f>F12/$D$8</f>
         <v>167.49</v>
       </c>
-      <c r="H12" s="133">
+      <c r="H12" s="134">
         <f>G12*$D$4</f>
         <v>41.8725</v>
       </c>
-      <c r="I12" s="134">
+      <c r="I12" s="135">
         <f>G12-F12-H12</f>
         <v>58.6215</v>
       </c>
@@ -2345,35 +2338,35 @@
         <f>I12/G12</f>
         <v>0.35</v>
       </c>
-      <c r="K12" s="135">
+      <c r="K12" s="136">
         <f>G12*$D$6</f>
         <v>234.486</v>
       </c>
-      <c r="L12" s="136">
+      <c r="L12" s="137">
         <f>F12/(1-$D$4)</f>
         <v>89.32800000000002</v>
       </c>
-      <c r="M12" s="136">
+      <c r="M12" s="137">
         <f>L12*$D$6</f>
         <v>125.05920000000002</v>
       </c>
-      <c r="N12" s="137">
+      <c r="N12" s="138">
         <f>G12-F12</f>
         <v>100.494</v>
       </c>
-      <c r="O12" s="138">
+      <c r="O12" s="139">
         <f>N12-H12</f>
         <v>58.6215</v>
       </c>
-      <c r="P12" s="139">
+      <c r="P12" s="140">
         <f>$F12/(1-$D$4-$P$9)</f>
         <v>148.88000000000002</v>
       </c>
-      <c r="Q12" s="140">
+      <c r="Q12" s="141">
         <f>P12*$D$4</f>
         <v>37.220000000000006</v>
       </c>
-      <c r="R12" s="141">
+      <c r="R12" s="142">
         <f>P12-$F12-Q12</f>
         <v>44.66400000000001</v>
       </c>
@@ -2381,19 +2374,19 @@
         <f>R12/P12</f>
         <v>0.3</v>
       </c>
-      <c r="T12" s="139">
+      <c r="T12" s="140">
         <f>P12*$D$6</f>
         <v>208.43200000000002</v>
       </c>
-      <c r="U12" s="139">
+      <c r="U12" s="140">
         <f>$F12/(1-$D$4-$U$9)</f>
         <v>133.99200000000002</v>
       </c>
-      <c r="V12" s="140">
+      <c r="V12" s="141">
         <f>U12*$D$4</f>
         <v>33.498000000000005</v>
       </c>
-      <c r="W12" s="141">
+      <c r="W12" s="142">
         <f>U12-$F12-V12</f>
         <v>33.498000000000005</v>
       </c>
@@ -2401,19 +2394,19 @@
         <f>W12/U12</f>
         <v>0.25</v>
       </c>
-      <c r="Y12" s="139">
+      <c r="Y12" s="140">
         <f>U12*$D$6</f>
         <v>187.58880000000002</v>
       </c>
-      <c r="Z12" s="139">
+      <c r="Z12" s="140">
         <f>$F12/(1-$D$4-$Z$9)</f>
         <v>121.81090909090909</v>
       </c>
-      <c r="AA12" s="140">
+      <c r="AA12" s="141">
         <f>Z12*$D$4</f>
         <v>30.452727272727273</v>
       </c>
-      <c r="AB12" s="141">
+      <c r="AB12" s="142">
         <f>Z12-$F12-AA12</f>
         <v>24.36218181818181</v>
       </c>
@@ -2421,19 +2414,19 @@
         <f>AB12/Z12</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD12" s="139">
+      <c r="AD12" s="140">
         <f>Z12*$D$6</f>
         <v>170.5352727272727</v>
       </c>
-      <c r="AE12" s="139">
+      <c r="AE12" s="140">
         <f>$F12/(1-$D$4-$AE$9)</f>
         <v>111.66000000000003</v>
       </c>
-      <c r="AF12" s="140">
+      <c r="AF12" s="141">
         <f>AE12*$D$4</f>
         <v>27.915000000000006</v>
       </c>
-      <c r="AG12" s="141">
+      <c r="AG12" s="142">
         <f>AE12-$F12-AF12</f>
         <v>16.74900000000001</v>
       </c>
@@ -2441,7 +2434,7 @@
         <f>AG12/AE12</f>
         <v>0.15000000000000005</v>
       </c>
-      <c r="AI12" s="139">
+      <c r="AI12" s="140">
         <f>AE12*$D$6</f>
         <v>156.324</v>
       </c>
@@ -2463,22 +2456,22 @@
       <c r="D13" s="8" t="n">
         <v>113</v>
       </c>
-      <c r="E13" s="130" t="n">
+      <c r="E13" s="131" t="n">
         <v>1.134046875</v>
       </c>
-      <c r="F13" s="131">
+      <c r="F13" s="132">
         <f>IF(AND(ISNUMBER(E13),ISNUMBER($D$8)),E13*$D$3,NA())</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="G13" s="132">
+      <c r="G13" s="133">
         <f>F13/$D$8</f>
         <v>145.158</v>
       </c>
-      <c r="H13" s="133">
+      <c r="H13" s="134">
         <f>G13*$D$4</f>
         <v>36.2895</v>
       </c>
-      <c r="I13" s="134">
+      <c r="I13" s="135">
         <f>G13-F13-H13</f>
         <v>50.805299999999995</v>
       </c>
@@ -2486,35 +2479,35 @@
         <f>I13/G13</f>
         <v>0.35</v>
       </c>
-      <c r="K13" s="135">
+      <c r="K13" s="136">
         <f>G13*$D$6</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="L13" s="136">
+      <c r="L13" s="137">
         <f>F13/(1-$D$4)</f>
         <v>77.4176</v>
       </c>
-      <c r="M13" s="136">
+      <c r="M13" s="137">
         <f>L13*$D$6</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="N13" s="137">
+      <c r="N13" s="138">
         <f>G13-F13</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="O13" s="138">
+      <c r="O13" s="139">
         <f>N13-H13</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="P13" s="139">
+      <c r="P13" s="140">
         <f>$F13/(1-$D$4-$P$9)</f>
         <v>129.0293333333333</v>
       </c>
-      <c r="Q13" s="140">
+      <c r="Q13" s="141">
         <f>P13*$D$4</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="R13" s="141">
+      <c r="R13" s="142">
         <f>P13-$F13-Q13</f>
         <v>38.70879999999999</v>
       </c>
@@ -2522,19 +2515,19 @@
         <f>R13/P13</f>
         <v>0.3</v>
       </c>
-      <c r="T13" s="139">
+      <c r="T13" s="140">
         <f>P13*$D$6</f>
         <v>180.64106666666663</v>
       </c>
-      <c r="U13" s="139">
+      <c r="U13" s="140">
         <f>$F13/(1-$D$4-$U$9)</f>
         <v>116.12639999999999</v>
       </c>
-      <c r="V13" s="140">
+      <c r="V13" s="141">
         <f>U13*$D$4</f>
         <v>29.031599999999997</v>
       </c>
-      <c r="W13" s="141">
+      <c r="W13" s="142">
         <f>U13-$F13-V13</f>
         <v>29.031599999999997</v>
       </c>
@@ -2542,19 +2535,19 @@
         <f>W13/U13</f>
         <v>0.25</v>
       </c>
-      <c r="Y13" s="139">
+      <c r="Y13" s="140">
         <f>U13*$D$6</f>
         <v>162.57695999999999</v>
       </c>
-      <c r="Z13" s="139">
+      <c r="Z13" s="140">
         <f>$F13/(1-$D$4-$Z$9)</f>
         <v>105.56945454545453</v>
       </c>
-      <c r="AA13" s="140">
+      <c r="AA13" s="141">
         <f>Z13*$D$4</f>
         <v>26.392363636363633</v>
       </c>
-      <c r="AB13" s="141">
+      <c r="AB13" s="142">
         <f>Z13-$F13-AA13</f>
         <v>21.113890909090905</v>
       </c>
@@ -2562,19 +2555,19 @@
         <f>AB13/Z13</f>
         <v>0.19999999999999998</v>
       </c>
-      <c r="AD13" s="139">
+      <c r="AD13" s="140">
         <f>Z13*$D$6</f>
         <v>147.79723636363633</v>
       </c>
-      <c r="AE13" s="139">
+      <c r="AE13" s="140">
         <f>$F13/(1-$D$4-$AE$9)</f>
         <v>96.77199999999999</v>
       </c>
-      <c r="AF13" s="140">
+      <c r="AF13" s="141">
         <f>AE13*$D$4</f>
         <v>24.192999999999998</v>
       </c>
-      <c r="AG13" s="141">
+      <c r="AG13" s="142">
         <f>AE13-$F13-AF13</f>
         <v>14.515799999999999</v>
       </c>
@@ -2582,7 +2575,7 @@
         <f>AG13/AE13</f>
         <v>0.15</v>
       </c>
-      <c r="AI13" s="139">
+      <c r="AI13" s="140">
         <f>AE13*$D$6</f>
         <v>135.4808</v>
       </c>
@@ -2601,25 +2594,25 @@
           <t>Spicy Flavor 112.5 г</t>
         </is>
       </c>
-      <c r="D14" s="142" t="n">
+      <c r="D14" s="143" t="n">
         <v>112.5</v>
       </c>
-      <c r="E14" s="130" t="n">
+      <c r="E14" s="131" t="n">
         <v>1.134046875</v>
       </c>
-      <c r="F14" s="131">
+      <c r="F14" s="132">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($D$8)),E14*$D$3,NA())</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="G14" s="132">
+      <c r="G14" s="133">
         <f>F14/$D$8</f>
         <v>145.158</v>
       </c>
-      <c r="H14" s="133">
+      <c r="H14" s="134">
         <f>G14*$D$4</f>
         <v>36.2895</v>
       </c>
-      <c r="I14" s="134">
+      <c r="I14" s="135">
         <f>G14-F14-H14</f>
         <v>50.805299999999995</v>
       </c>
@@ -2627,35 +2620,35 @@
         <f>I14/G14</f>
         <v>0.35</v>
       </c>
-      <c r="K14" s="135">
+      <c r="K14" s="136">
         <f>G14*$D$6</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="L14" s="136">
+      <c r="L14" s="137">
         <f>F14/(1-$D$4)</f>
         <v>77.4176</v>
       </c>
-      <c r="M14" s="136">
+      <c r="M14" s="137">
         <f>L14*$D$6</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="N14" s="137">
+      <c r="N14" s="138">
         <f>G14-F14</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="O14" s="138">
+      <c r="O14" s="139">
         <f>N14-H14</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="P14" s="139">
+      <c r="P14" s="140">
         <f>$F14/(1-$D$4-$P$9)</f>
         <v>129.0293333333333</v>
       </c>
-      <c r="Q14" s="140">
+      <c r="Q14" s="141">
         <f>P14*$D$4</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="R14" s="141">
+      <c r="R14" s="142">
         <f>P14-$F14-Q14</f>
         <v>38.70879999999999</v>
       </c>
@@ -2663,19 +2656,19 @@
         <f>R14/P14</f>
         <v>0.3</v>
       </c>
-      <c r="T14" s="139">
+      <c r="T14" s="140">
         <f>P14*$D$6</f>
         <v>180.64106666666663</v>
       </c>
-      <c r="U14" s="139">
+      <c r="U14" s="140">
         <f>$F14/(1-$D$4-$U$9)</f>
         <v>116.12639999999999</v>
       </c>
-      <c r="V14" s="140">
+      <c r="V14" s="141">
         <f>U14*$D$4</f>
         <v>29.031599999999997</v>
       </c>
-      <c r="W14" s="141">
+      <c r="W14" s="142">
         <f>U14-$F14-V14</f>
         <v>29.031599999999997</v>
       </c>
@@ -2683,19 +2676,19 @@
         <f>W14/U14</f>
         <v>0.25</v>
       </c>
-      <c r="Y14" s="139">
+      <c r="Y14" s="140">
         <f>U14*$D$6</f>
         <v>162.57695999999999</v>
       </c>
-      <c r="Z14" s="139">
+      <c r="Z14" s="140">
         <f>$F14/(1-$D$4-$Z$9)</f>
         <v>105.56945454545453</v>
       </c>
-      <c r="AA14" s="140">
+      <c r="AA14" s="141">
         <f>Z14*$D$4</f>
         <v>26.392363636363633</v>
       </c>
-      <c r="AB14" s="141">
+      <c r="AB14" s="142">
         <f>Z14-$F14-AA14</f>
         <v>21.113890909090905</v>
       </c>
@@ -2703,19 +2696,19 @@
         <f>AB14/Z14</f>
         <v>0.19999999999999998</v>
       </c>
-      <c r="AD14" s="139">
+      <c r="AD14" s="140">
         <f>Z14*$D$6</f>
         <v>147.79723636363633</v>
       </c>
-      <c r="AE14" s="139">
+      <c r="AE14" s="140">
         <f>$F14/(1-$D$4-$AE$9)</f>
         <v>96.77199999999999</v>
       </c>
-      <c r="AF14" s="140">
+      <c r="AF14" s="141">
         <f>AE14*$D$4</f>
         <v>24.192999999999998</v>
       </c>
-      <c r="AG14" s="141">
+      <c r="AG14" s="142">
         <f>AE14-$F14-AF14</f>
         <v>14.515799999999999</v>
       </c>
@@ -2723,7 +2716,7 @@
         <f>AG14/AE14</f>
         <v>0.15</v>
       </c>
-      <c r="AI14" s="139">
+      <c r="AI14" s="140">
         <f>AE14*$D$6</f>
         <v>135.4808</v>
       </c>
@@ -2745,22 +2738,22 @@
       <c r="D15" s="8" t="n">
         <v>113</v>
       </c>
-      <c r="E15" s="130" t="n">
+      <c r="E15" s="131" t="n">
         <v>1.134046875</v>
       </c>
-      <c r="F15" s="131">
+      <c r="F15" s="132">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($D$8)),E15*$D$3,NA())</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="G15" s="132">
+      <c r="G15" s="133">
         <f>F15/$D$8</f>
         <v>145.158</v>
       </c>
-      <c r="H15" s="133">
+      <c r="H15" s="134">
         <f>G15*$D$4</f>
         <v>36.2895</v>
       </c>
-      <c r="I15" s="134">
+      <c r="I15" s="135">
         <f>G15-F15-H15</f>
         <v>50.805299999999995</v>
       </c>
@@ -2768,35 +2761,35 @@
         <f>I15/G15</f>
         <v>0.35</v>
       </c>
-      <c r="K15" s="135">
+      <c r="K15" s="136">
         <f>G15*$D$6</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="L15" s="136">
+      <c r="L15" s="137">
         <f>F15/(1-$D$4)</f>
         <v>77.4176</v>
       </c>
-      <c r="M15" s="136">
+      <c r="M15" s="137">
         <f>L15*$D$6</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="N15" s="137">
+      <c r="N15" s="138">
         <f>G15-F15</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="O15" s="138">
+      <c r="O15" s="139">
         <f>N15-H15</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="P15" s="139">
+      <c r="P15" s="140">
         <f>$F15/(1-$D$4-$P$9)</f>
         <v>129.0293333333333</v>
       </c>
-      <c r="Q15" s="140">
+      <c r="Q15" s="141">
         <f>P15*$D$4</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="R15" s="141">
+      <c r="R15" s="142">
         <f>P15-$F15-Q15</f>
         <v>38.70879999999999</v>
       </c>
@@ -2804,19 +2797,19 @@
         <f>R15/P15</f>
         <v>0.3</v>
       </c>
-      <c r="T15" s="139">
+      <c r="T15" s="140">
         <f>P15*$D$6</f>
         <v>180.64106666666663</v>
       </c>
-      <c r="U15" s="139">
+      <c r="U15" s="140">
         <f>$F15/(1-$D$4-$U$9)</f>
         <v>116.12639999999999</v>
       </c>
-      <c r="V15" s="140">
+      <c r="V15" s="141">
         <f>U15*$D$4</f>
         <v>29.031599999999997</v>
       </c>
-      <c r="W15" s="141">
+      <c r="W15" s="142">
         <f>U15-$F15-V15</f>
         <v>29.031599999999997</v>
       </c>
@@ -2824,19 +2817,19 @@
         <f>W15/U15</f>
         <v>0.25</v>
       </c>
-      <c r="Y15" s="139">
+      <c r="Y15" s="140">
         <f>U15*$D$6</f>
         <v>162.57695999999999</v>
       </c>
-      <c r="Z15" s="139">
+      <c r="Z15" s="140">
         <f>$F15/(1-$D$4-$Z$9)</f>
         <v>105.56945454545453</v>
       </c>
-      <c r="AA15" s="140">
+      <c r="AA15" s="141">
         <f>Z15*$D$4</f>
         <v>26.392363636363633</v>
       </c>
-      <c r="AB15" s="141">
+      <c r="AB15" s="142">
         <f>Z15-$F15-AA15</f>
         <v>21.113890909090905</v>
       </c>
@@ -2844,19 +2837,19 @@
         <f>AB15/Z15</f>
         <v>0.19999999999999998</v>
       </c>
-      <c r="AD15" s="139">
+      <c r="AD15" s="140">
         <f>Z15*$D$6</f>
         <v>147.79723636363633</v>
       </c>
-      <c r="AE15" s="139">
+      <c r="AE15" s="140">
         <f>$F15/(1-$D$4-$AE$9)</f>
         <v>96.77199999999999</v>
       </c>
-      <c r="AF15" s="140">
+      <c r="AF15" s="141">
         <f>AE15*$D$4</f>
         <v>24.192999999999998</v>
       </c>
-      <c r="AG15" s="141">
+      <c r="AG15" s="142">
         <f>AE15-$F15-AF15</f>
         <v>14.515799999999999</v>
       </c>
@@ -2864,7 +2857,7 @@
         <f>AG15/AE15</f>
         <v>0.15</v>
       </c>
-      <c r="AI15" s="139">
+      <c r="AI15" s="140">
         <f>AE15*$D$6</f>
         <v>135.4808</v>
       </c>
@@ -2886,22 +2879,22 @@
       <c r="D16" s="8" t="n">
         <v>113</v>
       </c>
-      <c r="E16" s="130" t="n">
+      <c r="E16" s="131" t="n">
         <v>1.134046875</v>
       </c>
-      <c r="F16" s="131">
+      <c r="F16" s="132">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($D$8)),E16*$D$3,NA())</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="G16" s="132">
+      <c r="G16" s="133">
         <f>F16/$D$8</f>
         <v>145.158</v>
       </c>
-      <c r="H16" s="133">
+      <c r="H16" s="134">
         <f>G16*$D$4</f>
         <v>36.2895</v>
       </c>
-      <c r="I16" s="134">
+      <c r="I16" s="135">
         <f>G16-F16-H16</f>
         <v>50.805299999999995</v>
       </c>
@@ -2909,35 +2902,35 @@
         <f>I16/G16</f>
         <v>0.35</v>
       </c>
-      <c r="K16" s="135">
+      <c r="K16" s="136">
         <f>G16*$D$6</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="L16" s="136">
+      <c r="L16" s="137">
         <f>F16/(1-$D$4)</f>
         <v>77.4176</v>
       </c>
-      <c r="M16" s="136">
+      <c r="M16" s="137">
         <f>L16*$D$6</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="N16" s="137">
+      <c r="N16" s="138">
         <f>G16-F16</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="O16" s="138">
+      <c r="O16" s="139">
         <f>N16-H16</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="P16" s="139">
+      <c r="P16" s="140">
         <f>$F16/(1-$D$4-$P$9)</f>
         <v>129.0293333333333</v>
       </c>
-      <c r="Q16" s="140">
+      <c r="Q16" s="141">
         <f>P16*$D$4</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="R16" s="141">
+      <c r="R16" s="142">
         <f>P16-$F16-Q16</f>
         <v>38.70879999999999</v>
       </c>
@@ -2945,19 +2938,19 @@
         <f>R16/P16</f>
         <v>0.3</v>
       </c>
-      <c r="T16" s="139">
+      <c r="T16" s="140">
         <f>P16*$D$6</f>
         <v>180.64106666666663</v>
       </c>
-      <c r="U16" s="139">
+      <c r="U16" s="140">
         <f>$F16/(1-$D$4-$U$9)</f>
         <v>116.12639999999999</v>
       </c>
-      <c r="V16" s="140">
+      <c r="V16" s="141">
         <f>U16*$D$4</f>
         <v>29.031599999999997</v>
       </c>
-      <c r="W16" s="141">
+      <c r="W16" s="142">
         <f>U16-$F16-V16</f>
         <v>29.031599999999997</v>
       </c>
@@ -2965,19 +2958,19 @@
         <f>W16/U16</f>
         <v>0.25</v>
       </c>
-      <c r="Y16" s="139">
+      <c r="Y16" s="140">
         <f>U16*$D$6</f>
         <v>162.57695999999999</v>
       </c>
-      <c r="Z16" s="139">
+      <c r="Z16" s="140">
         <f>$F16/(1-$D$4-$Z$9)</f>
         <v>105.56945454545453</v>
       </c>
-      <c r="AA16" s="140">
+      <c r="AA16" s="141">
         <f>Z16*$D$4</f>
         <v>26.392363636363633</v>
       </c>
-      <c r="AB16" s="141">
+      <c r="AB16" s="142">
         <f>Z16-$F16-AA16</f>
         <v>21.113890909090905</v>
       </c>
@@ -2985,19 +2978,19 @@
         <f>AB16/Z16</f>
         <v>0.19999999999999998</v>
       </c>
-      <c r="AD16" s="139">
+      <c r="AD16" s="140">
         <f>Z16*$D$6</f>
         <v>147.79723636363633</v>
       </c>
-      <c r="AE16" s="139">
+      <c r="AE16" s="140">
         <f>$F16/(1-$D$4-$AE$9)</f>
         <v>96.77199999999999</v>
       </c>
-      <c r="AF16" s="140">
+      <c r="AF16" s="141">
         <f>AE16*$D$4</f>
         <v>24.192999999999998</v>
       </c>
-      <c r="AG16" s="141">
+      <c r="AG16" s="142">
         <f>AE16-$F16-AF16</f>
         <v>14.515799999999999</v>
       </c>
@@ -3005,14 +2998,14 @@
         <f>AG16/AE16</f>
         <v>0.15</v>
       </c>
-      <c r="AI16" s="139">
+      <c r="AI16" s="140">
         <f>AE16*$D$6</f>
         <v>135.4808</v>
       </c>
     </row>
     <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="27" t="n"/>
-      <c r="B19" s="143" t="inlineStr">
+      <c r="B19" s="144" t="inlineStr">
         <is>
           <t>Кожен крок формування ціни — за вашим прикладом</t>
         </is>
@@ -3037,12 +3030,12 @@
           <t>№</t>
         </is>
       </c>
-      <c r="B21" s="144" t="inlineStr">
+      <c r="B21" s="145" t="inlineStr">
         <is>
           <t>Що рахуємо</t>
         </is>
       </c>
-      <c r="D21" s="144" t="inlineStr">
+      <c r="D21" s="145" t="inlineStr">
         <is>
           <t>Дія</t>
         </is>
@@ -3081,34 +3074,34 @@
           <t>Собівартість в Україні, EUR/уп.</t>
         </is>
       </c>
-      <c r="C22" s="145" t="n"/>
+      <c r="C22" s="146" t="n"/>
       <c r="D22" s="86" t="inlineStr">
         <is>
           <t>Із Self-Cost</t>
         </is>
       </c>
-      <c r="E22" s="145" t="n"/>
-      <c r="F22" s="146">
+      <c r="E22" s="146" t="n"/>
+      <c r="F22" s="147">
         <f>E11</f>
         <v>1.308515625</v>
       </c>
-      <c r="G22" s="146">
+      <c r="G22" s="147">
         <f>E12</f>
         <v>1.308515625</v>
       </c>
-      <c r="H22" s="146">
+      <c r="H22" s="147">
         <f>E13</f>
         <v>1.134046875</v>
       </c>
-      <c r="I22" s="146">
+      <c r="I22" s="147">
         <f>E14</f>
         <v>1.134046875</v>
       </c>
-      <c r="J22" s="146">
+      <c r="J22" s="147">
         <f>E15</f>
         <v>1.134046875</v>
       </c>
-      <c r="K22" s="146">
+      <c r="K22" s="147">
         <f>E16</f>
         <v>1.134046875</v>
       </c>
@@ -3122,13 +3115,13 @@
           <t>Курс, грн/EUR</t>
         </is>
       </c>
-      <c r="C23" s="145" t="n"/>
+      <c r="C23" s="146" t="n"/>
       <c r="D23" s="86" t="inlineStr">
         <is>
           <t>Умова в D3</t>
         </is>
       </c>
-      <c r="E23" s="145" t="n"/>
+      <c r="E23" s="146" t="n"/>
       <c r="F23" s="31">
         <f>$D$3</f>
         <v>51.2</v>
@@ -3163,34 +3156,34 @@
           <t>Собівартість в Україні, грн/уп.</t>
         </is>
       </c>
-      <c r="C24" s="145" t="n"/>
+      <c r="C24" s="146" t="n"/>
       <c r="D24" s="86" t="inlineStr">
         <is>
           <t>Крок 1 × крок 2</t>
         </is>
       </c>
-      <c r="E24" s="145" t="n"/>
-      <c r="F24" s="147">
+      <c r="E24" s="146" t="n"/>
+      <c r="F24" s="148">
         <f>F11</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="G24" s="147">
+      <c r="G24" s="148">
         <f>F12</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="H24" s="147">
+      <c r="H24" s="148">
         <f>F13</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="I24" s="147">
+      <c r="I24" s="148">
         <f>F14</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="J24" s="147">
+      <c r="J24" s="148">
         <f>F15</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="K24" s="147">
+      <c r="K24" s="148">
         <f>F16</f>
         <v>58.063199999999995</v>
       </c>
@@ -3204,13 +3197,13 @@
           <t>Повна ціна партнеру, %</t>
         </is>
       </c>
-      <c r="C25" s="145" t="n"/>
+      <c r="C25" s="146" t="n"/>
       <c r="D25" s="86" t="inlineStr">
         <is>
           <t>База для всіх відсотків</t>
         </is>
       </c>
-      <c r="E25" s="145" t="n"/>
+      <c r="E25" s="146" t="n"/>
       <c r="F25" s="33" t="n">
         <v>1</v>
       </c>
@@ -3239,13 +3232,13 @@
           <t>Бонус мережі, %</t>
         </is>
       </c>
-      <c r="C26" s="145" t="n"/>
+      <c r="C26" s="146" t="n"/>
       <c r="D26" s="86" t="inlineStr">
         <is>
           <t>Умова в D4</t>
         </is>
       </c>
-      <c r="E26" s="145" t="n"/>
+      <c r="E26" s="146" t="n"/>
       <c r="F26" s="33">
         <f>$D$4</f>
         <v>0.25</v>
@@ -3280,13 +3273,13 @@
           <t>Частка ціни після бонусу, %</t>
         </is>
       </c>
-      <c r="C27" s="145" t="n"/>
+      <c r="C27" s="146" t="n"/>
       <c r="D27" s="86" t="inlineStr">
         <is>
           <t>Крок 4 − крок 5</t>
         </is>
       </c>
-      <c r="E27" s="145" t="n"/>
+      <c r="E27" s="146" t="n"/>
       <c r="F27" s="33">
         <f>1-$D$4</f>
         <v>0.75</v>
@@ -3321,13 +3314,13 @@
           <t>Наша цільова маржа, %</t>
         </is>
       </c>
-      <c r="C28" s="145" t="n"/>
+      <c r="C28" s="146" t="n"/>
       <c r="D28" s="86" t="inlineStr">
         <is>
           <t>Умова в D5</t>
         </is>
       </c>
-      <c r="E28" s="145" t="n"/>
+      <c r="E28" s="146" t="n"/>
       <c r="F28" s="33">
         <f>$D$5</f>
         <v>0.35</v>
@@ -3362,13 +3355,13 @@
           <t>Частка ціни для собівартості, %</t>
         </is>
       </c>
-      <c r="C29" s="145" t="n"/>
+      <c r="C29" s="146" t="n"/>
       <c r="D29" s="86" t="inlineStr">
         <is>
           <t>Крок 6 − крок 7</t>
         </is>
       </c>
-      <c r="E29" s="145" t="n"/>
+      <c r="E29" s="146" t="n"/>
       <c r="F29" s="33">
         <f>$D$8</f>
         <v>0.4</v>
@@ -3403,34 +3396,34 @@
           <t>Ціна партнеру з ПДВ, грн/уп.</t>
         </is>
       </c>
-      <c r="C30" s="145" t="n"/>
+      <c r="C30" s="146" t="n"/>
       <c r="D30" s="90" t="inlineStr">
         <is>
           <t>Крок 3 ÷ крок 8</t>
         </is>
       </c>
-      <c r="E30" s="145" t="n"/>
-      <c r="F30" s="148">
+      <c r="E30" s="146" t="n"/>
+      <c r="F30" s="149">
         <f>G11</f>
         <v>167.49</v>
       </c>
-      <c r="G30" s="148">
+      <c r="G30" s="149">
         <f>G12</f>
         <v>167.49</v>
       </c>
-      <c r="H30" s="148">
+      <c r="H30" s="149">
         <f>G13</f>
         <v>145.158</v>
       </c>
-      <c r="I30" s="148">
+      <c r="I30" s="149">
         <f>G14</f>
         <v>145.158</v>
       </c>
-      <c r="J30" s="148">
+      <c r="J30" s="149">
         <f>G15</f>
         <v>145.158</v>
       </c>
-      <c r="K30" s="148">
+      <c r="K30" s="149">
         <f>G16</f>
         <v>145.158</v>
       </c>
@@ -3444,34 +3437,34 @@
           <t>Валовий прибуток до бонусу, грн/уп.</t>
         </is>
       </c>
-      <c r="C31" s="145" t="n"/>
+      <c r="C31" s="146" t="n"/>
       <c r="D31" s="86" t="inlineStr">
         <is>
           <t>Крок 9 − крок 3</t>
         </is>
       </c>
-      <c r="E31" s="145" t="n"/>
-      <c r="F31" s="147">
+      <c r="E31" s="146" t="n"/>
+      <c r="F31" s="148">
         <f>N11</f>
         <v>100.494</v>
       </c>
-      <c r="G31" s="147">
+      <c r="G31" s="148">
         <f>N12</f>
         <v>100.494</v>
       </c>
-      <c r="H31" s="147">
+      <c r="H31" s="148">
         <f>N13</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="I31" s="147">
+      <c r="I31" s="148">
         <f>N14</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="J31" s="147">
+      <c r="J31" s="148">
         <f>N15</f>
         <v>87.09479999999999</v>
       </c>
-      <c r="K31" s="147">
+      <c r="K31" s="148">
         <f>N16</f>
         <v>87.09479999999999</v>
       </c>
@@ -3485,34 +3478,34 @@
           <t>Бонус мережі, грн/уп.</t>
         </is>
       </c>
-      <c r="C32" s="145" t="n"/>
+      <c r="C32" s="146" t="n"/>
       <c r="D32" s="86" t="inlineStr">
         <is>
           <t>Крок 9 × крок 5</t>
         </is>
       </c>
-      <c r="E32" s="145" t="n"/>
-      <c r="F32" s="147">
+      <c r="E32" s="146" t="n"/>
+      <c r="F32" s="148">
         <f>H11</f>
         <v>41.8725</v>
       </c>
-      <c r="G32" s="147">
+      <c r="G32" s="148">
         <f>H12</f>
         <v>41.8725</v>
       </c>
-      <c r="H32" s="147">
+      <c r="H32" s="148">
         <f>H13</f>
         <v>36.2895</v>
       </c>
-      <c r="I32" s="147">
+      <c r="I32" s="148">
         <f>H14</f>
         <v>36.2895</v>
       </c>
-      <c r="J32" s="147">
+      <c r="J32" s="148">
         <f>H15</f>
         <v>36.2895</v>
       </c>
-      <c r="K32" s="147">
+      <c r="K32" s="148">
         <f>H16</f>
         <v>36.2895</v>
       </c>
@@ -3526,34 +3519,34 @@
           <t>Нам залишається після собівартості та бонусу, грн/уп.</t>
         </is>
       </c>
-      <c r="C33" s="145" t="n"/>
+      <c r="C33" s="146" t="n"/>
       <c r="D33" s="92" t="inlineStr">
         <is>
           <t>Крок 10 − крок 11</t>
         </is>
       </c>
-      <c r="E33" s="145" t="n"/>
-      <c r="F33" s="149">
+      <c r="E33" s="146" t="n"/>
+      <c r="F33" s="150">
         <f>I11</f>
         <v>58.6215</v>
       </c>
-      <c r="G33" s="149">
+      <c r="G33" s="150">
         <f>I12</f>
         <v>58.6215</v>
       </c>
-      <c r="H33" s="149">
+      <c r="H33" s="150">
         <f>I13</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="I33" s="149">
+      <c r="I33" s="150">
         <f>I14</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="J33" s="149">
+      <c r="J33" s="150">
         <f>I15</f>
         <v>50.805299999999995</v>
       </c>
-      <c r="K33" s="149">
+      <c r="K33" s="150">
         <f>I16</f>
         <v>50.805299999999995</v>
       </c>
@@ -3567,13 +3560,13 @@
           <t>Перевірка нашої маржі після бонусу, %</t>
         </is>
       </c>
-      <c r="C34" s="145" t="n"/>
+      <c r="C34" s="146" t="n"/>
       <c r="D34" s="92" t="inlineStr">
         <is>
           <t>Крок 12 ÷ крок 9</t>
         </is>
       </c>
-      <c r="E34" s="145" t="n"/>
+      <c r="E34" s="146" t="n"/>
       <c r="F34" s="38">
         <f>J11</f>
         <v>0.35</v>
@@ -3608,13 +3601,13 @@
           <t>Націнка ритейлера для полиці, %</t>
         </is>
       </c>
-      <c r="C35" s="145" t="n"/>
+      <c r="C35" s="146" t="n"/>
       <c r="D35" s="86" t="inlineStr">
         <is>
           <t>Множник D6 − 1</t>
         </is>
       </c>
-      <c r="E35" s="145" t="n"/>
+      <c r="E35" s="146" t="n"/>
       <c r="F35" s="33">
         <f>$D$6-1</f>
         <v>0.3999999999999999</v>
@@ -3649,34 +3642,34 @@
           <t>Множник ритейлера</t>
         </is>
       </c>
-      <c r="C36" s="145" t="n"/>
+      <c r="C36" s="146" t="n"/>
       <c r="D36" s="86" t="inlineStr">
         <is>
           <t>1 + крок 14</t>
         </is>
       </c>
-      <c r="E36" s="145" t="n"/>
-      <c r="F36" s="150">
+      <c r="E36" s="146" t="n"/>
+      <c r="F36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="G36" s="150">
+      <c r="G36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="H36" s="150">
+      <c r="H36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="I36" s="150">
+      <c r="I36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="J36" s="150">
+      <c r="J36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="K36" s="150">
+      <c r="K36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
@@ -3690,34 +3683,34 @@
           <t>Ціна на полиці з ПДВ, грн/уп.</t>
         </is>
       </c>
-      <c r="C37" s="145" t="n"/>
+      <c r="C37" s="146" t="n"/>
       <c r="D37" s="90" t="inlineStr">
         <is>
           <t>Крок 9 × крок 15</t>
         </is>
       </c>
-      <c r="E37" s="145" t="n"/>
-      <c r="F37" s="148">
+      <c r="E37" s="146" t="n"/>
+      <c r="F37" s="149">
         <f>K11</f>
         <v>234.486</v>
       </c>
-      <c r="G37" s="148">
+      <c r="G37" s="149">
         <f>K12</f>
         <v>234.486</v>
       </c>
-      <c r="H37" s="148">
+      <c r="H37" s="149">
         <f>K13</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="I37" s="148">
+      <c r="I37" s="149">
         <f>K14</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="J37" s="148">
+      <c r="J37" s="149">
         <f>K15</f>
         <v>203.22119999999998</v>
       </c>
-      <c r="K37" s="148">
+      <c r="K37" s="149">
         <f>K16</f>
         <v>203.22119999999998</v>
       </c>
@@ -3731,34 +3724,34 @@
           <t>Ціна партнеру при нульовому нашому прибутку, грн/уп.</t>
         </is>
       </c>
-      <c r="C38" s="145" t="n"/>
+      <c r="C38" s="146" t="n"/>
       <c r="D38" s="86" t="inlineStr">
         <is>
           <t>Крок 3 ÷ крок 6</t>
         </is>
       </c>
-      <c r="E38" s="145" t="n"/>
-      <c r="F38" s="147">
+      <c r="E38" s="146" t="n"/>
+      <c r="F38" s="148">
         <f>L11</f>
         <v>89.32800000000002</v>
       </c>
-      <c r="G38" s="147">
+      <c r="G38" s="148">
         <f>L12</f>
         <v>89.32800000000002</v>
       </c>
-      <c r="H38" s="147">
+      <c r="H38" s="148">
         <f>L13</f>
         <v>77.4176</v>
       </c>
-      <c r="I38" s="147">
+      <c r="I38" s="148">
         <f>L14</f>
         <v>77.4176</v>
       </c>
-      <c r="J38" s="147">
+      <c r="J38" s="148">
         <f>L15</f>
         <v>77.4176</v>
       </c>
-      <c r="K38" s="147">
+      <c r="K38" s="148">
         <f>L16</f>
         <v>77.4176</v>
       </c>
@@ -3772,44 +3765,42 @@
           <t>Полиця при нульовому нашому прибутку, грн/уп.</t>
         </is>
       </c>
-      <c r="C39" s="145" t="n"/>
+      <c r="C39" s="146" t="n"/>
       <c r="D39" s="86" t="inlineStr">
         <is>
           <t>Крок 17 × крок 15</t>
         </is>
       </c>
-      <c r="E39" s="145" t="n"/>
-      <c r="F39" s="147">
+      <c r="E39" s="146" t="n"/>
+      <c r="F39" s="148">
         <f>M11</f>
         <v>125.05920000000002</v>
       </c>
-      <c r="G39" s="147">
+      <c r="G39" s="148">
         <f>M12</f>
         <v>125.05920000000002</v>
       </c>
-      <c r="H39" s="147">
+      <c r="H39" s="148">
         <f>M13</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="I39" s="147">
+      <c r="I39" s="148">
         <f>M14</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="J39" s="147">
+      <c r="J39" s="148">
         <f>M15</f>
         <v>108.38463999999999</v>
       </c>
-      <c r="K39" s="147">
+      <c r="K39" s="148">
         <f>M16</f>
         <v>108.38463999999999</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="73">
-    <mergeCell ref="L2:M2"/>
+  <mergeCells count="63">
     <mergeCell ref="U9:Y9"/>
     <mergeCell ref="Z9:AD9"/>
-    <mergeCell ref="L7:M7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
@@ -3824,28 +3815,22 @@
     <mergeCell ref="P9:T9"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="B39:C39"/>
-    <mergeCell ref="L3:M3"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="G9:J9"/>
-    <mergeCell ref="N3:O3"/>
     <mergeCell ref="D35:E35"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="D27:E27"/>
-    <mergeCell ref="N2:O2"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="D32:E32"/>
-    <mergeCell ref="L5:M5"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="N5:O5"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="E5:K5"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="L4:M4"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
@@ -3864,7 +3849,6 @@
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L6:M6"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D29:E29"/>
@@ -3878,7 +3862,6 @@
     <mergeCell ref="B19:K19"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="N4:O4"/>
   </mergeCells>
   <conditionalFormatting sqref="E33:K36">
     <cfRule type="expression" priority="2" dxfId="4">
@@ -3954,10 +3937,8 @@
       <c r="I2" s="123" t="n"/>
       <c r="J2" s="123" t="n"/>
       <c r="K2" s="122" t="n"/>
-      <c r="L2" s="7" t="n"/>
-      <c r="M2" s="121" t="n"/>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="121" t="n"/>
+      <c r="L2" s="124" t="n"/>
+      <c r="N2" s="124" t="n"/>
     </row>
     <row r="3" ht="37.5" customHeight="1">
       <c r="B3" s="1" t="inlineStr">
@@ -3980,10 +3961,8 @@
       <c r="I3" s="120" t="n"/>
       <c r="J3" s="120" t="n"/>
       <c r="K3" s="121" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="121" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="121" t="n"/>
+      <c r="L3" s="124" t="n"/>
+      <c r="N3" s="124" t="n"/>
     </row>
     <row r="4" ht="37.5" customHeight="1">
       <c r="B4" s="1" t="inlineStr">
@@ -4006,10 +3985,8 @@
       <c r="I4" s="120" t="n"/>
       <c r="J4" s="120" t="n"/>
       <c r="K4" s="121" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="121" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="121" t="n"/>
+      <c r="L4" s="124" t="n"/>
+      <c r="N4" s="124" t="n"/>
     </row>
     <row r="5" ht="61.5" customHeight="1">
       <c r="B5" s="1" t="inlineStr">
@@ -4032,10 +4009,8 @@
       <c r="I5" s="120" t="n"/>
       <c r="J5" s="120" t="n"/>
       <c r="K5" s="121" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="121" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="121" t="n"/>
+      <c r="L5" s="124" t="n"/>
+      <c r="N5" s="124" t="n"/>
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="B6" s="1" t="inlineStr">
@@ -4058,8 +4033,7 @@
       <c r="I6" s="120" t="n"/>
       <c r="J6" s="120" t="n"/>
       <c r="K6" s="121" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="121" t="n"/>
+      <c r="L6" s="124" t="n"/>
     </row>
     <row r="7" ht="27.75" customHeight="1">
       <c r="B7" s="1" t="inlineStr">
@@ -4084,8 +4058,7 @@
       <c r="I7" s="120" t="n"/>
       <c r="J7" s="120" t="n"/>
       <c r="K7" s="121" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="121" t="n"/>
+      <c r="L7" s="124" t="n"/>
     </row>
     <row r="8" ht="30" customFormat="1" customHeight="1" s="21">
       <c r="B8" s="80" t="inlineStr">
@@ -4093,12 +4066,12 @@
           <t>Частка ціни для собівартості</t>
         </is>
       </c>
-      <c r="C8" s="124" t="n"/>
+      <c r="C8" s="125" t="n"/>
       <c r="D8" s="24">
         <f>IF(AND(COUNT(D3:D6)=4,D3&gt;0,D4&gt;=0,D5&gt;=0,D4+D5&lt;1,D6&gt;0),1-D4-D5,NA())</f>
         <v>0.4</v>
       </c>
-      <c r="E8" s="125" t="inlineStr">
+      <c r="E8" s="126" t="inlineStr">
         <is>
           <t>100% − бонус − маржа. За поточних умов: 100% − 25% − 35% = 40%.</t>
         </is>
@@ -4150,34 +4123,34 @@
         </is>
       </c>
       <c r="O9" s="121" t="n"/>
-      <c r="P9" s="126" t="n">
+      <c r="P9" s="127" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q9" s="127" t="n"/>
-      <c r="R9" s="127" t="n"/>
-      <c r="S9" s="127" t="n"/>
-      <c r="T9" s="128" t="n"/>
-      <c r="U9" s="129" t="n">
+      <c r="Q9" s="128" t="n"/>
+      <c r="R9" s="128" t="n"/>
+      <c r="S9" s="128" t="n"/>
+      <c r="T9" s="129" t="n"/>
+      <c r="U9" s="130" t="n">
         <v>0.25</v>
       </c>
-      <c r="V9" s="127" t="n"/>
-      <c r="W9" s="127" t="n"/>
-      <c r="X9" s="127" t="n"/>
-      <c r="Y9" s="128" t="n"/>
-      <c r="Z9" s="126" t="n">
+      <c r="V9" s="128" t="n"/>
+      <c r="W9" s="128" t="n"/>
+      <c r="X9" s="128" t="n"/>
+      <c r="Y9" s="129" t="n"/>
+      <c r="Z9" s="127" t="n">
         <v>0.2</v>
       </c>
-      <c r="AA9" s="127" t="n"/>
-      <c r="AB9" s="127" t="n"/>
-      <c r="AC9" s="127" t="n"/>
-      <c r="AD9" s="128" t="n"/>
-      <c r="AE9" s="129" t="n">
+      <c r="AA9" s="128" t="n"/>
+      <c r="AB9" s="128" t="n"/>
+      <c r="AC9" s="128" t="n"/>
+      <c r="AD9" s="129" t="n"/>
+      <c r="AE9" s="130" t="n">
         <v>0.15</v>
       </c>
-      <c r="AF9" s="127" t="n"/>
-      <c r="AG9" s="127" t="n"/>
-      <c r="AH9" s="127" t="n"/>
-      <c r="AI9" s="128" t="n"/>
+      <c r="AF9" s="128" t="n"/>
+      <c r="AG9" s="128" t="n"/>
+      <c r="AH9" s="128" t="n"/>
+      <c r="AI9" s="129" t="n"/>
     </row>
     <row r="10" ht="41.4" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -4373,22 +4346,22 @@
       <c r="D11" s="8" t="n">
         <v>123</v>
       </c>
-      <c r="E11" s="130" t="n">
+      <c r="E11" s="131" t="n">
         <v>1.018131154266958</v>
       </c>
-      <c r="F11" s="131">
+      <c r="F11" s="132">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($D$8)),E11*$D$3,NA())</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="G11" s="132">
+      <c r="G11" s="133">
         <f>F11/$D$8</f>
         <v>130.32078774617062</v>
       </c>
-      <c r="H11" s="133">
+      <c r="H11" s="134">
         <f>G11*$D$4</f>
         <v>32.580196936542656</v>
       </c>
-      <c r="I11" s="134">
+      <c r="I11" s="135">
         <f>G11-F11-H11</f>
         <v>45.61227571115972</v>
       </c>
@@ -4396,35 +4369,35 @@
         <f>I11/G11</f>
         <v>0.35</v>
       </c>
-      <c r="K11" s="135">
+      <c r="K11" s="136">
         <f>G11*$D$6</f>
         <v>182.44910284463887</v>
       </c>
-      <c r="L11" s="136">
+      <c r="L11" s="137">
         <f>F11/(1-$D$4)</f>
         <v>69.504420131291</v>
       </c>
-      <c r="M11" s="136">
+      <c r="M11" s="137">
         <f>L11*$D$6</f>
         <v>97.3061881838074</v>
       </c>
-      <c r="N11" s="137">
+      <c r="N11" s="138">
         <f>G11-F11</f>
         <v>78.19247264770237</v>
       </c>
-      <c r="O11" s="138">
+      <c r="O11" s="139">
         <f>N11-H11</f>
         <v>45.61227571115972</v>
       </c>
-      <c r="P11" s="139">
+      <c r="P11" s="140">
         <f>$F11/(1-$D$4-$P$9)</f>
         <v>115.84070021881833</v>
       </c>
-      <c r="Q11" s="140">
+      <c r="Q11" s="141">
         <f>P11*$D$4</f>
         <v>28.96017505470458</v>
       </c>
-      <c r="R11" s="141">
+      <c r="R11" s="142">
         <f>P11-$F11-Q11</f>
         <v>34.7522100656455</v>
       </c>
@@ -4432,19 +4405,19 @@
         <f>R11/P11</f>
         <v>0.3</v>
       </c>
-      <c r="T11" s="139">
+      <c r="T11" s="140">
         <f>P11*$D$6</f>
         <v>162.17698030634565</v>
       </c>
-      <c r="U11" s="139">
+      <c r="U11" s="140">
         <f>$F11/(1-$D$4-$U$9)</f>
         <v>104.2566301969365</v>
       </c>
-      <c r="V11" s="140">
+      <c r="V11" s="141">
         <f>U11*$D$4</f>
         <v>26.064157549234125</v>
       </c>
-      <c r="W11" s="141">
+      <c r="W11" s="142">
         <f>U11-$F11-V11</f>
         <v>26.064157549234125</v>
       </c>
@@ -4452,19 +4425,19 @@
         <f>W11/U11</f>
         <v>0.25</v>
       </c>
-      <c r="Y11" s="139">
+      <c r="Y11" s="140">
         <f>U11*$D$6</f>
         <v>145.95928227571108</v>
       </c>
-      <c r="Z11" s="139">
+      <c r="Z11" s="140">
         <f>$F11/(1-$D$4-$Z$9)</f>
         <v>94.77875472448771</v>
       </c>
-      <c r="AA11" s="140">
+      <c r="AA11" s="141">
         <f>Z11*$D$4</f>
         <v>23.694688681121928</v>
       </c>
-      <c r="AB11" s="141">
+      <c r="AB11" s="142">
         <f>Z11-$F11-AA11</f>
         <v>18.955750944897535</v>
       </c>
@@ -4472,19 +4445,19 @@
         <f>AB11/Z11</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD11" s="139">
+      <c r="AD11" s="140">
         <f>Z11*$D$6</f>
         <v>132.6902566142828</v>
       </c>
-      <c r="AE11" s="139">
+      <c r="AE11" s="140">
         <f>$F11/(1-$D$4-$AE$9)</f>
         <v>86.88052516411375</v>
       </c>
-      <c r="AF11" s="140">
+      <c r="AF11" s="141">
         <f>AE11*$D$4</f>
         <v>21.720131291028437</v>
       </c>
-      <c r="AG11" s="141">
+      <c r="AG11" s="142">
         <f>AE11-$F11-AF11</f>
         <v>13.032078774617062</v>
       </c>
@@ -4492,7 +4465,7 @@
         <f>AG11/AE11</f>
         <v>0.15</v>
       </c>
-      <c r="AI11" s="139">
+      <c r="AI11" s="140">
         <f>AE11*$D$6</f>
         <v>121.63273522975923</v>
       </c>
@@ -4514,22 +4487,22 @@
       <c r="D12" s="8" t="n">
         <v>131</v>
       </c>
-      <c r="E12" s="130" t="n">
+      <c r="E12" s="131" t="n">
         <v>1.018131154266958</v>
       </c>
-      <c r="F12" s="131">
+      <c r="F12" s="132">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($D$8)),E12*$D$3,NA())</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="G12" s="132">
+      <c r="G12" s="133">
         <f>F12/$D$8</f>
         <v>130.32078774617062</v>
       </c>
-      <c r="H12" s="133">
+      <c r="H12" s="134">
         <f>G12*$D$4</f>
         <v>32.580196936542656</v>
       </c>
-      <c r="I12" s="134">
+      <c r="I12" s="135">
         <f>G12-F12-H12</f>
         <v>45.61227571115972</v>
       </c>
@@ -4537,35 +4510,35 @@
         <f>I12/G12</f>
         <v>0.35</v>
       </c>
-      <c r="K12" s="135">
+      <c r="K12" s="136">
         <f>G12*$D$6</f>
         <v>182.44910284463887</v>
       </c>
-      <c r="L12" s="136">
+      <c r="L12" s="137">
         <f>F12/(1-$D$4)</f>
         <v>69.504420131291</v>
       </c>
-      <c r="M12" s="136">
+      <c r="M12" s="137">
         <f>L12*$D$6</f>
         <v>97.3061881838074</v>
       </c>
-      <c r="N12" s="137">
+      <c r="N12" s="138">
         <f>G12-F12</f>
         <v>78.19247264770237</v>
       </c>
-      <c r="O12" s="138">
+      <c r="O12" s="139">
         <f>N12-H12</f>
         <v>45.61227571115972</v>
       </c>
-      <c r="P12" s="139">
+      <c r="P12" s="140">
         <f>$F12/(1-$D$4-$P$9)</f>
         <v>115.84070021881833</v>
       </c>
-      <c r="Q12" s="140">
+      <c r="Q12" s="141">
         <f>P12*$D$4</f>
         <v>28.96017505470458</v>
       </c>
-      <c r="R12" s="141">
+      <c r="R12" s="142">
         <f>P12-$F12-Q12</f>
         <v>34.7522100656455</v>
       </c>
@@ -4573,19 +4546,19 @@
         <f>R12/P12</f>
         <v>0.3</v>
       </c>
-      <c r="T12" s="139">
+      <c r="T12" s="140">
         <f>P12*$D$6</f>
         <v>162.17698030634565</v>
       </c>
-      <c r="U12" s="139">
+      <c r="U12" s="140">
         <f>$F12/(1-$D$4-$U$9)</f>
         <v>104.2566301969365</v>
       </c>
-      <c r="V12" s="140">
+      <c r="V12" s="141">
         <f>U12*$D$4</f>
         <v>26.064157549234125</v>
       </c>
-      <c r="W12" s="141">
+      <c r="W12" s="142">
         <f>U12-$F12-V12</f>
         <v>26.064157549234125</v>
       </c>
@@ -4593,19 +4566,19 @@
         <f>W12/U12</f>
         <v>0.25</v>
       </c>
-      <c r="Y12" s="139">
+      <c r="Y12" s="140">
         <f>U12*$D$6</f>
         <v>145.95928227571108</v>
       </c>
-      <c r="Z12" s="139">
+      <c r="Z12" s="140">
         <f>$F12/(1-$D$4-$Z$9)</f>
         <v>94.77875472448771</v>
       </c>
-      <c r="AA12" s="140">
+      <c r="AA12" s="141">
         <f>Z12*$D$4</f>
         <v>23.694688681121928</v>
       </c>
-      <c r="AB12" s="141">
+      <c r="AB12" s="142">
         <f>Z12-$F12-AA12</f>
         <v>18.955750944897535</v>
       </c>
@@ -4613,19 +4586,19 @@
         <f>AB12/Z12</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD12" s="139">
+      <c r="AD12" s="140">
         <f>Z12*$D$6</f>
         <v>132.6902566142828</v>
       </c>
-      <c r="AE12" s="139">
+      <c r="AE12" s="140">
         <f>$F12/(1-$D$4-$AE$9)</f>
         <v>86.88052516411375</v>
       </c>
-      <c r="AF12" s="140">
+      <c r="AF12" s="141">
         <f>AE12*$D$4</f>
         <v>21.720131291028437</v>
       </c>
-      <c r="AG12" s="141">
+      <c r="AG12" s="142">
         <f>AE12-$F12-AF12</f>
         <v>13.032078774617062</v>
       </c>
@@ -4633,7 +4606,7 @@
         <f>AG12/AE12</f>
         <v>0.15</v>
       </c>
-      <c r="AI12" s="139">
+      <c r="AI12" s="140">
         <f>AE12*$D$6</f>
         <v>121.63273522975923</v>
       </c>
@@ -4655,22 +4628,22 @@
       <c r="D13" s="8" t="n">
         <v>113</v>
       </c>
-      <c r="E13" s="130" t="n">
+      <c r="E13" s="131" t="n">
         <v>0.8823803336980306</v>
       </c>
-      <c r="F13" s="131">
+      <c r="F13" s="132">
         <f>IF(AND(ISNUMBER(E13),ISNUMBER($D$8)),E13*$D$3,NA())</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="G13" s="132">
+      <c r="G13" s="133">
         <f>F13/$D$8</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="H13" s="133">
+      <c r="H13" s="134">
         <f>G13*$D$4</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="I13" s="134">
+      <c r="I13" s="135">
         <f>G13-F13-H13</f>
         <v>39.5306389496718</v>
       </c>
@@ -4678,35 +4651,35 @@
         <f>I13/G13</f>
         <v>0.35000000000000003</v>
       </c>
-      <c r="K13" s="135">
+      <c r="K13" s="136">
         <f>G13*$D$6</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="L13" s="136">
+      <c r="L13" s="137">
         <f>F13/(1-$D$4)</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="M13" s="136">
+      <c r="M13" s="137">
         <f>L13*$D$6</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="N13" s="137">
+      <c r="N13" s="138">
         <f>G13-F13</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="O13" s="138">
+      <c r="O13" s="139">
         <f>N13-H13</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="P13" s="139">
+      <c r="P13" s="140">
         <f>$F13/(1-$D$4-$P$9)</f>
         <v>100.39527352297598</v>
       </c>
-      <c r="Q13" s="140">
+      <c r="Q13" s="141">
         <f>P13*$D$4</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="R13" s="141">
+      <c r="R13" s="142">
         <f>P13-$F13-Q13</f>
         <v>30.118582056892794</v>
       </c>
@@ -4714,19 +4687,19 @@
         <f>R13/P13</f>
         <v>0.3</v>
       </c>
-      <c r="T13" s="139">
+      <c r="T13" s="140">
         <f>P13*$D$6</f>
         <v>140.55338293216636</v>
       </c>
-      <c r="U13" s="139">
+      <c r="U13" s="140">
         <f>$F13/(1-$D$4-$U$9)</f>
         <v>90.35574617067839</v>
       </c>
-      <c r="V13" s="140">
+      <c r="V13" s="141">
         <f>U13*$D$4</f>
         <v>22.588936542669597</v>
       </c>
-      <c r="W13" s="141">
+      <c r="W13" s="142">
         <f>U13-$F13-V13</f>
         <v>22.588936542669597</v>
       </c>
@@ -4734,19 +4707,19 @@
         <f>W13/U13</f>
         <v>0.25</v>
       </c>
-      <c r="Y13" s="139">
+      <c r="Y13" s="140">
         <f>U13*$D$6</f>
         <v>126.49804463894974</v>
       </c>
-      <c r="Z13" s="139">
+      <c r="Z13" s="140">
         <f>$F13/(1-$D$4-$Z$9)</f>
         <v>82.14158742788943</v>
       </c>
-      <c r="AA13" s="140">
+      <c r="AA13" s="141">
         <f>Z13*$D$4</f>
         <v>20.53539685697236</v>
       </c>
-      <c r="AB13" s="141">
+      <c r="AB13" s="142">
         <f>Z13-$F13-AA13</f>
         <v>16.42831748557788</v>
       </c>
@@ -4754,19 +4727,19 @@
         <f>AB13/Z13</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD13" s="139">
+      <c r="AD13" s="140">
         <f>Z13*$D$6</f>
         <v>114.9982223990452</v>
       </c>
-      <c r="AE13" s="139">
+      <c r="AE13" s="140">
         <f>$F13/(1-$D$4-$AE$9)</f>
         <v>75.29645514223199</v>
       </c>
-      <c r="AF13" s="140">
+      <c r="AF13" s="141">
         <f>AE13*$D$4</f>
         <v>18.824113785557998</v>
       </c>
-      <c r="AG13" s="141">
+      <c r="AG13" s="142">
         <f>AE13-$F13-AF13</f>
         <v>11.2944682713348</v>
       </c>
@@ -4774,7 +4747,7 @@
         <f>AG13/AE13</f>
         <v>0.15000000000000002</v>
       </c>
-      <c r="AI13" s="139">
+      <c r="AI13" s="140">
         <f>AE13*$D$6</f>
         <v>105.41503719912478</v>
       </c>
@@ -4793,25 +4766,25 @@
           <t>Spicy Flavor 112.5 г</t>
         </is>
       </c>
-      <c r="D14" s="142" t="n">
+      <c r="D14" s="143" t="n">
         <v>112.5</v>
       </c>
-      <c r="E14" s="130" t="n">
+      <c r="E14" s="131" t="n">
         <v>0.8823803336980306</v>
       </c>
-      <c r="F14" s="131">
+      <c r="F14" s="132">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($D$8)),E14*$D$3,NA())</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="G14" s="132">
+      <c r="G14" s="133">
         <f>F14/$D$8</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="H14" s="133">
+      <c r="H14" s="134">
         <f>G14*$D$4</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="I14" s="134">
+      <c r="I14" s="135">
         <f>G14-F14-H14</f>
         <v>39.5306389496718</v>
       </c>
@@ -4819,35 +4792,35 @@
         <f>I14/G14</f>
         <v>0.35000000000000003</v>
       </c>
-      <c r="K14" s="135">
+      <c r="K14" s="136">
         <f>G14*$D$6</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="L14" s="136">
+      <c r="L14" s="137">
         <f>F14/(1-$D$4)</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="M14" s="136">
+      <c r="M14" s="137">
         <f>L14*$D$6</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="N14" s="137">
+      <c r="N14" s="138">
         <f>G14-F14</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="O14" s="138">
+      <c r="O14" s="139">
         <f>N14-H14</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="P14" s="139">
+      <c r="P14" s="140">
         <f>$F14/(1-$D$4-$P$9)</f>
         <v>100.39527352297598</v>
       </c>
-      <c r="Q14" s="140">
+      <c r="Q14" s="141">
         <f>P14*$D$4</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="R14" s="141">
+      <c r="R14" s="142">
         <f>P14-$F14-Q14</f>
         <v>30.118582056892794</v>
       </c>
@@ -4855,19 +4828,19 @@
         <f>R14/P14</f>
         <v>0.3</v>
       </c>
-      <c r="T14" s="139">
+      <c r="T14" s="140">
         <f>P14*$D$6</f>
         <v>140.55338293216636</v>
       </c>
-      <c r="U14" s="139">
+      <c r="U14" s="140">
         <f>$F14/(1-$D$4-$U$9)</f>
         <v>90.35574617067839</v>
       </c>
-      <c r="V14" s="140">
+      <c r="V14" s="141">
         <f>U14*$D$4</f>
         <v>22.588936542669597</v>
       </c>
-      <c r="W14" s="141">
+      <c r="W14" s="142">
         <f>U14-$F14-V14</f>
         <v>22.588936542669597</v>
       </c>
@@ -4875,19 +4848,19 @@
         <f>W14/U14</f>
         <v>0.25</v>
       </c>
-      <c r="Y14" s="139">
+      <c r="Y14" s="140">
         <f>U14*$D$6</f>
         <v>126.49804463894974</v>
       </c>
-      <c r="Z14" s="139">
+      <c r="Z14" s="140">
         <f>$F14/(1-$D$4-$Z$9)</f>
         <v>82.14158742788943</v>
       </c>
-      <c r="AA14" s="140">
+      <c r="AA14" s="141">
         <f>Z14*$D$4</f>
         <v>20.53539685697236</v>
       </c>
-      <c r="AB14" s="141">
+      <c r="AB14" s="142">
         <f>Z14-$F14-AA14</f>
         <v>16.42831748557788</v>
       </c>
@@ -4895,19 +4868,19 @@
         <f>AB14/Z14</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD14" s="139">
+      <c r="AD14" s="140">
         <f>Z14*$D$6</f>
         <v>114.9982223990452</v>
       </c>
-      <c r="AE14" s="139">
+      <c r="AE14" s="140">
         <f>$F14/(1-$D$4-$AE$9)</f>
         <v>75.29645514223199</v>
       </c>
-      <c r="AF14" s="140">
+      <c r="AF14" s="141">
         <f>AE14*$D$4</f>
         <v>18.824113785557998</v>
       </c>
-      <c r="AG14" s="141">
+      <c r="AG14" s="142">
         <f>AE14-$F14-AF14</f>
         <v>11.2944682713348</v>
       </c>
@@ -4915,7 +4888,7 @@
         <f>AG14/AE14</f>
         <v>0.15000000000000002</v>
       </c>
-      <c r="AI14" s="139">
+      <c r="AI14" s="140">
         <f>AE14*$D$6</f>
         <v>105.41503719912478</v>
       </c>
@@ -4937,22 +4910,22 @@
       <c r="D15" s="8" t="n">
         <v>113</v>
       </c>
-      <c r="E15" s="130" t="n">
+      <c r="E15" s="131" t="n">
         <v>0.8823803336980306</v>
       </c>
-      <c r="F15" s="131">
+      <c r="F15" s="132">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($D$8)),E15*$D$3,NA())</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="G15" s="132">
+      <c r="G15" s="133">
         <f>F15/$D$8</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="H15" s="133">
+      <c r="H15" s="134">
         <f>G15*$D$4</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="I15" s="134">
+      <c r="I15" s="135">
         <f>G15-F15-H15</f>
         <v>39.5306389496718</v>
       </c>
@@ -4960,35 +4933,35 @@
         <f>I15/G15</f>
         <v>0.35000000000000003</v>
       </c>
-      <c r="K15" s="135">
+      <c r="K15" s="136">
         <f>G15*$D$6</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="L15" s="136">
+      <c r="L15" s="137">
         <f>F15/(1-$D$4)</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="M15" s="136">
+      <c r="M15" s="137">
         <f>L15*$D$6</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="N15" s="137">
+      <c r="N15" s="138">
         <f>G15-F15</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="O15" s="138">
+      <c r="O15" s="139">
         <f>N15-H15</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="P15" s="139">
+      <c r="P15" s="140">
         <f>$F15/(1-$D$4-$P$9)</f>
         <v>100.39527352297598</v>
       </c>
-      <c r="Q15" s="140">
+      <c r="Q15" s="141">
         <f>P15*$D$4</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="R15" s="141">
+      <c r="R15" s="142">
         <f>P15-$F15-Q15</f>
         <v>30.118582056892794</v>
       </c>
@@ -4996,19 +4969,19 @@
         <f>R15/P15</f>
         <v>0.3</v>
       </c>
-      <c r="T15" s="139">
+      <c r="T15" s="140">
         <f>P15*$D$6</f>
         <v>140.55338293216636</v>
       </c>
-      <c r="U15" s="139">
+      <c r="U15" s="140">
         <f>$F15/(1-$D$4-$U$9)</f>
         <v>90.35574617067839</v>
       </c>
-      <c r="V15" s="140">
+      <c r="V15" s="141">
         <f>U15*$D$4</f>
         <v>22.588936542669597</v>
       </c>
-      <c r="W15" s="141">
+      <c r="W15" s="142">
         <f>U15-$F15-V15</f>
         <v>22.588936542669597</v>
       </c>
@@ -5016,19 +4989,19 @@
         <f>W15/U15</f>
         <v>0.25</v>
       </c>
-      <c r="Y15" s="139">
+      <c r="Y15" s="140">
         <f>U15*$D$6</f>
         <v>126.49804463894974</v>
       </c>
-      <c r="Z15" s="139">
+      <c r="Z15" s="140">
         <f>$F15/(1-$D$4-$Z$9)</f>
         <v>82.14158742788943</v>
       </c>
-      <c r="AA15" s="140">
+      <c r="AA15" s="141">
         <f>Z15*$D$4</f>
         <v>20.53539685697236</v>
       </c>
-      <c r="AB15" s="141">
+      <c r="AB15" s="142">
         <f>Z15-$F15-AA15</f>
         <v>16.42831748557788</v>
       </c>
@@ -5036,19 +5009,19 @@
         <f>AB15/Z15</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD15" s="139">
+      <c r="AD15" s="140">
         <f>Z15*$D$6</f>
         <v>114.9982223990452</v>
       </c>
-      <c r="AE15" s="139">
+      <c r="AE15" s="140">
         <f>$F15/(1-$D$4-$AE$9)</f>
         <v>75.29645514223199</v>
       </c>
-      <c r="AF15" s="140">
+      <c r="AF15" s="141">
         <f>AE15*$D$4</f>
         <v>18.824113785557998</v>
       </c>
-      <c r="AG15" s="141">
+      <c r="AG15" s="142">
         <f>AE15-$F15-AF15</f>
         <v>11.2944682713348</v>
       </c>
@@ -5056,7 +5029,7 @@
         <f>AG15/AE15</f>
         <v>0.15000000000000002</v>
       </c>
-      <c r="AI15" s="139">
+      <c r="AI15" s="140">
         <f>AE15*$D$6</f>
         <v>105.41503719912478</v>
       </c>
@@ -5078,22 +5051,22 @@
       <c r="D16" s="8" t="n">
         <v>113</v>
       </c>
-      <c r="E16" s="130" t="n">
+      <c r="E16" s="131" t="n">
         <v>0.8823803336980306</v>
       </c>
-      <c r="F16" s="131">
+      <c r="F16" s="132">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($D$8)),E16*$D$3,NA())</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="G16" s="132">
+      <c r="G16" s="133">
         <f>F16/$D$8</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="H16" s="133">
+      <c r="H16" s="134">
         <f>G16*$D$4</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="I16" s="134">
+      <c r="I16" s="135">
         <f>G16-F16-H16</f>
         <v>39.5306389496718</v>
       </c>
@@ -5101,35 +5074,35 @@
         <f>I16/G16</f>
         <v>0.35000000000000003</v>
       </c>
-      <c r="K16" s="135">
+      <c r="K16" s="136">
         <f>G16*$D$6</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="L16" s="136">
+      <c r="L16" s="137">
         <f>F16/(1-$D$4)</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="M16" s="136">
+      <c r="M16" s="137">
         <f>L16*$D$6</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="N16" s="137">
+      <c r="N16" s="138">
         <f>G16-F16</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="O16" s="138">
+      <c r="O16" s="139">
         <f>N16-H16</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="P16" s="139">
+      <c r="P16" s="140">
         <f>$F16/(1-$D$4-$P$9)</f>
         <v>100.39527352297598</v>
       </c>
-      <c r="Q16" s="140">
+      <c r="Q16" s="141">
         <f>P16*$D$4</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="R16" s="141">
+      <c r="R16" s="142">
         <f>P16-$F16-Q16</f>
         <v>30.118582056892794</v>
       </c>
@@ -5137,19 +5110,19 @@
         <f>R16/P16</f>
         <v>0.3</v>
       </c>
-      <c r="T16" s="139">
+      <c r="T16" s="140">
         <f>P16*$D$6</f>
         <v>140.55338293216636</v>
       </c>
-      <c r="U16" s="139">
+      <c r="U16" s="140">
         <f>$F16/(1-$D$4-$U$9)</f>
         <v>90.35574617067839</v>
       </c>
-      <c r="V16" s="140">
+      <c r="V16" s="141">
         <f>U16*$D$4</f>
         <v>22.588936542669597</v>
       </c>
-      <c r="W16" s="141">
+      <c r="W16" s="142">
         <f>U16-$F16-V16</f>
         <v>22.588936542669597</v>
       </c>
@@ -5157,19 +5130,19 @@
         <f>W16/U16</f>
         <v>0.25</v>
       </c>
-      <c r="Y16" s="139">
+      <c r="Y16" s="140">
         <f>U16*$D$6</f>
         <v>126.49804463894974</v>
       </c>
-      <c r="Z16" s="139">
+      <c r="Z16" s="140">
         <f>$F16/(1-$D$4-$Z$9)</f>
         <v>82.14158742788943</v>
       </c>
-      <c r="AA16" s="140">
+      <c r="AA16" s="141">
         <f>Z16*$D$4</f>
         <v>20.53539685697236</v>
       </c>
-      <c r="AB16" s="141">
+      <c r="AB16" s="142">
         <f>Z16-$F16-AA16</f>
         <v>16.42831748557788</v>
       </c>
@@ -5177,19 +5150,19 @@
         <f>AB16/Z16</f>
         <v>0.19999999999999993</v>
       </c>
-      <c r="AD16" s="139">
+      <c r="AD16" s="140">
         <f>Z16*$D$6</f>
         <v>114.9982223990452</v>
       </c>
-      <c r="AE16" s="139">
+      <c r="AE16" s="140">
         <f>$F16/(1-$D$4-$AE$9)</f>
         <v>75.29645514223199</v>
       </c>
-      <c r="AF16" s="140">
+      <c r="AF16" s="141">
         <f>AE16*$D$4</f>
         <v>18.824113785557998</v>
       </c>
-      <c r="AG16" s="141">
+      <c r="AG16" s="142">
         <f>AE16-$F16-AF16</f>
         <v>11.2944682713348</v>
       </c>
@@ -5197,14 +5170,14 @@
         <f>AG16/AE16</f>
         <v>0.15000000000000002</v>
       </c>
-      <c r="AI16" s="139">
+      <c r="AI16" s="140">
         <f>AE16*$D$6</f>
         <v>105.41503719912478</v>
       </c>
     </row>
     <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="27" t="n"/>
-      <c r="B19" s="143" t="inlineStr">
+      <c r="B19" s="144" t="inlineStr">
         <is>
           <t>Кожен крок формування ціни — за вашим прикладом</t>
         </is>
@@ -5229,12 +5202,12 @@
           <t>№</t>
         </is>
       </c>
-      <c r="B21" s="144" t="inlineStr">
+      <c r="B21" s="145" t="inlineStr">
         <is>
           <t>Що рахуємо</t>
         </is>
       </c>
-      <c r="D21" s="144" t="inlineStr">
+      <c r="D21" s="145" t="inlineStr">
         <is>
           <t>Дія</t>
         </is>
@@ -5273,34 +5246,34 @@
           <t>Собівартість в Україні, EUR/уп.</t>
         </is>
       </c>
-      <c r="C22" s="145" t="n"/>
+      <c r="C22" s="146" t="n"/>
       <c r="D22" s="86" t="inlineStr">
         <is>
           <t>Із Self-Cost</t>
         </is>
       </c>
-      <c r="E22" s="145" t="n"/>
-      <c r="F22" s="146">
+      <c r="E22" s="146" t="n"/>
+      <c r="F22" s="147">
         <f>E11</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="G22" s="146">
+      <c r="G22" s="147">
         <f>E12</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="H22" s="146">
+      <c r="H22" s="147">
         <f>E13</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="I22" s="146">
+      <c r="I22" s="147">
         <f>E14</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="J22" s="146">
+      <c r="J22" s="147">
         <f>E15</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="K22" s="146">
+      <c r="K22" s="147">
         <f>E16</f>
         <v>0.882380333698031</v>
       </c>
@@ -5314,13 +5287,13 @@
           <t>Курс, грн/EUR</t>
         </is>
       </c>
-      <c r="C23" s="145" t="n"/>
+      <c r="C23" s="146" t="n"/>
       <c r="D23" s="86" t="inlineStr">
         <is>
           <t>Умова в D3</t>
         </is>
       </c>
-      <c r="E23" s="145" t="n"/>
+      <c r="E23" s="146" t="n"/>
       <c r="F23" s="31">
         <f>$D$3</f>
         <v>51.2</v>
@@ -5355,34 +5328,34 @@
           <t>Собівартість в Україні, грн/уп.</t>
         </is>
       </c>
-      <c r="C24" s="145" t="n"/>
+      <c r="C24" s="146" t="n"/>
       <c r="D24" s="86" t="inlineStr">
         <is>
           <t>Крок 1 × крок 2</t>
         </is>
       </c>
-      <c r="E24" s="145" t="n"/>
-      <c r="F24" s="147">
+      <c r="E24" s="146" t="n"/>
+      <c r="F24" s="148">
         <f>F11</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="G24" s="147">
+      <c r="G24" s="148">
         <f>F12</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="H24" s="147">
+      <c r="H24" s="148">
         <f>F13</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="I24" s="147">
+      <c r="I24" s="148">
         <f>F14</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="J24" s="147">
+      <c r="J24" s="148">
         <f>F15</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="K24" s="147">
+      <c r="K24" s="148">
         <f>F16</f>
         <v>45.17787308533919</v>
       </c>
@@ -5396,13 +5369,13 @@
           <t>Повна ціна партнеру, %</t>
         </is>
       </c>
-      <c r="C25" s="145" t="n"/>
+      <c r="C25" s="146" t="n"/>
       <c r="D25" s="86" t="inlineStr">
         <is>
           <t>База для всіх відсотків</t>
         </is>
       </c>
-      <c r="E25" s="145" t="n"/>
+      <c r="E25" s="146" t="n"/>
       <c r="F25" s="33" t="n">
         <v>1</v>
       </c>
@@ -5431,13 +5404,13 @@
           <t>Бонус мережі, %</t>
         </is>
       </c>
-      <c r="C26" s="145" t="n"/>
+      <c r="C26" s="146" t="n"/>
       <c r="D26" s="86" t="inlineStr">
         <is>
           <t>Умова в D4</t>
         </is>
       </c>
-      <c r="E26" s="145" t="n"/>
+      <c r="E26" s="146" t="n"/>
       <c r="F26" s="33">
         <f>$D$4</f>
         <v>0.25</v>
@@ -5472,13 +5445,13 @@
           <t>Частка ціни після бонусу, %</t>
         </is>
       </c>
-      <c r="C27" s="145" t="n"/>
+      <c r="C27" s="146" t="n"/>
       <c r="D27" s="86" t="inlineStr">
         <is>
           <t>Крок 4 − крок 5</t>
         </is>
       </c>
-      <c r="E27" s="145" t="n"/>
+      <c r="E27" s="146" t="n"/>
       <c r="F27" s="33">
         <f>1-$D$4</f>
         <v>0.75</v>
@@ -5513,13 +5486,13 @@
           <t>Наша цільова маржа, %</t>
         </is>
       </c>
-      <c r="C28" s="145" t="n"/>
+      <c r="C28" s="146" t="n"/>
       <c r="D28" s="86" t="inlineStr">
         <is>
           <t>Умова в D5</t>
         </is>
       </c>
-      <c r="E28" s="145" t="n"/>
+      <c r="E28" s="146" t="n"/>
       <c r="F28" s="33">
         <f>$D$5</f>
         <v>0.35</v>
@@ -5554,13 +5527,13 @@
           <t>Частка ціни для собівартості, %</t>
         </is>
       </c>
-      <c r="C29" s="145" t="n"/>
+      <c r="C29" s="146" t="n"/>
       <c r="D29" s="86" t="inlineStr">
         <is>
           <t>Крок 6 − крок 7</t>
         </is>
       </c>
-      <c r="E29" s="145" t="n"/>
+      <c r="E29" s="146" t="n"/>
       <c r="F29" s="33">
         <f>$D$8</f>
         <v>0.4</v>
@@ -5595,34 +5568,34 @@
           <t>Ціна партнеру з ПДВ, грн/уп.</t>
         </is>
       </c>
-      <c r="C30" s="145" t="n"/>
+      <c r="C30" s="146" t="n"/>
       <c r="D30" s="90" t="inlineStr">
         <is>
           <t>Крок 3 ÷ крок 8</t>
         </is>
       </c>
-      <c r="E30" s="145" t="n"/>
-      <c r="F30" s="148">
+      <c r="E30" s="146" t="n"/>
+      <c r="F30" s="149">
         <f>G11</f>
         <v>130.32078774617062</v>
       </c>
-      <c r="G30" s="148">
+      <c r="G30" s="149">
         <f>G12</f>
         <v>130.32078774617062</v>
       </c>
-      <c r="H30" s="148">
+      <c r="H30" s="149">
         <f>G13</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="I30" s="148">
+      <c r="I30" s="149">
         <f>G14</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="J30" s="148">
+      <c r="J30" s="149">
         <f>G15</f>
         <v>112.94468271334797</v>
       </c>
-      <c r="K30" s="148">
+      <c r="K30" s="149">
         <f>G16</f>
         <v>112.94468271334797</v>
       </c>
@@ -5636,34 +5609,34 @@
           <t>Валовий прибуток до бонусу, грн/уп.</t>
         </is>
       </c>
-      <c r="C31" s="145" t="n"/>
+      <c r="C31" s="146" t="n"/>
       <c r="D31" s="86" t="inlineStr">
         <is>
           <t>Крок 9 − крок 3</t>
         </is>
       </c>
-      <c r="E31" s="145" t="n"/>
-      <c r="F31" s="147">
+      <c r="E31" s="146" t="n"/>
+      <c r="F31" s="148">
         <f>N11</f>
         <v>78.19247264770237</v>
       </c>
-      <c r="G31" s="147">
+      <c r="G31" s="148">
         <f>N12</f>
         <v>78.19247264770237</v>
       </c>
-      <c r="H31" s="147">
+      <c r="H31" s="148">
         <f>N13</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="I31" s="147">
+      <c r="I31" s="148">
         <f>N14</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="J31" s="147">
+      <c r="J31" s="148">
         <f>N15</f>
         <v>67.76680962800879</v>
       </c>
-      <c r="K31" s="147">
+      <c r="K31" s="148">
         <f>N16</f>
         <v>67.76680962800879</v>
       </c>
@@ -5677,34 +5650,34 @@
           <t>Бонус мережі, грн/уп.</t>
         </is>
       </c>
-      <c r="C32" s="145" t="n"/>
+      <c r="C32" s="146" t="n"/>
       <c r="D32" s="86" t="inlineStr">
         <is>
           <t>Крок 9 × крок 5</t>
         </is>
       </c>
-      <c r="E32" s="145" t="n"/>
-      <c r="F32" s="147">
+      <c r="E32" s="146" t="n"/>
+      <c r="F32" s="148">
         <f>H11</f>
         <v>32.580196936542656</v>
       </c>
-      <c r="G32" s="147">
+      <c r="G32" s="148">
         <f>H12</f>
         <v>32.580196936542656</v>
       </c>
-      <c r="H32" s="147">
+      <c r="H32" s="148">
         <f>H13</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="I32" s="147">
+      <c r="I32" s="148">
         <f>H14</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="J32" s="147">
+      <c r="J32" s="148">
         <f>H15</f>
         <v>28.236170678336993</v>
       </c>
-      <c r="K32" s="147">
+      <c r="K32" s="148">
         <f>H16</f>
         <v>28.236170678336993</v>
       </c>
@@ -5718,34 +5691,34 @@
           <t>Нам залишається після собівартості та бонусу, грн/уп.</t>
         </is>
       </c>
-      <c r="C33" s="145" t="n"/>
+      <c r="C33" s="146" t="n"/>
       <c r="D33" s="92" t="inlineStr">
         <is>
           <t>Крок 10 − крок 11</t>
         </is>
       </c>
-      <c r="E33" s="145" t="n"/>
-      <c r="F33" s="149">
+      <c r="E33" s="146" t="n"/>
+      <c r="F33" s="150">
         <f>I11</f>
         <v>45.61227571115972</v>
       </c>
-      <c r="G33" s="149">
+      <c r="G33" s="150">
         <f>I12</f>
         <v>45.61227571115972</v>
       </c>
-      <c r="H33" s="149">
+      <c r="H33" s="150">
         <f>I13</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="I33" s="149">
+      <c r="I33" s="150">
         <f>I14</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="J33" s="149">
+      <c r="J33" s="150">
         <f>I15</f>
         <v>39.5306389496718</v>
       </c>
-      <c r="K33" s="149">
+      <c r="K33" s="150">
         <f>I16</f>
         <v>39.5306389496718</v>
       </c>
@@ -5759,13 +5732,13 @@
           <t>Перевірка нашої маржі після бонусу, %</t>
         </is>
       </c>
-      <c r="C34" s="145" t="n"/>
+      <c r="C34" s="146" t="n"/>
       <c r="D34" s="92" t="inlineStr">
         <is>
           <t>Крок 12 ÷ крок 9</t>
         </is>
       </c>
-      <c r="E34" s="145" t="n"/>
+      <c r="E34" s="146" t="n"/>
       <c r="F34" s="38">
         <f>J11</f>
         <v>0.35</v>
@@ -5800,13 +5773,13 @@
           <t>Націнка ритейлера для полиці, %</t>
         </is>
       </c>
-      <c r="C35" s="145" t="n"/>
+      <c r="C35" s="146" t="n"/>
       <c r="D35" s="86" t="inlineStr">
         <is>
           <t>Множник D6 − 1</t>
         </is>
       </c>
-      <c r="E35" s="145" t="n"/>
+      <c r="E35" s="146" t="n"/>
       <c r="F35" s="33">
         <f>$D$6-1</f>
         <v>0.3999999999999999</v>
@@ -5841,34 +5814,34 @@
           <t>Множник ритейлера</t>
         </is>
       </c>
-      <c r="C36" s="145" t="n"/>
+      <c r="C36" s="146" t="n"/>
       <c r="D36" s="86" t="inlineStr">
         <is>
           <t>1 + крок 14</t>
         </is>
       </c>
-      <c r="E36" s="145" t="n"/>
-      <c r="F36" s="150">
+      <c r="E36" s="146" t="n"/>
+      <c r="F36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="G36" s="150">
+      <c r="G36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="H36" s="150">
+      <c r="H36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="I36" s="150">
+      <c r="I36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="J36" s="150">
+      <c r="J36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
-      <c r="K36" s="150">
+      <c r="K36" s="151">
         <f>$D$6</f>
         <v>1.4</v>
       </c>
@@ -5882,34 +5855,34 @@
           <t>Ціна на полиці з ПДВ, грн/уп.</t>
         </is>
       </c>
-      <c r="C37" s="145" t="n"/>
+      <c r="C37" s="146" t="n"/>
       <c r="D37" s="90" t="inlineStr">
         <is>
           <t>Крок 9 × крок 15</t>
         </is>
       </c>
-      <c r="E37" s="145" t="n"/>
-      <c r="F37" s="148">
+      <c r="E37" s="146" t="n"/>
+      <c r="F37" s="149">
         <f>K11</f>
         <v>182.44910284463887</v>
       </c>
-      <c r="G37" s="148">
+      <c r="G37" s="149">
         <f>K12</f>
         <v>182.44910284463887</v>
       </c>
-      <c r="H37" s="148">
+      <c r="H37" s="149">
         <f>K13</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="I37" s="148">
+      <c r="I37" s="149">
         <f>K14</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="J37" s="148">
+      <c r="J37" s="149">
         <f>K15</f>
         <v>158.12255579868716</v>
       </c>
-      <c r="K37" s="148">
+      <c r="K37" s="149">
         <f>K16</f>
         <v>158.12255579868716</v>
       </c>
@@ -5923,34 +5896,34 @@
           <t>Ціна партнеру при нульовому нашому прибутку, грн/уп.</t>
         </is>
       </c>
-      <c r="C38" s="145" t="n"/>
+      <c r="C38" s="146" t="n"/>
       <c r="D38" s="86" t="inlineStr">
         <is>
           <t>Крок 3 ÷ крок 6</t>
         </is>
       </c>
-      <c r="E38" s="145" t="n"/>
-      <c r="F38" s="147">
+      <c r="E38" s="146" t="n"/>
+      <c r="F38" s="148">
         <f>L11</f>
         <v>69.504420131291</v>
       </c>
-      <c r="G38" s="147">
+      <c r="G38" s="148">
         <f>L12</f>
         <v>69.504420131291</v>
       </c>
-      <c r="H38" s="147">
+      <c r="H38" s="148">
         <f>L13</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="I38" s="147">
+      <c r="I38" s="148">
         <f>L14</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="J38" s="147">
+      <c r="J38" s="148">
         <f>L15</f>
         <v>60.23716411378559</v>
       </c>
-      <c r="K38" s="147">
+      <c r="K38" s="148">
         <f>L16</f>
         <v>60.23716411378559</v>
       </c>
@@ -5964,44 +5937,42 @@
           <t>Полиця при нульовому нашому прибутку, грн/уп.</t>
         </is>
       </c>
-      <c r="C39" s="145" t="n"/>
+      <c r="C39" s="146" t="n"/>
       <c r="D39" s="86" t="inlineStr">
         <is>
           <t>Крок 17 × крок 15</t>
         </is>
       </c>
-      <c r="E39" s="145" t="n"/>
-      <c r="F39" s="147">
+      <c r="E39" s="146" t="n"/>
+      <c r="F39" s="148">
         <f>M11</f>
         <v>97.3061881838074</v>
       </c>
-      <c r="G39" s="147">
+      <c r="G39" s="148">
         <f>M12</f>
         <v>97.3061881838074</v>
       </c>
-      <c r="H39" s="147">
+      <c r="H39" s="148">
         <f>M13</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="I39" s="147">
+      <c r="I39" s="148">
         <f>M14</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="J39" s="147">
+      <c r="J39" s="148">
         <f>M15</f>
         <v>84.33202975929981</v>
       </c>
-      <c r="K39" s="147">
+      <c r="K39" s="148">
         <f>M16</f>
         <v>84.33202975929981</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="73">
-    <mergeCell ref="L2:M2"/>
+  <mergeCells count="63">
     <mergeCell ref="U9:Y9"/>
     <mergeCell ref="Z9:AD9"/>
-    <mergeCell ref="L7:M7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
@@ -6016,28 +5987,22 @@
     <mergeCell ref="P9:T9"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="B39:C39"/>
-    <mergeCell ref="L3:M3"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="G9:J9"/>
-    <mergeCell ref="N3:O3"/>
     <mergeCell ref="D35:E35"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="D27:E27"/>
-    <mergeCell ref="N2:O2"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="D32:E32"/>
-    <mergeCell ref="L5:M5"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="N5:O5"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="E5:K5"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="L4:M4"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
@@ -6056,7 +6021,6 @@
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L6:M6"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D29:E29"/>
@@ -6070,7 +6034,6 @@
     <mergeCell ref="B19:K19"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="N4:O4"/>
   </mergeCells>
   <conditionalFormatting sqref="E33:K36">
     <cfRule type="expression" priority="2" dxfId="4">
@@ -6110,580 +6073,580 @@
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="151" t="inlineStr">
+      <c r="B2" s="152" t="inlineStr">
         <is>
           <t>SIAS · было → стало · от себестоимости в Украине до полки · 6 паллет</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="152" t="str">
+      <c r="B3" s="153" t="str">
         <f>"Полка "&amp;ROUND(C14,0)&amp;" ₴ достижима при себестоимости "&amp;ROUND(D9,2)&amp;" ₴ (сейчас "&amp;ROUND(D7,2)&amp;"–"&amp;ROUND(D8,2)&amp;" ₴). Для этого закупка SIAS должна быть €"&amp;ROUND(C21,2)&amp;" вместо €"&amp;MIN(C20,E20)&amp;"–€"&amp;MAX(C20,E20)&amp;" (−"&amp;ROUND((1-C21/MIN(C20,E20))*100,0)&amp;"…"&amp;ROUND((1-C21/MAX(C20,E20))*100,0)&amp;"%)."</f>
         <v>Полка 120 ₴ достижима при себестоимости 38.16 ₴ (сейчас 58.06–67 ₴). Для этого закупка SIAS должна быть €0.32 вместо €0.65–€0.75 (−51…57%).</v>
       </c>
-      <c r="C3" s="153" t="n"/>
-      <c r="D3" s="153" t="n"/>
-      <c r="E3" s="153" t="n"/>
-      <c r="F3" s="153" t="n"/>
-      <c r="G3" s="153" t="n"/>
-      <c r="H3" s="153" t="n"/>
-      <c r="I3" s="153" t="n"/>
-      <c r="J3" s="153" t="n"/>
-      <c r="K3" s="153" t="n"/>
-      <c r="L3" s="153" t="n"/>
-      <c r="M3" s="153" t="n"/>
-      <c r="N3" s="153" t="n"/>
+      <c r="C3" s="154" t="n"/>
+      <c r="D3" s="154" t="n"/>
+      <c r="E3" s="154" t="n"/>
+      <c r="F3" s="154" t="n"/>
+      <c r="G3" s="154" t="n"/>
+      <c r="H3" s="154" t="n"/>
+      <c r="I3" s="154" t="n"/>
+      <c r="J3" s="154" t="n"/>
+      <c r="K3" s="154" t="n"/>
+      <c r="L3" s="154" t="n"/>
+      <c r="M3" s="154" t="n"/>
+      <c r="N3" s="154" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="154" t="inlineStr"/>
-      <c r="C5" s="154" t="inlineStr">
+      <c r="B5" s="155" t="inlineStr"/>
+      <c r="C5" s="155" t="inlineStr">
         <is>
           <t>Себестоимость в Украине (СС)</t>
         </is>
       </c>
-      <c r="D5" s="155" t="n"/>
-      <c r="E5" s="154" t="inlineStr">
+      <c r="D5" s="156" t="n"/>
+      <c r="E5" s="155" t="inlineStr">
         <is>
           <t>Цена партнёру (магазину)</t>
         </is>
       </c>
-      <c r="F5" s="155" t="n"/>
-      <c r="G5" s="154" t="inlineStr">
+      <c r="F5" s="156" t="n"/>
+      <c r="G5" s="155" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="H5" s="155" t="n"/>
-      <c r="I5" s="154" t="inlineStr">
+      <c r="H5" s="156" t="n"/>
+      <c r="I5" s="155" t="inlineStr">
         <is>
           <t>Наша прибыль</t>
         </is>
       </c>
-      <c r="J5" s="155" t="n"/>
-      <c r="K5" s="154" t="inlineStr">
+      <c r="J5" s="156" t="n"/>
+      <c r="K5" s="155" t="inlineStr">
         <is>
           <t>Наценка магазина</t>
         </is>
       </c>
-      <c r="L5" s="155" t="n"/>
-      <c r="M5" s="154" t="inlineStr">
+      <c r="L5" s="156" t="n"/>
+      <c r="M5" s="155" t="inlineStr">
         <is>
           <t>ПОЛКА с НДС</t>
         </is>
       </c>
-      <c r="N5" s="155" t="n"/>
+      <c r="N5" s="156" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="154" t="inlineStr">
+      <c r="B6" s="155" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="C6" s="156" t="inlineStr">
+      <c r="C6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="D6" s="156" t="inlineStr">
+      <c r="D6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="E6" s="156" t="inlineStr">
+      <c r="E6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="F6" s="156" t="inlineStr">
+      <c r="F6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="G6" s="156" t="inlineStr">
+      <c r="G6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="H6" s="156" t="inlineStr">
+      <c r="H6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="I6" s="156" t="inlineStr">
+      <c r="I6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="J6" s="156" t="inlineStr">
+      <c r="J6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="K6" s="156" t="inlineStr">
+      <c r="K6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="L6" s="156" t="inlineStr">
+      <c r="L6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="M6" s="156" t="inlineStr">
+      <c r="M6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="N6" s="156" t="inlineStr">
+      <c r="N6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="157" t="str">
+      <c r="B7" s="158" t="str">
         <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
         <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
       </c>
-      <c r="C7" s="158">
+      <c r="C7" s="159">
         <f>'Финмодель 6 паллет'!E13</f>
         <v>1.134046875</v>
       </c>
-      <c r="D7" s="159">
+      <c r="D7" s="160">
         <f>C7*K14</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="E7" s="160">
+      <c r="E7" s="161">
         <f>F7/K14</f>
         <v>2.520104166666666</v>
       </c>
-      <c r="F7" s="159">
+      <c r="F7" s="160">
         <f>D7/(1-G14-E14)</f>
         <v>129.0293333333333</v>
       </c>
-      <c r="G7" s="160">
+      <c r="G7" s="161">
         <f>H7/K14</f>
         <v>0.6300260416666665</v>
       </c>
-      <c r="H7" s="161">
+      <c r="H7" s="162">
         <f>F7*G14</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="I7" s="160">
+      <c r="I7" s="161">
         <f>J7/K14</f>
         <v>0.7560312499999997</v>
       </c>
-      <c r="J7" s="161">
+      <c r="J7" s="162">
         <f>F7-D7-H7</f>
         <v>38.70879999999999</v>
       </c>
-      <c r="K7" s="160">
+      <c r="K7" s="161">
         <f>L7/K14</f>
         <v>1.0080416666666663</v>
       </c>
-      <c r="L7" s="161">
+      <c r="L7" s="162">
         <f>F7*(I14-1)</f>
         <v>51.61173333333331</v>
       </c>
-      <c r="M7" s="160">
+      <c r="M7" s="161">
         <f>N7/K14</f>
         <v>3.5281458333333324</v>
       </c>
-      <c r="N7" s="162">
+      <c r="N7" s="163">
         <f>F7*I14</f>
         <v>180.64106666666663</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="163" t="str">
+      <c r="B8" s="164" t="str">
         <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
         <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
       </c>
-      <c r="C8" s="158">
+      <c r="C8" s="159">
         <f>'Финмодель 6 паллет'!E11</f>
         <v>1.308515625</v>
       </c>
-      <c r="D8" s="164">
+      <c r="D8" s="165">
         <f>C8*K14</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="E8" s="165">
+      <c r="E8" s="166">
         <f>F8/K14</f>
         <v>2.9078125000000004</v>
       </c>
-      <c r="F8" s="164">
+      <c r="F8" s="165">
         <f>D8/(1-G14-E14)</f>
         <v>148.88000000000002</v>
       </c>
-      <c r="G8" s="165">
+      <c r="G8" s="166">
         <f>H8/K14</f>
         <v>0.7269531250000001</v>
       </c>
-      <c r="H8" s="166">
+      <c r="H8" s="167">
         <f>F8*G14</f>
         <v>37.220000000000006</v>
       </c>
-      <c r="I8" s="165">
+      <c r="I8" s="166">
         <f>J8/K14</f>
         <v>0.8723437500000001</v>
       </c>
-      <c r="J8" s="166">
+      <c r="J8" s="167">
         <f>F8-D8-H8</f>
         <v>44.66400000000001</v>
       </c>
-      <c r="K8" s="165">
+      <c r="K8" s="166">
         <f>L8/K14</f>
         <v>1.163125</v>
       </c>
-      <c r="L8" s="166">
+      <c r="L8" s="167">
         <f>F8*(I14-1)</f>
         <v>59.552</v>
       </c>
-      <c r="M8" s="165">
+      <c r="M8" s="166">
         <f>N8/K14</f>
         <v>4.0709375</v>
       </c>
-      <c r="N8" s="167">
+      <c r="N8" s="168">
         <f>F8*I14</f>
         <v>208.43200000000002</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="168" t="str">
+      <c r="B9" s="169" t="str">
         <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
         <v>ПОСЛЕ · запрос SIAS €0.32 (все 6 SKU)</v>
       </c>
-      <c r="C9" s="169">
+      <c r="C9" s="170">
         <f>D9/K14</f>
         <v>0.7453031249999998</v>
       </c>
-      <c r="D9" s="170">
+      <c r="D9" s="171">
         <f>C23</f>
         <v>38.15951999999999</v>
       </c>
-      <c r="E9" s="169">
+      <c r="E9" s="170">
         <f>F9/K14</f>
         <v>1.6562291666666664</v>
       </c>
-      <c r="F9" s="170">
+      <c r="F9" s="171">
         <f>D9/(1-G14-E14)</f>
         <v>84.79893333333332</v>
       </c>
-      <c r="G9" s="169">
+      <c r="G9" s="170">
         <f>H9/K14</f>
         <v>0.4140572916666666</v>
       </c>
-      <c r="H9" s="171">
+      <c r="H9" s="172">
         <f>F9*G14</f>
         <v>21.19973333333333</v>
       </c>
-      <c r="I9" s="169">
+      <c r="I9" s="170">
         <f>J9/K14</f>
         <v>0.49686874999999997</v>
       </c>
-      <c r="J9" s="171">
+      <c r="J9" s="172">
         <f>F9-D9-H9</f>
         <v>25.43968</v>
       </c>
-      <c r="K9" s="169">
+      <c r="K9" s="170">
         <f>L9/K14</f>
         <v>0.6624916666666665</v>
       </c>
-      <c r="L9" s="171">
+      <c r="L9" s="172">
         <f>F9*(I14-1)</f>
         <v>33.919573333333325</v>
       </c>
-      <c r="M9" s="169">
+      <c r="M9" s="170">
         <f>N9/K14</f>
         <v>2.318720833333333</v>
       </c>
-      <c r="N9" s="172">
+      <c r="N9" s="173">
         <f>F9*I14</f>
         <v>118.71850666666664</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="173" t="inlineStr">
+      <c r="B10" s="174" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="174">
+      <c r="C10" s="175">
         <f>C9-C7</f>
         <v>-0.38874375000000005</v>
       </c>
-      <c r="D10" s="175">
+      <c r="D10" s="176">
         <f>D9-D7</f>
         <v>-19.90368</v>
       </c>
-      <c r="E10" s="174">
+      <c r="E10" s="175">
         <f>E9-E7</f>
         <v>-0.8638749999999997</v>
       </c>
-      <c r="F10" s="175">
+      <c r="F10" s="176">
         <f>F9-F7</f>
         <v>-44.23039999999999</v>
       </c>
-      <c r="G10" s="174">
+      <c r="G10" s="175">
         <f>G9-G7</f>
         <v>-0.21596874999999993</v>
       </c>
-      <c r="H10" s="175">
+      <c r="H10" s="176">
         <f>H9-H7</f>
         <v>-11.057599999999997</v>
       </c>
-      <c r="I10" s="174">
+      <c r="I10" s="175">
         <f>I9-I7</f>
         <v>-0.25916249999999974</v>
       </c>
-      <c r="J10" s="175">
+      <c r="J10" s="176">
         <f>J9-J7</f>
         <v>-13.26911999999999</v>
       </c>
-      <c r="K10" s="174">
+      <c r="K10" s="175">
         <f>K9-K7</f>
         <v>-0.3455499999999998</v>
       </c>
-      <c r="L10" s="175">
+      <c r="L10" s="176">
         <f>L9-L7</f>
         <v>-17.692159999999987</v>
       </c>
-      <c r="M10" s="174">
+      <c r="M10" s="175">
         <f>M9-M7</f>
         <v>-1.2094249999999995</v>
       </c>
-      <c r="N10" s="175">
+      <c r="N10" s="176">
         <f>N9-N7</f>
         <v>-61.92255999999999</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="176" t="inlineStr">
+      <c r="B11" s="177" t="inlineStr">
         <is>
           <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="177" t="inlineStr">
+      <c r="B12" s="178" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 6 паллет»</t>
         </is>
       </c>
-      <c r="C12" s="178" t="n"/>
-      <c r="D12" s="178" t="n"/>
-      <c r="E12" s="178" t="n"/>
-      <c r="F12" s="178" t="n"/>
-      <c r="G12" s="178" t="n"/>
-      <c r="H12" s="178" t="n"/>
-      <c r="I12" s="178" t="n"/>
-      <c r="J12" s="178" t="n"/>
-      <c r="K12" s="178" t="n"/>
-      <c r="L12" s="178" t="n"/>
-      <c r="M12" s="178" t="n"/>
-      <c r="N12" s="178" t="n"/>
+      <c r="C12" s="179" t="n"/>
+      <c r="D12" s="179" t="n"/>
+      <c r="E12" s="179" t="n"/>
+      <c r="F12" s="179" t="n"/>
+      <c r="G12" s="179" t="n"/>
+      <c r="H12" s="179" t="n"/>
+      <c r="I12" s="179" t="n"/>
+      <c r="J12" s="179" t="n"/>
+      <c r="K12" s="179" t="n"/>
+      <c r="L12" s="179" t="n"/>
+      <c r="M12" s="179" t="n"/>
+      <c r="N12" s="179" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="C13" s="179" t="inlineStr">
+      <c r="C13" s="180" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E13" s="179" t="inlineStr">
+      <c r="E13" s="180" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G13" s="179" t="inlineStr">
+      <c r="G13" s="180" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I13" s="179" t="inlineStr">
+      <c r="I13" s="180" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K13" s="179" t="inlineStr">
+      <c r="K13" s="180" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="180" t="inlineStr">
+      <c r="B14" s="181" t="inlineStr">
         <is>
           <t>Цель расчёта и условия модели</t>
         </is>
       </c>
-      <c r="C14" s="181" t="n">
+      <c r="C14" s="182" t="n">
         <v>120</v>
       </c>
-      <c r="D14" s="182" t="n"/>
-      <c r="E14" s="183" t="n">
+      <c r="D14" s="183" t="n"/>
+      <c r="E14" s="184" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="182" t="n"/>
-      <c r="G14" s="184">
+      <c r="F14" s="183" t="n"/>
+      <c r="G14" s="185">
         <f>'Финмодель 6 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H14" s="185" t="n"/>
-      <c r="I14" s="186">
+      <c r="H14" s="186" t="n"/>
+      <c r="I14" s="187">
         <f>'Финмодель 6 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J14" s="185" t="n"/>
-      <c r="K14" s="187">
+      <c r="J14" s="186" t="n"/>
+      <c r="K14" s="188">
         <f>'Финмодель 6 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L14" s="185" t="n"/>
+      <c r="L14" s="186" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="188" t="inlineStr">
+      <c r="B15" s="189" t="inlineStr">
         <is>
           <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
         </is>
       </c>
     </row>
     <row r="16" hidden="1">
-      <c r="C16" s="179" t="inlineStr">
+      <c r="C16" s="180" t="inlineStr">
         <is>
           <t>Импортный ПДВ</t>
         </is>
       </c>
-      <c r="E16" s="179" t="inlineStr">
+      <c r="E16" s="180" t="inlineStr">
         <is>
           <t>Финансирование</t>
         </is>
       </c>
-      <c r="G16" s="179" t="inlineStr">
+      <c r="G16" s="180" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="I16" s="179" t="inlineStr">
+      <c r="I16" s="180" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="K16" s="179" t="inlineStr">
+      <c r="K16" s="180" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="M16" s="179" t="inlineStr">
+      <c r="M16" s="180" t="inlineStr">
         <is>
           <t>Прочие, €</t>
         </is>
       </c>
     </row>
     <row r="17" hidden="1">
-      <c r="C17" s="183" t="n">
+      <c r="C17" s="184" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="182" t="n"/>
-      <c r="E17" s="183" t="n">
+      <c r="D17" s="183" t="n"/>
+      <c r="E17" s="184" t="n">
         <v>0.025</v>
       </c>
-      <c r="F17" s="182" t="n"/>
-      <c r="G17" s="183" t="n">
+      <c r="F17" s="183" t="n"/>
+      <c r="G17" s="184" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="182" t="n"/>
-      <c r="I17" s="189" t="n">
+      <c r="H17" s="183" t="n"/>
+      <c r="I17" s="190" t="n">
         <v>2600</v>
       </c>
-      <c r="J17" s="182" t="n"/>
-      <c r="K17" s="189" t="n">
+      <c r="J17" s="183" t="n"/>
+      <c r="K17" s="190" t="n">
         <v>288</v>
       </c>
-      <c r="L17" s="182" t="n"/>
-      <c r="M17" s="189" t="n">
+      <c r="L17" s="183" t="n"/>
+      <c r="M17" s="190" t="n">
         <v>42</v>
       </c>
-      <c r="N17" s="182" t="n"/>
+      <c r="N17" s="183" t="n"/>
     </row>
     <row r="18" hidden="1">
-      <c r="C18" s="179" t="inlineStr">
+      <c r="C18" s="180" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="E18" s="179" t="inlineStr">
+      <c r="E18" s="180" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="G18" s="179" t="inlineStr">
+      <c r="G18" s="180" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
     <row r="19" hidden="1">
-      <c r="C19" s="190" t="n">
+      <c r="C19" s="191" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="182" t="n"/>
-      <c r="E19" s="189" t="n">
+      <c r="D19" s="183" t="n"/>
+      <c r="E19" s="190" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="182" t="n"/>
-      <c r="G19" s="189" t="n">
+      <c r="F19" s="183" t="n"/>
+      <c r="G19" s="190" t="n">
         <v>1600</v>
       </c>
-      <c r="H19" s="182" t="n"/>
+      <c r="H19" s="183" t="n"/>
     </row>
     <row r="20" hidden="1">
-      <c r="B20" s="191" t="inlineStr">
+      <c r="B20" s="192" t="inlineStr">
         <is>
           <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
         </is>
       </c>
-      <c r="C20" s="190" t="n">
+      <c r="C20" s="191" t="n">
         <v>0.65</v>
       </c>
-      <c r="E20" s="190" t="n">
+      <c r="E20" s="191" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="21" hidden="1">
-      <c r="B21" s="191" t="inlineStr">
+      <c r="B21" s="192" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
-      <c r="C21" s="192">
+      <c r="C21" s="193">
         <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
         <v>0.32</v>
       </c>
-      <c r="D21" s="193" t="n"/>
+      <c r="D21" s="194" t="n"/>
     </row>
     <row r="22" hidden="1">
-      <c r="B22" s="191" t="inlineStr">
+      <c r="B22" s="192" t="inlineStr">
         <is>
           <t>Предельная закупка до округления, €/уп.</t>
         </is>
       </c>
-      <c r="C22" s="194">
+      <c r="C22" s="195">
         <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
         <v>0.3265407229965157</v>
       </c>
-      <c r="D22" s="195" t="n"/>
+      <c r="D22" s="196" t="n"/>
     </row>
     <row r="23" hidden="1">
-      <c r="B23" s="191" t="inlineStr">
+      <c r="B23" s="192" t="inlineStr">
         <is>
           <t>Себестоимость в Украине при запросе, ₴/уп.</t>
         </is>
       </c>
-      <c r="C23" s="196">
+      <c r="C23" s="197">
         <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
         <v>38.15951999999999</v>
       </c>
-      <c r="D23" s="195" t="n"/>
+      <c r="D23" s="196" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="42">
@@ -6764,580 +6727,580 @@
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="151" t="inlineStr">
+      <c r="B2" s="152" t="inlineStr">
         <is>
           <t>SIAS · было → стало · от себестоимости в Украине до полки · 33 паллеты (Full Truck)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="152" t="str">
+      <c r="B3" s="153" t="str">
         <f>"Полка "&amp;ROUND(C14,0)&amp;" ₴ достижима при себестоимости "&amp;ROUND(D9,2)&amp;" ₴ (сейчас "&amp;ROUND(D7,2)&amp;"–"&amp;ROUND(D8,2)&amp;" ₴). Для этого закупка SIAS должна быть €"&amp;ROUND(C21,2)&amp;" вместо €"&amp;MIN(C20,E20)&amp;"–€"&amp;MAX(C20,E20)&amp;" (−"&amp;ROUND((1-C21/MIN(C20,E20))*100,0)&amp;"…"&amp;ROUND((1-C21/MAX(C20,E20))*100,0)&amp;"%)."</f>
         <v>Полка 120 ₴ достижима при себестоимости 38.53 ₴ (сейчас 45.18–52.13 ₴). Для этого закупка SIAS должна быть €0.54 вместо €0.65–€0.75 (−17…28%).</v>
       </c>
-      <c r="C3" s="153" t="n"/>
-      <c r="D3" s="153" t="n"/>
-      <c r="E3" s="153" t="n"/>
-      <c r="F3" s="153" t="n"/>
-      <c r="G3" s="153" t="n"/>
-      <c r="H3" s="153" t="n"/>
-      <c r="I3" s="153" t="n"/>
-      <c r="J3" s="153" t="n"/>
-      <c r="K3" s="153" t="n"/>
-      <c r="L3" s="153" t="n"/>
-      <c r="M3" s="153" t="n"/>
-      <c r="N3" s="153" t="n"/>
+      <c r="C3" s="154" t="n"/>
+      <c r="D3" s="154" t="n"/>
+      <c r="E3" s="154" t="n"/>
+      <c r="F3" s="154" t="n"/>
+      <c r="G3" s="154" t="n"/>
+      <c r="H3" s="154" t="n"/>
+      <c r="I3" s="154" t="n"/>
+      <c r="J3" s="154" t="n"/>
+      <c r="K3" s="154" t="n"/>
+      <c r="L3" s="154" t="n"/>
+      <c r="M3" s="154" t="n"/>
+      <c r="N3" s="154" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="154" t="inlineStr"/>
-      <c r="C5" s="154" t="inlineStr">
+      <c r="B5" s="155" t="inlineStr"/>
+      <c r="C5" s="155" t="inlineStr">
         <is>
           <t>Себестоимость в Украине (СС)</t>
         </is>
       </c>
-      <c r="D5" s="155" t="n"/>
-      <c r="E5" s="154" t="inlineStr">
+      <c r="D5" s="156" t="n"/>
+      <c r="E5" s="155" t="inlineStr">
         <is>
           <t>Цена партнёру (магазину)</t>
         </is>
       </c>
-      <c r="F5" s="155" t="n"/>
-      <c r="G5" s="154" t="inlineStr">
+      <c r="F5" s="156" t="n"/>
+      <c r="G5" s="155" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="H5" s="155" t="n"/>
-      <c r="I5" s="154" t="inlineStr">
+      <c r="H5" s="156" t="n"/>
+      <c r="I5" s="155" t="inlineStr">
         <is>
           <t>Наша прибыль</t>
         </is>
       </c>
-      <c r="J5" s="155" t="n"/>
-      <c r="K5" s="154" t="inlineStr">
+      <c r="J5" s="156" t="n"/>
+      <c r="K5" s="155" t="inlineStr">
         <is>
           <t>Наценка магазина</t>
         </is>
       </c>
-      <c r="L5" s="155" t="n"/>
-      <c r="M5" s="154" t="inlineStr">
+      <c r="L5" s="156" t="n"/>
+      <c r="M5" s="155" t="inlineStr">
         <is>
           <t>ПОЛКА с НДС</t>
         </is>
       </c>
-      <c r="N5" s="155" t="n"/>
+      <c r="N5" s="156" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="154" t="inlineStr">
+      <c r="B6" s="155" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="C6" s="156" t="inlineStr">
+      <c r="C6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="D6" s="156" t="inlineStr">
+      <c r="D6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="E6" s="156" t="inlineStr">
+      <c r="E6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="F6" s="156" t="inlineStr">
+      <c r="F6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="G6" s="156" t="inlineStr">
+      <c r="G6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="H6" s="156" t="inlineStr">
+      <c r="H6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="I6" s="156" t="inlineStr">
+      <c r="I6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="J6" s="156" t="inlineStr">
+      <c r="J6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="K6" s="156" t="inlineStr">
+      <c r="K6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="L6" s="156" t="inlineStr">
+      <c r="L6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="M6" s="156" t="inlineStr">
+      <c r="M6" s="157" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="N6" s="156" t="inlineStr">
+      <c r="N6" s="157" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="157" t="str">
+      <c r="B7" s="158" t="str">
         <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
         <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
       </c>
-      <c r="C7" s="158">
+      <c r="C7" s="159">
         <f>'Финмодель 33 паллет'!E13</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="D7" s="159">
+      <c r="D7" s="160">
         <f>C7*K14</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="E7" s="160">
+      <c r="E7" s="161">
         <f>F7/K14</f>
         <v>1.9608451859956246</v>
       </c>
-      <c r="F7" s="159">
+      <c r="F7" s="160">
         <f>D7/(1-G14-E14)</f>
         <v>100.39527352297598</v>
       </c>
-      <c r="G7" s="160">
+      <c r="G7" s="161">
         <f>H7/K14</f>
         <v>0.49021129649890616</v>
       </c>
-      <c r="H7" s="161">
+      <c r="H7" s="162">
         <f>F7*G14</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="I7" s="160">
+      <c r="I7" s="161">
         <f>J7/K14</f>
         <v>0.5882535557986873</v>
       </c>
-      <c r="J7" s="161">
+      <c r="J7" s="162">
         <f>F7-D7-H7</f>
         <v>30.118582056892794</v>
       </c>
-      <c r="K7" s="160">
+      <c r="K7" s="161">
         <f>L7/K14</f>
         <v>0.7843380743982498</v>
       </c>
-      <c r="L7" s="161">
+      <c r="L7" s="162">
         <f>F7*(I14-1)</f>
         <v>40.15810940919039</v>
       </c>
-      <c r="M7" s="160">
+      <c r="M7" s="161">
         <f>N7/K14</f>
         <v>2.745183260393874</v>
       </c>
-      <c r="N7" s="162">
+      <c r="N7" s="163">
         <f>F7*I14</f>
         <v>140.55338293216636</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="163" t="str">
+      <c r="B8" s="164" t="str">
         <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
         <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
       </c>
-      <c r="C8" s="158">
+      <c r="C8" s="159">
         <f>'Финмодель 33 паллет'!E11</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="D8" s="164">
+      <c r="D8" s="165">
         <f>C8*K14</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="E8" s="165">
+      <c r="E8" s="166">
         <f>F8/K14</f>
         <v>2.2625136761487954</v>
       </c>
-      <c r="F8" s="164">
+      <c r="F8" s="165">
         <f>D8/(1-G14-E14)</f>
         <v>115.84070021881833</v>
       </c>
-      <c r="G8" s="165">
+      <c r="G8" s="166">
         <f>H8/K14</f>
         <v>0.5656284190371988</v>
       </c>
-      <c r="H8" s="166">
+      <c r="H8" s="167">
         <f>F8*G14</f>
         <v>28.96017505470458</v>
       </c>
-      <c r="I8" s="165">
+      <c r="I8" s="166">
         <f>J8/K14</f>
         <v>0.6787541028446387</v>
       </c>
-      <c r="J8" s="166">
+      <c r="J8" s="167">
         <f>F8-D8-H8</f>
         <v>34.7522100656455</v>
       </c>
-      <c r="K8" s="165">
+      <c r="K8" s="166">
         <f>L8/K14</f>
         <v>0.905005470459518</v>
       </c>
-      <c r="L8" s="166">
+      <c r="L8" s="167">
         <f>F8*(I14-1)</f>
         <v>46.33628008752732</v>
       </c>
-      <c r="M8" s="165">
+      <c r="M8" s="166">
         <f>N8/K14</f>
         <v>3.1675191466083135</v>
       </c>
-      <c r="N8" s="167">
+      <c r="N8" s="168">
         <f>F8*I14</f>
         <v>162.17698030634565</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="168" t="str">
+      <c r="B9" s="169" t="str">
         <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
         <v>ПОСЛЕ · запрос SIAS €0.54 (все 6 SKU)</v>
       </c>
-      <c r="C9" s="169">
+      <c r="C9" s="170">
         <f>D9/K14</f>
         <v>0.7524897727272728</v>
       </c>
-      <c r="D9" s="170">
+      <c r="D9" s="171">
         <f>C23</f>
         <v>38.52747636363637</v>
       </c>
-      <c r="E9" s="169">
+      <c r="E9" s="170">
         <f>F9/K14</f>
         <v>1.672199494949495</v>
       </c>
-      <c r="F9" s="170">
+      <c r="F9" s="171">
         <f>D9/(1-G14-E14)</f>
         <v>85.61661414141415</v>
       </c>
-      <c r="G9" s="169">
+      <c r="G9" s="170">
         <f>H9/K14</f>
         <v>0.41804987373737373</v>
       </c>
-      <c r="H9" s="171">
+      <c r="H9" s="172">
         <f>F9*G14</f>
         <v>21.404153535353537</v>
       </c>
-      <c r="I9" s="169">
+      <c r="I9" s="170">
         <f>J9/K14</f>
         <v>0.5016598484848485</v>
       </c>
-      <c r="J9" s="171">
+      <c r="J9" s="172">
         <f>F9-D9-H9</f>
         <v>25.684984242424242</v>
       </c>
-      <c r="K9" s="169">
+      <c r="K9" s="170">
         <f>L9/K14</f>
         <v>0.6688797979797979</v>
       </c>
-      <c r="L9" s="171">
+      <c r="L9" s="172">
         <f>F9*(I14-1)</f>
         <v>34.246645656565654</v>
       </c>
-      <c r="M9" s="169">
+      <c r="M9" s="170">
         <f>N9/K14</f>
         <v>2.3410792929292925</v>
       </c>
-      <c r="N9" s="172">
+      <c r="N9" s="173">
         <f>F9*I14</f>
         <v>119.8632597979798</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="173" t="inlineStr">
+      <c r="B10" s="174" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="174">
+      <c r="C10" s="175">
         <f>C9-C7</f>
         <v>-0.12989056097075824</v>
       </c>
-      <c r="D10" s="175">
+      <c r="D10" s="176">
         <f>D9-D7</f>
         <v>-6.650396721702826</v>
       </c>
-      <c r="E10" s="174">
+      <c r="E10" s="175">
         <f>E9-E7</f>
         <v>-0.2886456910461297</v>
       </c>
-      <c r="F10" s="175">
+      <c r="F10" s="176">
         <f>F9-F7</f>
         <v>-14.778659381561837</v>
       </c>
-      <c r="G10" s="174">
+      <c r="G10" s="175">
         <f>G9-G7</f>
         <v>-0.07216142276153242</v>
       </c>
-      <c r="H10" s="175">
+      <c r="H10" s="176">
         <f>H9-H7</f>
         <v>-3.6946648453904594</v>
       </c>
-      <c r="I10" s="174">
+      <c r="I10" s="175">
         <f>I9-I7</f>
         <v>-0.08659370731383886</v>
       </c>
-      <c r="J10" s="175">
+      <c r="J10" s="176">
         <f>J9-J7</f>
         <v>-4.433597814468552</v>
       </c>
-      <c r="K10" s="174">
+      <c r="K10" s="175">
         <f>K9-K7</f>
         <v>-0.11545827641845186</v>
       </c>
-      <c r="L10" s="175">
+      <c r="L10" s="176">
         <f>L9-L7</f>
         <v>-5.911463752624734</v>
       </c>
-      <c r="M10" s="174">
+      <c r="M10" s="175">
         <f>M9-M7</f>
         <v>-0.40410396746458144</v>
       </c>
-      <c r="N10" s="175">
+      <c r="N10" s="176">
         <f>N9-N7</f>
         <v>-20.690123134186564</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="176" t="inlineStr">
+      <c r="B11" s="177" t="inlineStr">
         <is>
           <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="177" t="inlineStr">
+      <c r="B12" s="178" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 33 паллет»</t>
         </is>
       </c>
-      <c r="C12" s="178" t="n"/>
-      <c r="D12" s="178" t="n"/>
-      <c r="E12" s="178" t="n"/>
-      <c r="F12" s="178" t="n"/>
-      <c r="G12" s="178" t="n"/>
-      <c r="H12" s="178" t="n"/>
-      <c r="I12" s="178" t="n"/>
-      <c r="J12" s="178" t="n"/>
-      <c r="K12" s="178" t="n"/>
-      <c r="L12" s="178" t="n"/>
-      <c r="M12" s="178" t="n"/>
-      <c r="N12" s="178" t="n"/>
+      <c r="C12" s="179" t="n"/>
+      <c r="D12" s="179" t="n"/>
+      <c r="E12" s="179" t="n"/>
+      <c r="F12" s="179" t="n"/>
+      <c r="G12" s="179" t="n"/>
+      <c r="H12" s="179" t="n"/>
+      <c r="I12" s="179" t="n"/>
+      <c r="J12" s="179" t="n"/>
+      <c r="K12" s="179" t="n"/>
+      <c r="L12" s="179" t="n"/>
+      <c r="M12" s="179" t="n"/>
+      <c r="N12" s="179" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="C13" s="179" t="inlineStr">
+      <c r="C13" s="180" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E13" s="179" t="inlineStr">
+      <c r="E13" s="180" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G13" s="179" t="inlineStr">
+      <c r="G13" s="180" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I13" s="179" t="inlineStr">
+      <c r="I13" s="180" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K13" s="179" t="inlineStr">
+      <c r="K13" s="180" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="180" t="inlineStr">
+      <c r="B14" s="181" t="inlineStr">
         <is>
           <t>Цель расчёта и условия модели</t>
         </is>
       </c>
-      <c r="C14" s="181" t="n">
+      <c r="C14" s="182" t="n">
         <v>120</v>
       </c>
-      <c r="D14" s="182" t="n"/>
-      <c r="E14" s="183" t="n">
+      <c r="D14" s="183" t="n"/>
+      <c r="E14" s="184" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="182" t="n"/>
-      <c r="G14" s="184">
+      <c r="F14" s="183" t="n"/>
+      <c r="G14" s="185">
         <f>'Финмодель 33 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H14" s="185" t="n"/>
-      <c r="I14" s="186">
+      <c r="H14" s="186" t="n"/>
+      <c r="I14" s="187">
         <f>'Финмодель 33 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J14" s="185" t="n"/>
-      <c r="K14" s="187">
+      <c r="J14" s="186" t="n"/>
+      <c r="K14" s="188">
         <f>'Финмодель 33 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L14" s="185" t="n"/>
+      <c r="L14" s="186" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="188" t="inlineStr">
+      <c r="B15" s="189" t="inlineStr">
         <is>
           <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
         </is>
       </c>
     </row>
     <row r="16" hidden="1">
-      <c r="C16" s="179" t="inlineStr">
+      <c r="C16" s="180" t="inlineStr">
         <is>
           <t>Импортный ПДВ</t>
         </is>
       </c>
-      <c r="E16" s="179" t="inlineStr">
+      <c r="E16" s="180" t="inlineStr">
         <is>
           <t>Финансирование</t>
         </is>
       </c>
-      <c r="G16" s="179" t="inlineStr">
+      <c r="G16" s="180" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="I16" s="179" t="inlineStr">
+      <c r="I16" s="180" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="K16" s="179" t="inlineStr">
+      <c r="K16" s="180" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="M16" s="179" t="inlineStr">
+      <c r="M16" s="180" t="inlineStr">
         <is>
           <t>Прочие, €</t>
         </is>
       </c>
     </row>
     <row r="17" hidden="1">
-      <c r="C17" s="183" t="n">
+      <c r="C17" s="184" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="182" t="n"/>
-      <c r="E17" s="183" t="n">
+      <c r="D17" s="183" t="n"/>
+      <c r="E17" s="184" t="n">
         <v>0.025</v>
       </c>
-      <c r="F17" s="182" t="n"/>
-      <c r="G17" s="183" t="n">
+      <c r="F17" s="183" t="n"/>
+      <c r="G17" s="184" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="182" t="n"/>
-      <c r="I17" s="189" t="n">
+      <c r="H17" s="183" t="n"/>
+      <c r="I17" s="190" t="n">
         <v>3700</v>
       </c>
-      <c r="J17" s="182" t="n"/>
-      <c r="K17" s="189" t="n">
+      <c r="J17" s="183" t="n"/>
+      <c r="K17" s="190" t="n">
         <v>288</v>
       </c>
-      <c r="L17" s="182" t="n"/>
-      <c r="M17" s="189" t="n">
+      <c r="L17" s="183" t="n"/>
+      <c r="M17" s="190" t="n">
         <v>42</v>
       </c>
-      <c r="N17" s="182" t="n"/>
+      <c r="N17" s="183" t="n"/>
     </row>
     <row r="18" hidden="1">
-      <c r="C18" s="179" t="inlineStr">
+      <c r="C18" s="180" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="E18" s="179" t="inlineStr">
+      <c r="E18" s="180" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="G18" s="179" t="inlineStr">
+      <c r="G18" s="180" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
     <row r="19" hidden="1">
-      <c r="C19" s="190" t="n">
+      <c r="C19" s="191" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="182" t="n"/>
-      <c r="E19" s="189" t="n">
+      <c r="D19" s="183" t="n"/>
+      <c r="E19" s="190" t="n">
         <v>33</v>
       </c>
-      <c r="F19" s="182" t="n"/>
-      <c r="G19" s="189" t="n">
+      <c r="F19" s="183" t="n"/>
+      <c r="G19" s="190" t="n">
         <v>1600</v>
       </c>
-      <c r="H19" s="182" t="n"/>
+      <c r="H19" s="183" t="n"/>
     </row>
     <row r="20" hidden="1">
-      <c r="B20" s="191" t="inlineStr">
+      <c r="B20" s="192" t="inlineStr">
         <is>
           <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
         </is>
       </c>
-      <c r="C20" s="190" t="n">
+      <c r="C20" s="191" t="n">
         <v>0.65</v>
       </c>
-      <c r="E20" s="190" t="n">
+      <c r="E20" s="191" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="21" hidden="1">
-      <c r="B21" s="191" t="inlineStr">
+      <c r="B21" s="192" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
-      <c r="C21" s="192">
+      <c r="C21" s="193">
         <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
         <v>0.54</v>
       </c>
-      <c r="D21" s="193" t="n"/>
+      <c r="D21" s="194" t="n"/>
     </row>
     <row r="22" hidden="1">
-      <c r="B22" s="191" t="inlineStr">
+      <c r="B22" s="192" t="inlineStr">
         <is>
           <t>Предельная закупка до округления, €/уп.</t>
         </is>
       </c>
-      <c r="C22" s="194">
+      <c r="C22" s="195">
         <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
         <v>0.5406979199662126</v>
       </c>
-      <c r="D22" s="195" t="n"/>
+      <c r="D22" s="196" t="n"/>
     </row>
     <row r="23" hidden="1">
-      <c r="B23" s="191" t="inlineStr">
+      <c r="B23" s="192" t="inlineStr">
         <is>
           <t>Себестоимость в Украине при запросе, ₴/уп.</t>
         </is>
       </c>
-      <c r="C23" s="196">
+      <c r="C23" s="197">
         <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
         <v>38.52747636363637</v>
       </c>
-      <c r="D23" s="195" t="n"/>
+      <c r="D23" s="196" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="42">

</xml_diff>

<commit_message>
Finmodel tabs 3-4: show requested SIAS price prominently
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
+++ b/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
@@ -44,7 +44,7 @@
     <numFmt numFmtId="186" formatCode="+&quot;€&quot;0.000;-&quot;€&quot;0.000"/>
     <numFmt numFmtId="187" formatCode="+#,##0.00;-#,##0.00"/>
   </numFmts>
-  <fonts count="51">
+  <fonts count="52">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -225,6 +225,23 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00172B46"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005E6D7E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B53A3A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
@@ -258,19 +275,8 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="005E6D7E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00223A5E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00B53A3A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -459,6 +465,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE3A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="003E5A85"/>
       </patternFill>
     </fill>
@@ -474,16 +485,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE3A6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF4D2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -767,11 +773,6 @@
       </bottom>
     </border>
     <border>
-      <bottom style="medium">
-        <color rgb="00223A5E"/>
-      </bottom>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -804,6 +805,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5DCE8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5DCE8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00223A5E"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
@@ -814,7 +831,7 @@
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="198">
+  <cellXfs count="203">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1258,121 +1275,134 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="32" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="34" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="37" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="35" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="38" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="38" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="33" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="36" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="39" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="37" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="40" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="35" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="38" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="38" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="33" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="36" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="39" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="37" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="38" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="33" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="35" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="38" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="36" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="39" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="37" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="40" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="186" fontId="34" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="187" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="187" fontId="34" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="45" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="44" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="46" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="46" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="46" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="172" fontId="49" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="50" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="50" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="51" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="50" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="51" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6097,559 +6127,591 @@
       <c r="M3" s="154" t="n"/>
       <c r="N3" s="154" t="n"/>
     </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="B4" s="155" t="inlineStr">
+        <is>
+          <t>ЗАПРОС ДЛЯ SIAS, €/пачку</t>
+        </is>
+      </c>
+      <c r="C4" s="156">
+        <f>C21</f>
+        <v>0.32</v>
+      </c>
+      <c r="D4" s="157" t="n"/>
+      <c r="E4" s="158" t="str">
+        <f>"сейчас €"&amp;C20&amp;" (4 SKU) / €"&amp;E20&amp;" (2 SKU)"</f>
+        <v>сейчас €0.65 (4 SKU) / €0.75 (2 SKU)</v>
+      </c>
+      <c r="F4" s="159" t="n"/>
+      <c r="G4" s="159" t="n"/>
+      <c r="H4" s="159" t="n"/>
+      <c r="I4" s="160" t="str">
+        <f>"снижение −"&amp;ROUND((1-C21/C20)*100,0)&amp;" % / −"&amp;ROUND((1-C21/E20)*100,0)&amp;" %"</f>
+        <v>снижение −51 % / −57 %</v>
+      </c>
+      <c r="J4" s="159" t="n"/>
+      <c r="K4" s="159" t="n"/>
+      <c r="L4" s="158" t="inlineStr">
+        <is>
+          <t>одна цена для всех 6 SKU</t>
+        </is>
+      </c>
+      <c r="M4" s="159" t="n"/>
+      <c r="N4" s="159" t="n"/>
+    </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="155" t="inlineStr"/>
-      <c r="C5" s="155" t="inlineStr">
+      <c r="B5" s="161" t="inlineStr"/>
+      <c r="C5" s="161" t="inlineStr">
         <is>
           <t>Себестоимость в Украине (СС)</t>
         </is>
       </c>
-      <c r="D5" s="156" t="n"/>
-      <c r="E5" s="155" t="inlineStr">
+      <c r="D5" s="162" t="n"/>
+      <c r="E5" s="161" t="inlineStr">
         <is>
           <t>Цена партнёру (магазину)</t>
         </is>
       </c>
-      <c r="F5" s="156" t="n"/>
-      <c r="G5" s="155" t="inlineStr">
+      <c r="F5" s="162" t="n"/>
+      <c r="G5" s="161" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="H5" s="156" t="n"/>
-      <c r="I5" s="155" t="inlineStr">
+      <c r="H5" s="162" t="n"/>
+      <c r="I5" s="161" t="inlineStr">
         <is>
           <t>Наша прибыль</t>
         </is>
       </c>
-      <c r="J5" s="156" t="n"/>
-      <c r="K5" s="155" t="inlineStr">
+      <c r="J5" s="162" t="n"/>
+      <c r="K5" s="161" t="inlineStr">
         <is>
           <t>Наценка магазина</t>
         </is>
       </c>
-      <c r="L5" s="156" t="n"/>
-      <c r="M5" s="155" t="inlineStr">
+      <c r="L5" s="162" t="n"/>
+      <c r="M5" s="161" t="inlineStr">
         <is>
           <t>ПОЛКА с НДС</t>
         </is>
       </c>
-      <c r="N5" s="156" t="n"/>
+      <c r="N5" s="162" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="155" t="inlineStr">
+      <c r="B6" s="161" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="C6" s="157" t="inlineStr">
+      <c r="C6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="D6" s="157" t="inlineStr">
+      <c r="D6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="E6" s="157" t="inlineStr">
+      <c r="E6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="F6" s="157" t="inlineStr">
+      <c r="F6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="G6" s="157" t="inlineStr">
+      <c r="G6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="H6" s="157" t="inlineStr">
+      <c r="H6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="I6" s="157" t="inlineStr">
+      <c r="I6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="J6" s="157" t="inlineStr">
+      <c r="J6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="K6" s="157" t="inlineStr">
+      <c r="K6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="L6" s="157" t="inlineStr">
+      <c r="L6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="M6" s="157" t="inlineStr">
+      <c r="M6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="N6" s="157" t="inlineStr">
+      <c r="N6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="158" t="str">
+      <c r="B7" s="164" t="str">
         <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
         <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
       </c>
-      <c r="C7" s="159">
+      <c r="C7" s="165">
         <f>'Финмодель 6 паллет'!E13</f>
         <v>1.134046875</v>
       </c>
-      <c r="D7" s="160">
+      <c r="D7" s="166">
         <f>C7*K14</f>
         <v>58.063199999999995</v>
       </c>
-      <c r="E7" s="161">
+      <c r="E7" s="167">
         <f>F7/K14</f>
         <v>2.520104166666666</v>
       </c>
-      <c r="F7" s="160">
+      <c r="F7" s="166">
         <f>D7/(1-G14-E14)</f>
         <v>129.0293333333333</v>
       </c>
-      <c r="G7" s="161">
+      <c r="G7" s="167">
         <f>H7/K14</f>
         <v>0.6300260416666665</v>
       </c>
-      <c r="H7" s="162">
+      <c r="H7" s="168">
         <f>F7*G14</f>
         <v>32.25733333333333</v>
       </c>
-      <c r="I7" s="161">
+      <c r="I7" s="167">
         <f>J7/K14</f>
         <v>0.7560312499999997</v>
       </c>
-      <c r="J7" s="162">
+      <c r="J7" s="168">
         <f>F7-D7-H7</f>
         <v>38.70879999999999</v>
       </c>
-      <c r="K7" s="161">
+      <c r="K7" s="167">
         <f>L7/K14</f>
         <v>1.0080416666666663</v>
       </c>
-      <c r="L7" s="162">
+      <c r="L7" s="168">
         <f>F7*(I14-1)</f>
         <v>51.61173333333331</v>
       </c>
-      <c r="M7" s="161">
+      <c r="M7" s="167">
         <f>N7/K14</f>
         <v>3.5281458333333324</v>
       </c>
-      <c r="N7" s="163">
+      <c r="N7" s="169">
         <f>F7*I14</f>
         <v>180.64106666666663</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="164" t="str">
+      <c r="B8" s="170" t="str">
         <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
         <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
       </c>
-      <c r="C8" s="159">
+      <c r="C8" s="165">
         <f>'Финмодель 6 паллет'!E11</f>
         <v>1.308515625</v>
       </c>
-      <c r="D8" s="165">
+      <c r="D8" s="171">
         <f>C8*K14</f>
         <v>66.99600000000001</v>
       </c>
-      <c r="E8" s="166">
+      <c r="E8" s="172">
         <f>F8/K14</f>
         <v>2.9078125000000004</v>
       </c>
-      <c r="F8" s="165">
+      <c r="F8" s="171">
         <f>D8/(1-G14-E14)</f>
         <v>148.88000000000002</v>
       </c>
-      <c r="G8" s="166">
+      <c r="G8" s="172">
         <f>H8/K14</f>
         <v>0.7269531250000001</v>
       </c>
-      <c r="H8" s="167">
+      <c r="H8" s="173">
         <f>F8*G14</f>
         <v>37.220000000000006</v>
       </c>
-      <c r="I8" s="166">
+      <c r="I8" s="172">
         <f>J8/K14</f>
         <v>0.8723437500000001</v>
       </c>
-      <c r="J8" s="167">
+      <c r="J8" s="173">
         <f>F8-D8-H8</f>
         <v>44.66400000000001</v>
       </c>
-      <c r="K8" s="166">
+      <c r="K8" s="172">
         <f>L8/K14</f>
         <v>1.163125</v>
       </c>
-      <c r="L8" s="167">
+      <c r="L8" s="173">
         <f>F8*(I14-1)</f>
         <v>59.552</v>
       </c>
-      <c r="M8" s="166">
+      <c r="M8" s="172">
         <f>N8/K14</f>
         <v>4.0709375</v>
       </c>
-      <c r="N8" s="168">
+      <c r="N8" s="174">
         <f>F8*I14</f>
         <v>208.43200000000002</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="169" t="str">
+      <c r="B9" s="175" t="str">
         <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
         <v>ПОСЛЕ · запрос SIAS €0.32 (все 6 SKU)</v>
       </c>
-      <c r="C9" s="170">
+      <c r="C9" s="176">
         <f>D9/K14</f>
         <v>0.7453031249999998</v>
       </c>
-      <c r="D9" s="171">
+      <c r="D9" s="177">
         <f>C23</f>
         <v>38.15951999999999</v>
       </c>
-      <c r="E9" s="170">
+      <c r="E9" s="176">
         <f>F9/K14</f>
         <v>1.6562291666666664</v>
       </c>
-      <c r="F9" s="171">
+      <c r="F9" s="177">
         <f>D9/(1-G14-E14)</f>
         <v>84.79893333333332</v>
       </c>
-      <c r="G9" s="170">
+      <c r="G9" s="176">
         <f>H9/K14</f>
         <v>0.4140572916666666</v>
       </c>
-      <c r="H9" s="172">
+      <c r="H9" s="178">
         <f>F9*G14</f>
         <v>21.19973333333333</v>
       </c>
-      <c r="I9" s="170">
+      <c r="I9" s="176">
         <f>J9/K14</f>
         <v>0.49686874999999997</v>
       </c>
-      <c r="J9" s="172">
+      <c r="J9" s="178">
         <f>F9-D9-H9</f>
         <v>25.43968</v>
       </c>
-      <c r="K9" s="170">
+      <c r="K9" s="176">
         <f>L9/K14</f>
         <v>0.6624916666666665</v>
       </c>
-      <c r="L9" s="172">
+      <c r="L9" s="178">
         <f>F9*(I14-1)</f>
         <v>33.919573333333325</v>
       </c>
-      <c r="M9" s="170">
+      <c r="M9" s="176">
         <f>N9/K14</f>
         <v>2.318720833333333</v>
       </c>
-      <c r="N9" s="173">
+      <c r="N9" s="179">
         <f>F9*I14</f>
         <v>118.71850666666664</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="174" t="inlineStr">
+      <c r="B10" s="180" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="175">
+      <c r="C10" s="181">
         <f>C9-C7</f>
         <v>-0.38874375000000005</v>
       </c>
-      <c r="D10" s="176">
+      <c r="D10" s="182">
         <f>D9-D7</f>
         <v>-19.90368</v>
       </c>
-      <c r="E10" s="175">
+      <c r="E10" s="181">
         <f>E9-E7</f>
         <v>-0.8638749999999997</v>
       </c>
-      <c r="F10" s="176">
+      <c r="F10" s="182">
         <f>F9-F7</f>
         <v>-44.23039999999999</v>
       </c>
-      <c r="G10" s="175">
+      <c r="G10" s="181">
         <f>G9-G7</f>
         <v>-0.21596874999999993</v>
       </c>
-      <c r="H10" s="176">
+      <c r="H10" s="182">
         <f>H9-H7</f>
         <v>-11.057599999999997</v>
       </c>
-      <c r="I10" s="175">
+      <c r="I10" s="181">
         <f>I9-I7</f>
         <v>-0.25916249999999974</v>
       </c>
-      <c r="J10" s="176">
+      <c r="J10" s="182">
         <f>J9-J7</f>
         <v>-13.26911999999999</v>
       </c>
-      <c r="K10" s="175">
+      <c r="K10" s="181">
         <f>K9-K7</f>
         <v>-0.3455499999999998</v>
       </c>
-      <c r="L10" s="176">
+      <c r="L10" s="182">
         <f>L9-L7</f>
         <v>-17.692159999999987</v>
       </c>
-      <c r="M10" s="175">
+      <c r="M10" s="181">
         <f>M9-M7</f>
         <v>-1.2094249999999995</v>
       </c>
-      <c r="N10" s="176">
+      <c r="N10" s="182">
         <f>N9-N7</f>
         <v>-61.92255999999999</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="177" t="inlineStr">
+      <c r="B11" s="183" t="inlineStr">
         <is>
           <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="178" t="inlineStr">
+      <c r="B12" s="184" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 6 паллет»</t>
         </is>
       </c>
-      <c r="C12" s="179" t="n"/>
-      <c r="D12" s="179" t="n"/>
-      <c r="E12" s="179" t="n"/>
-      <c r="F12" s="179" t="n"/>
-      <c r="G12" s="179" t="n"/>
-      <c r="H12" s="179" t="n"/>
-      <c r="I12" s="179" t="n"/>
-      <c r="J12" s="179" t="n"/>
-      <c r="K12" s="179" t="n"/>
-      <c r="L12" s="179" t="n"/>
-      <c r="M12" s="179" t="n"/>
-      <c r="N12" s="179" t="n"/>
+      <c r="C12" s="185" t="n"/>
+      <c r="D12" s="185" t="n"/>
+      <c r="E12" s="185" t="n"/>
+      <c r="F12" s="185" t="n"/>
+      <c r="G12" s="185" t="n"/>
+      <c r="H12" s="185" t="n"/>
+      <c r="I12" s="185" t="n"/>
+      <c r="J12" s="185" t="n"/>
+      <c r="K12" s="185" t="n"/>
+      <c r="L12" s="185" t="n"/>
+      <c r="M12" s="185" t="n"/>
+      <c r="N12" s="185" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="C13" s="180" t="inlineStr">
+      <c r="C13" s="186" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E13" s="180" t="inlineStr">
+      <c r="E13" s="186" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G13" s="180" t="inlineStr">
+      <c r="G13" s="186" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I13" s="180" t="inlineStr">
+      <c r="I13" s="186" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K13" s="180" t="inlineStr">
+      <c r="K13" s="186" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="181" t="inlineStr">
+      <c r="B14" s="187" t="inlineStr">
         <is>
           <t>Цель расчёта и условия модели</t>
         </is>
       </c>
-      <c r="C14" s="182" t="n">
+      <c r="C14" s="188" t="n">
         <v>120</v>
       </c>
-      <c r="D14" s="183" t="n"/>
-      <c r="E14" s="184" t="n">
+      <c r="D14" s="189" t="n"/>
+      <c r="E14" s="190" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="183" t="n"/>
-      <c r="G14" s="185">
+      <c r="F14" s="189" t="n"/>
+      <c r="G14" s="191">
         <f>'Финмодель 6 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H14" s="186" t="n"/>
-      <c r="I14" s="187">
+      <c r="H14" s="192" t="n"/>
+      <c r="I14" s="193">
         <f>'Финмодель 6 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J14" s="186" t="n"/>
-      <c r="K14" s="188">
+      <c r="J14" s="192" t="n"/>
+      <c r="K14" s="194">
         <f>'Финмодель 6 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L14" s="186" t="n"/>
+      <c r="L14" s="192" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="189" t="inlineStr">
+      <c r="B15" s="195" t="inlineStr">
         <is>
           <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
         </is>
       </c>
     </row>
     <row r="16" hidden="1">
-      <c r="C16" s="180" t="inlineStr">
+      <c r="C16" s="186" t="inlineStr">
         <is>
           <t>Импортный ПДВ</t>
         </is>
       </c>
-      <c r="E16" s="180" t="inlineStr">
+      <c r="E16" s="186" t="inlineStr">
         <is>
           <t>Финансирование</t>
         </is>
       </c>
-      <c r="G16" s="180" t="inlineStr">
+      <c r="G16" s="186" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="I16" s="180" t="inlineStr">
+      <c r="I16" s="186" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="K16" s="180" t="inlineStr">
+      <c r="K16" s="186" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="M16" s="180" t="inlineStr">
+      <c r="M16" s="186" t="inlineStr">
         <is>
           <t>Прочие, €</t>
         </is>
       </c>
     </row>
     <row r="17" hidden="1">
-      <c r="C17" s="184" t="n">
+      <c r="C17" s="190" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="183" t="n"/>
-      <c r="E17" s="184" t="n">
+      <c r="D17" s="189" t="n"/>
+      <c r="E17" s="190" t="n">
         <v>0.025</v>
       </c>
-      <c r="F17" s="183" t="n"/>
-      <c r="G17" s="184" t="n">
+      <c r="F17" s="189" t="n"/>
+      <c r="G17" s="190" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="183" t="n"/>
-      <c r="I17" s="190" t="n">
+      <c r="H17" s="189" t="n"/>
+      <c r="I17" s="196" t="n">
         <v>2600</v>
       </c>
-      <c r="J17" s="183" t="n"/>
-      <c r="K17" s="190" t="n">
+      <c r="J17" s="189" t="n"/>
+      <c r="K17" s="196" t="n">
         <v>288</v>
       </c>
-      <c r="L17" s="183" t="n"/>
-      <c r="M17" s="190" t="n">
+      <c r="L17" s="189" t="n"/>
+      <c r="M17" s="196" t="n">
         <v>42</v>
       </c>
-      <c r="N17" s="183" t="n"/>
+      <c r="N17" s="189" t="n"/>
     </row>
     <row r="18" hidden="1">
-      <c r="C18" s="180" t="inlineStr">
+      <c r="C18" s="186" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="E18" s="180" t="inlineStr">
+      <c r="E18" s="186" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="G18" s="180" t="inlineStr">
+      <c r="G18" s="186" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
     <row r="19" hidden="1">
-      <c r="C19" s="191" t="n">
+      <c r="C19" s="197" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="183" t="n"/>
-      <c r="E19" s="190" t="n">
+      <c r="D19" s="189" t="n"/>
+      <c r="E19" s="196" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="183" t="n"/>
-      <c r="G19" s="190" t="n">
+      <c r="F19" s="189" t="n"/>
+      <c r="G19" s="196" t="n">
         <v>1600</v>
       </c>
-      <c r="H19" s="183" t="n"/>
+      <c r="H19" s="189" t="n"/>
     </row>
     <row r="20" hidden="1">
-      <c r="B20" s="192" t="inlineStr">
+      <c r="B20" s="198" t="inlineStr">
         <is>
           <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
         </is>
       </c>
-      <c r="C20" s="191" t="n">
+      <c r="C20" s="197" t="n">
         <v>0.65</v>
       </c>
-      <c r="E20" s="191" t="n">
+      <c r="E20" s="197" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="21" hidden="1">
-      <c r="B21" s="192" t="inlineStr">
+      <c r="B21" s="198" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
-      <c r="C21" s="193">
+      <c r="C21" s="199">
         <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
         <v>0.32</v>
       </c>
-      <c r="D21" s="194" t="n"/>
+      <c r="D21" s="157" t="n"/>
     </row>
     <row r="22" hidden="1">
-      <c r="B22" s="192" t="inlineStr">
+      <c r="B22" s="198" t="inlineStr">
         <is>
           <t>Предельная закупка до округления, €/уп.</t>
         </is>
       </c>
-      <c r="C22" s="195">
+      <c r="C22" s="200">
         <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
         <v>0.3265407229965157</v>
       </c>
-      <c r="D22" s="196" t="n"/>
+      <c r="D22" s="201" t="n"/>
     </row>
     <row r="23" hidden="1">
-      <c r="B23" s="192" t="inlineStr">
+      <c r="B23" s="198" t="inlineStr">
         <is>
           <t>Себестоимость в Украине при запросе, ₴/уп.</t>
         </is>
       </c>
-      <c r="C23" s="197">
+      <c r="C23" s="202">
         <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
         <v>38.15951999999999</v>
       </c>
-      <c r="D23" s="196" t="n"/>
+      <c r="D23" s="201" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="46">
     <mergeCell ref="K16:L16"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
@@ -6658,19 +6720,23 @@
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L4:N4"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:H17"/>
+    <mergeCell ref="C4:D4"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="I4:K4"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="M16:N16"/>
     <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E4:H4"/>
     <mergeCell ref="B12:N12"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="I5:J5"/>
@@ -6751,559 +6817,591 @@
       <c r="M3" s="154" t="n"/>
       <c r="N3" s="154" t="n"/>
     </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="B4" s="155" t="inlineStr">
+        <is>
+          <t>ЗАПРОС ДЛЯ SIAS, €/пачку</t>
+        </is>
+      </c>
+      <c r="C4" s="156">
+        <f>C21</f>
+        <v>0.54</v>
+      </c>
+      <c r="D4" s="157" t="n"/>
+      <c r="E4" s="158" t="str">
+        <f>"сейчас €"&amp;C20&amp;" (4 SKU) / €"&amp;E20&amp;" (2 SKU)"</f>
+        <v>сейчас €0.65 (4 SKU) / €0.75 (2 SKU)</v>
+      </c>
+      <c r="F4" s="159" t="n"/>
+      <c r="G4" s="159" t="n"/>
+      <c r="H4" s="159" t="n"/>
+      <c r="I4" s="160" t="str">
+        <f>"снижение −"&amp;ROUND((1-C21/C20)*100,0)&amp;" % / −"&amp;ROUND((1-C21/E20)*100,0)&amp;" %"</f>
+        <v>снижение −17 % / −28 %</v>
+      </c>
+      <c r="J4" s="159" t="n"/>
+      <c r="K4" s="159" t="n"/>
+      <c r="L4" s="158" t="inlineStr">
+        <is>
+          <t>одна цена для всех 6 SKU</t>
+        </is>
+      </c>
+      <c r="M4" s="159" t="n"/>
+      <c r="N4" s="159" t="n"/>
+    </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="155" t="inlineStr"/>
-      <c r="C5" s="155" t="inlineStr">
+      <c r="B5" s="161" t="inlineStr"/>
+      <c r="C5" s="161" t="inlineStr">
         <is>
           <t>Себестоимость в Украине (СС)</t>
         </is>
       </c>
-      <c r="D5" s="156" t="n"/>
-      <c r="E5" s="155" t="inlineStr">
+      <c r="D5" s="162" t="n"/>
+      <c r="E5" s="161" t="inlineStr">
         <is>
           <t>Цена партнёру (магазину)</t>
         </is>
       </c>
-      <c r="F5" s="156" t="n"/>
-      <c r="G5" s="155" t="inlineStr">
+      <c r="F5" s="162" t="n"/>
+      <c r="G5" s="161" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="H5" s="156" t="n"/>
-      <c r="I5" s="155" t="inlineStr">
+      <c r="H5" s="162" t="n"/>
+      <c r="I5" s="161" t="inlineStr">
         <is>
           <t>Наша прибыль</t>
         </is>
       </c>
-      <c r="J5" s="156" t="n"/>
-      <c r="K5" s="155" t="inlineStr">
+      <c r="J5" s="162" t="n"/>
+      <c r="K5" s="161" t="inlineStr">
         <is>
           <t>Наценка магазина</t>
         </is>
       </c>
-      <c r="L5" s="156" t="n"/>
-      <c r="M5" s="155" t="inlineStr">
+      <c r="L5" s="162" t="n"/>
+      <c r="M5" s="161" t="inlineStr">
         <is>
           <t>ПОЛКА с НДС</t>
         </is>
       </c>
-      <c r="N5" s="156" t="n"/>
+      <c r="N5" s="162" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="155" t="inlineStr">
+      <c r="B6" s="161" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="C6" s="157" t="inlineStr">
+      <c r="C6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="D6" s="157" t="inlineStr">
+      <c r="D6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="E6" s="157" t="inlineStr">
+      <c r="E6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="F6" s="157" t="inlineStr">
+      <c r="F6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="G6" s="157" t="inlineStr">
+      <c r="G6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="H6" s="157" t="inlineStr">
+      <c r="H6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="I6" s="157" t="inlineStr">
+      <c r="I6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="J6" s="157" t="inlineStr">
+      <c r="J6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="K6" s="157" t="inlineStr">
+      <c r="K6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="L6" s="157" t="inlineStr">
+      <c r="L6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
-      <c r="M6" s="157" t="inlineStr">
+      <c r="M6" s="163" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="N6" s="157" t="inlineStr">
+      <c r="N6" s="163" t="inlineStr">
         <is>
           <t>₴</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="158" t="str">
+      <c r="B7" s="164" t="str">
         <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
         <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
       </c>
-      <c r="C7" s="159">
+      <c r="C7" s="165">
         <f>'Финмодель 33 паллет'!E13</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="D7" s="160">
+      <c r="D7" s="166">
         <f>C7*K14</f>
         <v>45.17787308533919</v>
       </c>
-      <c r="E7" s="161">
+      <c r="E7" s="167">
         <f>F7/K14</f>
         <v>1.9608451859956246</v>
       </c>
-      <c r="F7" s="160">
+      <c r="F7" s="166">
         <f>D7/(1-G14-E14)</f>
         <v>100.39527352297598</v>
       </c>
-      <c r="G7" s="161">
+      <c r="G7" s="167">
         <f>H7/K14</f>
         <v>0.49021129649890616</v>
       </c>
-      <c r="H7" s="162">
+      <c r="H7" s="168">
         <f>F7*G14</f>
         <v>25.098818380743996</v>
       </c>
-      <c r="I7" s="161">
+      <c r="I7" s="167">
         <f>J7/K14</f>
         <v>0.5882535557986873</v>
       </c>
-      <c r="J7" s="162">
+      <c r="J7" s="168">
         <f>F7-D7-H7</f>
         <v>30.118582056892794</v>
       </c>
-      <c r="K7" s="161">
+      <c r="K7" s="167">
         <f>L7/K14</f>
         <v>0.7843380743982498</v>
       </c>
-      <c r="L7" s="162">
+      <c r="L7" s="168">
         <f>F7*(I14-1)</f>
         <v>40.15810940919039</v>
       </c>
-      <c r="M7" s="161">
+      <c r="M7" s="167">
         <f>N7/K14</f>
         <v>2.745183260393874</v>
       </c>
-      <c r="N7" s="163">
+      <c r="N7" s="169">
         <f>F7*I14</f>
         <v>140.55338293216636</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="164" t="str">
+      <c r="B8" s="170" t="str">
         <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
         <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
       </c>
-      <c r="C8" s="159">
+      <c r="C8" s="165">
         <f>'Финмодель 33 паллет'!E11</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="D8" s="165">
+      <c r="D8" s="171">
         <f>C8*K14</f>
         <v>52.12831509846825</v>
       </c>
-      <c r="E8" s="166">
+      <c r="E8" s="172">
         <f>F8/K14</f>
         <v>2.2625136761487954</v>
       </c>
-      <c r="F8" s="165">
+      <c r="F8" s="171">
         <f>D8/(1-G14-E14)</f>
         <v>115.84070021881833</v>
       </c>
-      <c r="G8" s="166">
+      <c r="G8" s="172">
         <f>H8/K14</f>
         <v>0.5656284190371988</v>
       </c>
-      <c r="H8" s="167">
+      <c r="H8" s="173">
         <f>F8*G14</f>
         <v>28.96017505470458</v>
       </c>
-      <c r="I8" s="166">
+      <c r="I8" s="172">
         <f>J8/K14</f>
         <v>0.6787541028446387</v>
       </c>
-      <c r="J8" s="167">
+      <c r="J8" s="173">
         <f>F8-D8-H8</f>
         <v>34.7522100656455</v>
       </c>
-      <c r="K8" s="166">
+      <c r="K8" s="172">
         <f>L8/K14</f>
         <v>0.905005470459518</v>
       </c>
-      <c r="L8" s="167">
+      <c r="L8" s="173">
         <f>F8*(I14-1)</f>
         <v>46.33628008752732</v>
       </c>
-      <c r="M8" s="166">
+      <c r="M8" s="172">
         <f>N8/K14</f>
         <v>3.1675191466083135</v>
       </c>
-      <c r="N8" s="168">
+      <c r="N8" s="174">
         <f>F8*I14</f>
         <v>162.17698030634565</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="169" t="str">
+      <c r="B9" s="175" t="str">
         <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
         <v>ПОСЛЕ · запрос SIAS €0.54 (все 6 SKU)</v>
       </c>
-      <c r="C9" s="170">
+      <c r="C9" s="176">
         <f>D9/K14</f>
         <v>0.7524897727272728</v>
       </c>
-      <c r="D9" s="171">
+      <c r="D9" s="177">
         <f>C23</f>
         <v>38.52747636363637</v>
       </c>
-      <c r="E9" s="170">
+      <c r="E9" s="176">
         <f>F9/K14</f>
         <v>1.672199494949495</v>
       </c>
-      <c r="F9" s="171">
+      <c r="F9" s="177">
         <f>D9/(1-G14-E14)</f>
         <v>85.61661414141415</v>
       </c>
-      <c r="G9" s="170">
+      <c r="G9" s="176">
         <f>H9/K14</f>
         <v>0.41804987373737373</v>
       </c>
-      <c r="H9" s="172">
+      <c r="H9" s="178">
         <f>F9*G14</f>
         <v>21.404153535353537</v>
       </c>
-      <c r="I9" s="170">
+      <c r="I9" s="176">
         <f>J9/K14</f>
         <v>0.5016598484848485</v>
       </c>
-      <c r="J9" s="172">
+      <c r="J9" s="178">
         <f>F9-D9-H9</f>
         <v>25.684984242424242</v>
       </c>
-      <c r="K9" s="170">
+      <c r="K9" s="176">
         <f>L9/K14</f>
         <v>0.6688797979797979</v>
       </c>
-      <c r="L9" s="172">
+      <c r="L9" s="178">
         <f>F9*(I14-1)</f>
         <v>34.246645656565654</v>
       </c>
-      <c r="M9" s="170">
+      <c r="M9" s="176">
         <f>N9/K14</f>
         <v>2.3410792929292925</v>
       </c>
-      <c r="N9" s="173">
+      <c r="N9" s="179">
         <f>F9*I14</f>
         <v>119.8632597979798</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="174" t="inlineStr">
+      <c r="B10" s="180" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="175">
+      <c r="C10" s="181">
         <f>C9-C7</f>
         <v>-0.12989056097075824</v>
       </c>
-      <c r="D10" s="176">
+      <c r="D10" s="182">
         <f>D9-D7</f>
         <v>-6.650396721702826</v>
       </c>
-      <c r="E10" s="175">
+      <c r="E10" s="181">
         <f>E9-E7</f>
         <v>-0.2886456910461297</v>
       </c>
-      <c r="F10" s="176">
+      <c r="F10" s="182">
         <f>F9-F7</f>
         <v>-14.778659381561837</v>
       </c>
-      <c r="G10" s="175">
+      <c r="G10" s="181">
         <f>G9-G7</f>
         <v>-0.07216142276153242</v>
       </c>
-      <c r="H10" s="176">
+      <c r="H10" s="182">
         <f>H9-H7</f>
         <v>-3.6946648453904594</v>
       </c>
-      <c r="I10" s="175">
+      <c r="I10" s="181">
         <f>I9-I7</f>
         <v>-0.08659370731383886</v>
       </c>
-      <c r="J10" s="176">
+      <c r="J10" s="182">
         <f>J9-J7</f>
         <v>-4.433597814468552</v>
       </c>
-      <c r="K10" s="175">
+      <c r="K10" s="181">
         <f>K9-K7</f>
         <v>-0.11545827641845186</v>
       </c>
-      <c r="L10" s="176">
+      <c r="L10" s="182">
         <f>L9-L7</f>
         <v>-5.911463752624734</v>
       </c>
-      <c r="M10" s="175">
+      <c r="M10" s="181">
         <f>M9-M7</f>
         <v>-0.40410396746458144</v>
       </c>
-      <c r="N10" s="176">
+      <c r="N10" s="182">
         <f>N9-N7</f>
         <v>-20.690123134186564</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="177" t="inlineStr">
+      <c r="B11" s="183" t="inlineStr">
         <is>
           <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="178" t="inlineStr">
+      <c r="B12" s="184" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 33 паллет»</t>
         </is>
       </c>
-      <c r="C12" s="179" t="n"/>
-      <c r="D12" s="179" t="n"/>
-      <c r="E12" s="179" t="n"/>
-      <c r="F12" s="179" t="n"/>
-      <c r="G12" s="179" t="n"/>
-      <c r="H12" s="179" t="n"/>
-      <c r="I12" s="179" t="n"/>
-      <c r="J12" s="179" t="n"/>
-      <c r="K12" s="179" t="n"/>
-      <c r="L12" s="179" t="n"/>
-      <c r="M12" s="179" t="n"/>
-      <c r="N12" s="179" t="n"/>
+      <c r="C12" s="185" t="n"/>
+      <c r="D12" s="185" t="n"/>
+      <c r="E12" s="185" t="n"/>
+      <c r="F12" s="185" t="n"/>
+      <c r="G12" s="185" t="n"/>
+      <c r="H12" s="185" t="n"/>
+      <c r="I12" s="185" t="n"/>
+      <c r="J12" s="185" t="n"/>
+      <c r="K12" s="185" t="n"/>
+      <c r="L12" s="185" t="n"/>
+      <c r="M12" s="185" t="n"/>
+      <c r="N12" s="185" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="C13" s="180" t="inlineStr">
+      <c r="C13" s="186" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E13" s="180" t="inlineStr">
+      <c r="E13" s="186" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G13" s="180" t="inlineStr">
+      <c r="G13" s="186" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I13" s="180" t="inlineStr">
+      <c r="I13" s="186" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K13" s="180" t="inlineStr">
+      <c r="K13" s="186" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="181" t="inlineStr">
+      <c r="B14" s="187" t="inlineStr">
         <is>
           <t>Цель расчёта и условия модели</t>
         </is>
       </c>
-      <c r="C14" s="182" t="n">
+      <c r="C14" s="188" t="n">
         <v>120</v>
       </c>
-      <c r="D14" s="183" t="n"/>
-      <c r="E14" s="184" t="n">
+      <c r="D14" s="189" t="n"/>
+      <c r="E14" s="190" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="183" t="n"/>
-      <c r="G14" s="185">
+      <c r="F14" s="189" t="n"/>
+      <c r="G14" s="191">
         <f>'Финмодель 33 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H14" s="186" t="n"/>
-      <c r="I14" s="187">
+      <c r="H14" s="192" t="n"/>
+      <c r="I14" s="193">
         <f>'Финмодель 33 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J14" s="186" t="n"/>
-      <c r="K14" s="188">
+      <c r="J14" s="192" t="n"/>
+      <c r="K14" s="194">
         <f>'Финмодель 33 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L14" s="186" t="n"/>
+      <c r="L14" s="192" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="189" t="inlineStr">
+      <c r="B15" s="195" t="inlineStr">
         <is>
           <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
         </is>
       </c>
     </row>
     <row r="16" hidden="1">
-      <c r="C16" s="180" t="inlineStr">
+      <c r="C16" s="186" t="inlineStr">
         <is>
           <t>Импортный ПДВ</t>
         </is>
       </c>
-      <c r="E16" s="180" t="inlineStr">
+      <c r="E16" s="186" t="inlineStr">
         <is>
           <t>Финансирование</t>
         </is>
       </c>
-      <c r="G16" s="180" t="inlineStr">
+      <c r="G16" s="186" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="I16" s="180" t="inlineStr">
+      <c r="I16" s="186" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="K16" s="180" t="inlineStr">
+      <c r="K16" s="186" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="M16" s="180" t="inlineStr">
+      <c r="M16" s="186" t="inlineStr">
         <is>
           <t>Прочие, €</t>
         </is>
       </c>
     </row>
     <row r="17" hidden="1">
-      <c r="C17" s="184" t="n">
+      <c r="C17" s="190" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="183" t="n"/>
-      <c r="E17" s="184" t="n">
+      <c r="D17" s="189" t="n"/>
+      <c r="E17" s="190" t="n">
         <v>0.025</v>
       </c>
-      <c r="F17" s="183" t="n"/>
-      <c r="G17" s="184" t="n">
+      <c r="F17" s="189" t="n"/>
+      <c r="G17" s="190" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="183" t="n"/>
-      <c r="I17" s="190" t="n">
+      <c r="H17" s="189" t="n"/>
+      <c r="I17" s="196" t="n">
         <v>3700</v>
       </c>
-      <c r="J17" s="183" t="n"/>
-      <c r="K17" s="190" t="n">
+      <c r="J17" s="189" t="n"/>
+      <c r="K17" s="196" t="n">
         <v>288</v>
       </c>
-      <c r="L17" s="183" t="n"/>
-      <c r="M17" s="190" t="n">
+      <c r="L17" s="189" t="n"/>
+      <c r="M17" s="196" t="n">
         <v>42</v>
       </c>
-      <c r="N17" s="183" t="n"/>
+      <c r="N17" s="189" t="n"/>
     </row>
     <row r="18" hidden="1">
-      <c r="C18" s="180" t="inlineStr">
+      <c r="C18" s="186" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="E18" s="180" t="inlineStr">
+      <c r="E18" s="186" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="G18" s="180" t="inlineStr">
+      <c r="G18" s="186" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
     <row r="19" hidden="1">
-      <c r="C19" s="191" t="n">
+      <c r="C19" s="197" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="183" t="n"/>
-      <c r="E19" s="190" t="n">
+      <c r="D19" s="189" t="n"/>
+      <c r="E19" s="196" t="n">
         <v>33</v>
       </c>
-      <c r="F19" s="183" t="n"/>
-      <c r="G19" s="190" t="n">
+      <c r="F19" s="189" t="n"/>
+      <c r="G19" s="196" t="n">
         <v>1600</v>
       </c>
-      <c r="H19" s="183" t="n"/>
+      <c r="H19" s="189" t="n"/>
     </row>
     <row r="20" hidden="1">
-      <c r="B20" s="192" t="inlineStr">
+      <c r="B20" s="198" t="inlineStr">
         <is>
           <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
         </is>
       </c>
-      <c r="C20" s="191" t="n">
+      <c r="C20" s="197" t="n">
         <v>0.65</v>
       </c>
-      <c r="E20" s="191" t="n">
+      <c r="E20" s="197" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="21" hidden="1">
-      <c r="B21" s="192" t="inlineStr">
+      <c r="B21" s="198" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
-      <c r="C21" s="193">
+      <c r="C21" s="199">
         <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
         <v>0.54</v>
       </c>
-      <c r="D21" s="194" t="n"/>
+      <c r="D21" s="157" t="n"/>
     </row>
     <row r="22" hidden="1">
-      <c r="B22" s="192" t="inlineStr">
+      <c r="B22" s="198" t="inlineStr">
         <is>
           <t>Предельная закупка до округления, €/уп.</t>
         </is>
       </c>
-      <c r="C22" s="195">
+      <c r="C22" s="200">
         <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
         <v>0.5406979199662126</v>
       </c>
-      <c r="D22" s="196" t="n"/>
+      <c r="D22" s="201" t="n"/>
     </row>
     <row r="23" hidden="1">
-      <c r="B23" s="192" t="inlineStr">
+      <c r="B23" s="198" t="inlineStr">
         <is>
           <t>Себестоимость в Украине при запросе, ₴/уп.</t>
         </is>
       </c>
-      <c r="C23" s="197">
+      <c r="C23" s="202">
         <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
         <v>38.52747636363637</v>
       </c>
-      <c r="D23" s="196" t="n"/>
+      <c r="D23" s="201" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="46">
     <mergeCell ref="K16:L16"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
@@ -7312,19 +7410,23 @@
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L4:N4"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:H17"/>
+    <mergeCell ref="C4:D4"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="I4:K4"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="M16:N16"/>
     <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E4:H4"/>
     <mergeCell ref="B12:N12"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="I5:J5"/>

</xml_diff>

<commit_message>
Excel tabs 3-4: one-line model from SIAS purchase price; sync final deck slides
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
+++ b/RAMEN_FINMODEL_4_TABS_PRESENTATION_READABLE.xlsx
@@ -41,10 +41,10 @@
     <numFmt numFmtId="183" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
     <numFmt numFmtId="184" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
     <numFmt numFmtId="185" formatCode="&quot;€&quot;0.000"/>
-    <numFmt numFmtId="186" formatCode="+&quot;€&quot;0.000;-&quot;€&quot;0.000"/>
-    <numFmt numFmtId="187" formatCode="+#,##0.00;-#,##0.00"/>
+    <numFmt numFmtId="186" formatCode="+#,##0.00&quot; ₴&quot;;-#,##0.00&quot; ₴&quot;"/>
+    <numFmt numFmtId="187" formatCode="+&quot;€&quot;0.000;-&quot;€&quot;0.000"/>
   </numFmts>
-  <fonts count="52">
+  <fonts count="54">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -253,19 +253,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00008000"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00172B46"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00172B46"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -275,9 +265,36 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00172B46"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00172B46"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00223A5E"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B53A3A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005E6D7E"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -323,11 +340,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="005E6D7E"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00172B46"/>
       <sz val="11"/>
@@ -338,7 +350,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="31">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -475,11 +487,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="005A74A0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F2F5F9"/>
       </patternFill>
     </fill>
@@ -489,7 +496,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -806,11 +813,33 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="00D5DCE8"/>
+      </left>
       <right/>
-      <top style="thin">
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="00D5DCE8"/>
-      </top>
+      </left>
+      <right style="thin">
+        <color rgb="00D5DCE8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D5DCE8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D5DCE8"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color rgb="00D5DCE8"/>
       </bottom>
@@ -831,7 +860,7 @@
     <xf numFmtId="0" fontId="12" fillId="19" borderId="11"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="203">
+  <cellXfs count="202">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1292,117 +1321,118 @@
     <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="38" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="171" fontId="40" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="41" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="185" fontId="37" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="38" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="39" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="33" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="39" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="40" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="33" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="38" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="38" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="171" fontId="40" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="185" fontId="33" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="39" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="38" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="40" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="40" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="171" fontId="41" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="36" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="185" fontId="33" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="38" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="186" fontId="43" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="39" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="187" fontId="44" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="40" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="34" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="48" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="187" fontId="34" fillId="25" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="48" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="49" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="49" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="49" fillId="28" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="48" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="48" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="52" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="53" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="46" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="46" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="46" fillId="29" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="45" fillId="30" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="50" fillId="26" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="51" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="51" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="53" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6081,38 +6111,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N23"/>
+  <dimension ref="B2:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="2" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="152" t="inlineStr">
         <is>
-          <t>SIAS · было → стало · от себестоимости в Украине до полки · 6 паллет</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>SIAS · от цены закупки до полки одной линией · 6 паллет</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="B3" s="153" t="str">
-        <f>"Полка "&amp;ROUND(C14,0)&amp;" ₴ достижима при себестоимости "&amp;ROUND(D9,2)&amp;" ₴ (сейчас "&amp;ROUND(D7,2)&amp;"–"&amp;ROUND(D8,2)&amp;" ₴). Для этого закупка SIAS должна быть €"&amp;ROUND(C21,2)&amp;" вместо €"&amp;MIN(C20,E20)&amp;"–€"&amp;MAX(C20,E20)&amp;" (−"&amp;ROUND((1-C21/MIN(C20,E20))*100,0)&amp;"…"&amp;ROUND((1-C21/MAX(C20,E20))*100,0)&amp;"%)."</f>
-        <v>Полка 120 ₴ достижима при себестоимости 38.16 ₴ (сейчас 58.06–67 ₴). Для этого закупка SIAS должна быть €0.32 вместо €0.65–€0.75 (−51…57%).</v>
+        <f>"Цена закупки SIAS €"&amp;ROUND(C26,2)&amp;" вместо €"&amp;MIN(C8,C10)&amp;"–€"&amp;MAX(C8,C10)&amp;" (−"&amp;ROUND((1-C26/MIN(C8,C10))*100,0)&amp;"…"&amp;ROUND((1-C26/MAX(C8,C10))*100,0)&amp;"%) → полка "&amp;ROUND(I11,2)&amp;" ₴ при марже "&amp;ROUND(D18*100,0)&amp;"%."</f>
+        <v>Цена закупки SIAS €0.32 вместо €0.65–€0.75 (−51…57%) → полка 118.72 ₴ при марже 30%.</v>
       </c>
       <c r="C3" s="154" t="n"/>
       <c r="D3" s="154" t="n"/>
@@ -6121,11 +6146,6 @@
       <c r="G3" s="154" t="n"/>
       <c r="H3" s="154" t="n"/>
       <c r="I3" s="154" t="n"/>
-      <c r="J3" s="154" t="n"/>
-      <c r="K3" s="154" t="n"/>
-      <c r="L3" s="154" t="n"/>
-      <c r="M3" s="154" t="n"/>
-      <c r="N3" s="154" t="n"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="B4" s="155" t="inlineStr">
@@ -6134,630 +6154,548 @@
         </is>
       </c>
       <c r="C4" s="156">
-        <f>C21</f>
+        <f>C26</f>
         <v>0.32</v>
       </c>
       <c r="D4" s="157" t="n"/>
       <c r="E4" s="158" t="str">
-        <f>"сейчас €"&amp;C20&amp;" (4 SKU) / €"&amp;E20&amp;" (2 SKU)"</f>
+        <f>"сейчас €"&amp;C8&amp;" (4 SKU) / €"&amp;C10&amp;" (2 SKU)"</f>
         <v>сейчас €0.65 (4 SKU) / €0.75 (2 SKU)</v>
       </c>
       <c r="F4" s="159" t="n"/>
-      <c r="G4" s="159" t="n"/>
+      <c r="G4" s="160" t="str">
+        <f>"снижение −"&amp;ROUND((1-C26/C8)*100,0)&amp;" % / −"&amp;ROUND((1-C26/C10)*100,0)&amp;" %"</f>
+        <v>снижение −51 % / −57 %</v>
+      </c>
       <c r="H4" s="159" t="n"/>
-      <c r="I4" s="160" t="str">
-        <f>"снижение −"&amp;ROUND((1-C21/C20)*100,0)&amp;" % / −"&amp;ROUND((1-C21/E20)*100,0)&amp;" %"</f>
-        <v>снижение −51 % / −57 %</v>
-      </c>
-      <c r="J4" s="159" t="n"/>
-      <c r="K4" s="159" t="n"/>
-      <c r="L4" s="158" t="inlineStr">
-        <is>
-          <t>одна цена для всех 6 SKU</t>
-        </is>
-      </c>
-      <c r="M4" s="159" t="n"/>
-      <c r="N4" s="159" t="n"/>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="161" t="inlineStr"/>
+      <c r="I4" s="158" t="inlineStr">
+        <is>
+          <t>одна цена на 6 SKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="B5" s="161" t="inlineStr">
+        <is>
+          <t>Вариант</t>
+        </is>
+      </c>
       <c r="C5" s="161" t="inlineStr">
         <is>
-          <t>Себестоимость в Украине (СС)</t>
-        </is>
-      </c>
-      <c r="D5" s="162" t="n"/>
+          <t>Закупка SIAS
+за пачку</t>
+        </is>
+      </c>
+      <c r="D5" s="161" t="inlineStr">
+        <is>
+          <t>Себестоимость в Украине
+товар + расходы в Украине</t>
+        </is>
+      </c>
       <c r="E5" s="161" t="inlineStr">
         <is>
-          <t>Цена партнёру (магазину)</t>
-        </is>
-      </c>
-      <c r="F5" s="162" t="n"/>
+          <t>Цена партнёру
+СС ÷ (1 − бонус − маржа)</t>
+        </is>
+      </c>
+      <c r="F5" s="161" t="inlineStr">
+        <is>
+          <t>Бонус сети
+25 % цены партнёру</t>
+        </is>
+      </c>
       <c r="G5" s="161" t="inlineStr">
         <is>
-          <t>Бонус сети</t>
-        </is>
-      </c>
-      <c r="H5" s="162" t="n"/>
+          <t>Наша прибыль
+30 % цены партнёру</t>
+        </is>
+      </c>
+      <c r="H5" s="161" t="inlineStr">
+        <is>
+          <t>Наценка магазина
++40 % к цене партнёру</t>
+        </is>
+      </c>
       <c r="I5" s="161" t="inlineStr">
         <is>
-          <t>Наша прибыль</t>
-        </is>
-      </c>
-      <c r="J5" s="162" t="n"/>
-      <c r="K5" s="161" t="inlineStr">
-        <is>
-          <t>Наценка магазина</t>
-        </is>
-      </c>
-      <c r="L5" s="162" t="n"/>
-      <c r="M5" s="161" t="inlineStr">
-        <is>
-          <t>ПОЛКА с НДС</t>
-        </is>
-      </c>
-      <c r="N5" s="162" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="161" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="C6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="D6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="E6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="F6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="G6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="H6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="I6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="J6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="K6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="L6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="M6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="N6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="164" t="str">
-        <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
-        <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
-      </c>
-      <c r="C7" s="165">
+          <t>ПОЛКА с НДС
+цена партнёру × 1,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="B7" s="162" t="inlineStr">
+        <is>
+          <t>ДО · Vegetable, Spicy, Beef, Chicken
+(4 SKU)</t>
+        </is>
+      </c>
+      <c r="C7" s="163">
+        <f>C8*G18</f>
+        <v>33.28</v>
+      </c>
+      <c r="D7" s="163">
+        <f>D8*G18</f>
+        <v>58.063199999999995</v>
+      </c>
+      <c r="E7" s="163">
+        <f>D7/(1-E18-D18)</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="F7" s="164">
+        <f>E7*E18</f>
+        <v>32.25733333333333</v>
+      </c>
+      <c r="G7" s="164">
+        <f>E7-D7-F7</f>
+        <v>38.70879999999999</v>
+      </c>
+      <c r="H7" s="164">
+        <f>E7*(F18-1)</f>
+        <v>51.61173333333331</v>
+      </c>
+      <c r="I7" s="165">
+        <f>E7*F18</f>
+        <v>180.64106666666663</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="166" t="n"/>
+      <c r="C8" s="167" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D8" s="168">
         <f>'Финмодель 6 паллет'!E13</f>
         <v>1.134046875</v>
       </c>
-      <c r="D7" s="166">
-        <f>C7*K14</f>
-        <v>58.063199999999995</v>
-      </c>
-      <c r="E7" s="167">
-        <f>F7/K14</f>
+      <c r="E8" s="169">
+        <f>E7/G18</f>
         <v>2.520104166666666</v>
       </c>
-      <c r="F7" s="166">
-        <f>D7/(1-G14-E14)</f>
-        <v>129.0293333333333</v>
-      </c>
-      <c r="G7" s="167">
-        <f>H7/K14</f>
+      <c r="F8" s="169">
+        <f>F7/G18</f>
         <v>0.6300260416666665</v>
       </c>
-      <c r="H7" s="168">
-        <f>F7*G14</f>
-        <v>32.25733333333333</v>
-      </c>
-      <c r="I7" s="167">
-        <f>J7/K14</f>
+      <c r="G8" s="169">
+        <f>G7/G18</f>
         <v>0.7560312499999997</v>
       </c>
-      <c r="J7" s="168">
-        <f>F7-D7-H7</f>
-        <v>38.70879999999999</v>
-      </c>
-      <c r="K7" s="167">
-        <f>L7/K14</f>
+      <c r="H8" s="169">
+        <f>H7/G18</f>
         <v>1.0080416666666663</v>
       </c>
-      <c r="L7" s="168">
-        <f>F7*(I14-1)</f>
-        <v>51.61173333333331</v>
-      </c>
-      <c r="M7" s="167">
-        <f>N7/K14</f>
+      <c r="I8" s="169">
+        <f>I7/G18</f>
         <v>3.5281458333333324</v>
       </c>
-      <c r="N7" s="169">
-        <f>F7*I14</f>
-        <v>180.64106666666663</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="170" t="str">
-        <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
-        <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
-      </c>
-      <c r="C8" s="165">
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="B9" s="170" t="inlineStr">
+        <is>
+          <t>ДО · Gouda Cheese, Carbonara Spicy
+(2 SKU)</t>
+        </is>
+      </c>
+      <c r="C9" s="171">
+        <f>C10*G18</f>
+        <v>38.400000000000006</v>
+      </c>
+      <c r="D9" s="171">
+        <f>D10*G18</f>
+        <v>66.99600000000001</v>
+      </c>
+      <c r="E9" s="171">
+        <f>D9/(1-E18-D18)</f>
+        <v>148.88000000000002</v>
+      </c>
+      <c r="F9" s="172">
+        <f>E9*E18</f>
+        <v>37.220000000000006</v>
+      </c>
+      <c r="G9" s="172">
+        <f>E9-D9-F9</f>
+        <v>44.66400000000001</v>
+      </c>
+      <c r="H9" s="172">
+        <f>E9*(F18-1)</f>
+        <v>59.552</v>
+      </c>
+      <c r="I9" s="173">
+        <f>E9*F18</f>
+        <v>208.43200000000002</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="174" t="n"/>
+      <c r="C10" s="167" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D10" s="168">
         <f>'Финмодель 6 паллет'!E11</f>
         <v>1.308515625</v>
       </c>
-      <c r="D8" s="171">
-        <f>C8*K14</f>
-        <v>66.99600000000001</v>
-      </c>
-      <c r="E8" s="172">
-        <f>F8/K14</f>
+      <c r="E10" s="175">
+        <f>E9/G18</f>
         <v>2.9078125000000004</v>
       </c>
-      <c r="F8" s="171">
-        <f>D8/(1-G14-E14)</f>
-        <v>148.88000000000002</v>
-      </c>
-      <c r="G8" s="172">
-        <f>H8/K14</f>
+      <c r="F10" s="175">
+        <f>F9/G18</f>
         <v>0.7269531250000001</v>
       </c>
-      <c r="H8" s="173">
-        <f>F8*G14</f>
-        <v>37.220000000000006</v>
-      </c>
-      <c r="I8" s="172">
-        <f>J8/K14</f>
+      <c r="G10" s="175">
+        <f>G9/G18</f>
         <v>0.8723437500000001</v>
       </c>
-      <c r="J8" s="173">
-        <f>F8-D8-H8</f>
-        <v>44.66400000000001</v>
-      </c>
-      <c r="K8" s="172">
-        <f>L8/K14</f>
+      <c r="H10" s="175">
+        <f>H9/G18</f>
         <v>1.163125</v>
       </c>
-      <c r="L8" s="173">
-        <f>F8*(I14-1)</f>
-        <v>59.552</v>
-      </c>
-      <c r="M8" s="172">
-        <f>N8/K14</f>
+      <c r="I10" s="175">
+        <f>I9/G18</f>
         <v>4.0709375</v>
       </c>
-      <c r="N8" s="174">
-        <f>F8*I14</f>
-        <v>208.43200000000002</v>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="175" t="str">
-        <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
-        <v>ПОСЛЕ · запрос SIAS €0.32 (все 6 SKU)</v>
-      </c>
-      <c r="C9" s="176">
-        <f>D9/K14</f>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="176" t="inlineStr">
+        <is>
+          <t>ПОСЛЕ · запрос SIAS
+(все 6 SKU)</t>
+        </is>
+      </c>
+      <c r="C11" s="177">
+        <f>C12*G18</f>
+        <v>16.384</v>
+      </c>
+      <c r="D11" s="177">
+        <f>C28</f>
+        <v>38.15951999999999</v>
+      </c>
+      <c r="E11" s="177">
+        <f>D11/(1-E18-D18)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="F11" s="178">
+        <f>E11*E18</f>
+        <v>21.19973333333333</v>
+      </c>
+      <c r="G11" s="178">
+        <f>E11-D11-F11</f>
+        <v>25.43968</v>
+      </c>
+      <c r="H11" s="178">
+        <f>E11*(F18-1)</f>
+        <v>33.919573333333325</v>
+      </c>
+      <c r="I11" s="179">
+        <f>E11*F18</f>
+        <v>118.71850666666664</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="157" t="n"/>
+      <c r="C12" s="180">
+        <f>C26</f>
+        <v>0.32</v>
+      </c>
+      <c r="D12" s="181">
+        <f>D11/G18</f>
         <v>0.7453031249999998</v>
       </c>
-      <c r="D9" s="177">
-        <f>C23</f>
-        <v>38.15951999999999</v>
-      </c>
-      <c r="E9" s="176">
-        <f>F9/K14</f>
+      <c r="E12" s="181">
+        <f>E11/G18</f>
         <v>1.6562291666666664</v>
       </c>
-      <c r="F9" s="177">
-        <f>D9/(1-G14-E14)</f>
-        <v>84.79893333333332</v>
-      </c>
-      <c r="G9" s="176">
-        <f>H9/K14</f>
+      <c r="F12" s="181">
+        <f>F11/G18</f>
         <v>0.4140572916666666</v>
       </c>
-      <c r="H9" s="178">
-        <f>F9*G14</f>
-        <v>21.19973333333333</v>
-      </c>
-      <c r="I9" s="176">
-        <f>J9/K14</f>
+      <c r="G12" s="181">
+        <f>G11/G18</f>
         <v>0.49686874999999997</v>
       </c>
-      <c r="J9" s="178">
-        <f>F9-D9-H9</f>
-        <v>25.43968</v>
-      </c>
-      <c r="K9" s="176">
-        <f>L9/K14</f>
+      <c r="H12" s="181">
+        <f>H11/G18</f>
         <v>0.6624916666666665</v>
       </c>
-      <c r="L9" s="178">
-        <f>F9*(I14-1)</f>
-        <v>33.919573333333325</v>
-      </c>
-      <c r="M9" s="176">
-        <f>N9/K14</f>
+      <c r="I12" s="181">
+        <f>I11/G18</f>
         <v>2.318720833333333</v>
       </c>
-      <c r="N9" s="179">
-        <f>F9*I14</f>
-        <v>118.71850666666664</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="180" t="inlineStr">
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="182" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="181">
-        <f>C9-C7</f>
+      <c r="C13" s="183">
+        <f>C11-C7</f>
+        <v>-16.896</v>
+      </c>
+      <c r="D13" s="183">
+        <f>D11-D7</f>
+        <v>-19.90368</v>
+      </c>
+      <c r="E13" s="183">
+        <f>E11-E7</f>
+        <v>-44.23039999999999</v>
+      </c>
+      <c r="F13" s="183">
+        <f>F11-F7</f>
+        <v>-11.057599999999997</v>
+      </c>
+      <c r="G13" s="183">
+        <f>G11-G7</f>
+        <v>-13.26911999999999</v>
+      </c>
+      <c r="H13" s="183">
+        <f>H11-H7</f>
+        <v>-17.692159999999987</v>
+      </c>
+      <c r="I13" s="183">
+        <f>I11-I7</f>
+        <v>-61.92255999999999</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="159" t="n"/>
+      <c r="C14" s="184">
+        <f>C12-C8</f>
+        <v>-0.33</v>
+      </c>
+      <c r="D14" s="184">
+        <f>D12-D8</f>
         <v>-0.38874375000000005</v>
       </c>
-      <c r="D10" s="182">
-        <f>D9-D7</f>
-        <v>-19.90368</v>
-      </c>
-      <c r="E10" s="181">
-        <f>E9-E7</f>
+      <c r="E14" s="184">
+        <f>E12-E8</f>
         <v>-0.8638749999999997</v>
       </c>
-      <c r="F10" s="182">
-        <f>F9-F7</f>
-        <v>-44.23039999999999</v>
-      </c>
-      <c r="G10" s="181">
-        <f>G9-G7</f>
+      <c r="F14" s="184">
+        <f>F12-F8</f>
         <v>-0.21596874999999993</v>
       </c>
-      <c r="H10" s="182">
-        <f>H9-H7</f>
-        <v>-11.057599999999997</v>
-      </c>
-      <c r="I10" s="181">
-        <f>I9-I7</f>
+      <c r="G14" s="184">
+        <f>G12-G8</f>
         <v>-0.25916249999999974</v>
       </c>
-      <c r="J10" s="182">
-        <f>J9-J7</f>
-        <v>-13.26911999999999</v>
-      </c>
-      <c r="K10" s="181">
-        <f>K9-K7</f>
+      <c r="H14" s="184">
+        <f>H12-H8</f>
         <v>-0.3455499999999998</v>
       </c>
-      <c r="L10" s="182">
-        <f>L9-L7</f>
-        <v>-17.692159999999987</v>
-      </c>
-      <c r="M10" s="181">
-        <f>M9-M7</f>
+      <c r="I14" s="184">
+        <f>I12-I8</f>
         <v>-1.2094249999999995</v>
       </c>
-      <c r="N10" s="182">
-        <f>N9-N7</f>
-        <v>-61.92255999999999</v>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="183" t="inlineStr">
-        <is>
-          <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="184" t="inlineStr">
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="185" t="inlineStr">
+        <is>
+          <t>Каждая линия читается слева направо: цена закупки → себестоимость в Украине → цена партнёру → бонус, наша прибыль, наценка → полка. Верхняя цифра — ₴, нижняя — €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="186" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 6 паллет»</t>
         </is>
       </c>
-      <c r="C12" s="185" t="n"/>
-      <c r="D12" s="185" t="n"/>
-      <c r="E12" s="185" t="n"/>
-      <c r="F12" s="185" t="n"/>
-      <c r="G12" s="185" t="n"/>
-      <c r="H12" s="185" t="n"/>
-      <c r="I12" s="185" t="n"/>
-      <c r="J12" s="185" t="n"/>
-      <c r="K12" s="185" t="n"/>
-      <c r="L12" s="185" t="n"/>
-      <c r="M12" s="185" t="n"/>
-      <c r="N12" s="185" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="C13" s="186" t="inlineStr">
+      <c r="C16" s="187" t="n"/>
+      <c r="D16" s="187" t="n"/>
+      <c r="E16" s="187" t="n"/>
+      <c r="F16" s="187" t="n"/>
+      <c r="G16" s="187" t="n"/>
+      <c r="H16" s="187" t="n"/>
+      <c r="I16" s="187" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="C17" s="188" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E13" s="186" t="inlineStr">
+      <c r="D17" s="188" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G13" s="186" t="inlineStr">
+      <c r="E17" s="188" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I13" s="186" t="inlineStr">
+      <c r="F17" s="188" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K13" s="186" t="inlineStr">
+      <c r="G17" s="188" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="187" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="189" t="inlineStr">
         <is>
           <t>Цель расчёта и условия модели</t>
         </is>
       </c>
-      <c r="C14" s="188" t="n">
+      <c r="C18" s="190" t="n">
         <v>120</v>
       </c>
-      <c r="D14" s="189" t="n"/>
-      <c r="E14" s="190" t="n">
+      <c r="D18" s="191" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="189" t="n"/>
-      <c r="G14" s="191">
+      <c r="E18" s="192">
         <f>'Финмодель 6 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H14" s="192" t="n"/>
-      <c r="I14" s="193">
+      <c r="F18" s="193">
         <f>'Финмодель 6 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J14" s="192" t="n"/>
-      <c r="K14" s="194">
+      <c r="G18" s="194">
         <f>'Финмодель 6 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L14" s="192" t="n"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="195" t="inlineStr">
-        <is>
-          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" hidden="1">
-      <c r="C16" s="186" t="inlineStr">
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="195" t="inlineStr">
+        <is>
+          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS не получено — это цена для переговоров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" hidden="1">
+      <c r="C21" s="188" t="inlineStr">
         <is>
           <t>Импортный ПДВ</t>
         </is>
       </c>
-      <c r="E16" s="186" t="inlineStr">
+      <c r="D21" s="188" t="inlineStr">
         <is>
           <t>Финансирование</t>
         </is>
       </c>
-      <c r="G16" s="186" t="inlineStr">
+      <c r="E21" s="188" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="I16" s="186" t="inlineStr">
+      <c r="F21" s="188" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="K16" s="186" t="inlineStr">
+      <c r="G21" s="188" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="M16" s="186" t="inlineStr">
+      <c r="H21" s="188" t="inlineStr">
         <is>
           <t>Прочие, €</t>
         </is>
       </c>
     </row>
-    <row r="17" hidden="1">
-      <c r="C17" s="190" t="n">
+    <row r="22" hidden="1">
+      <c r="C22" s="191" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="189" t="n"/>
-      <c r="E17" s="190" t="n">
+      <c r="D22" s="191" t="n">
         <v>0.025</v>
       </c>
-      <c r="F17" s="189" t="n"/>
-      <c r="G17" s="190" t="n">
+      <c r="E22" s="191" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="189" t="n"/>
-      <c r="I17" s="196" t="n">
+      <c r="F22" s="196" t="n">
         <v>2600</v>
       </c>
-      <c r="J17" s="189" t="n"/>
-      <c r="K17" s="196" t="n">
+      <c r="G22" s="196" t="n">
         <v>288</v>
       </c>
-      <c r="L17" s="189" t="n"/>
-      <c r="M17" s="196" t="n">
+      <c r="H22" s="196" t="n">
         <v>42</v>
       </c>
-      <c r="N17" s="189" t="n"/>
-    </row>
-    <row r="18" hidden="1">
-      <c r="C18" s="186" t="inlineStr">
+    </row>
+    <row r="23" hidden="1">
+      <c r="C23" s="188" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="E18" s="186" t="inlineStr">
+      <c r="D23" s="188" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="G18" s="186" t="inlineStr">
+      <c r="E23" s="188" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
-    <row r="19" hidden="1">
-      <c r="C19" s="197" t="n">
+    <row r="24" hidden="1">
+      <c r="C24" s="197" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="189" t="n"/>
-      <c r="E19" s="196" t="n">
+      <c r="D24" s="196" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="189" t="n"/>
-      <c r="G19" s="196" t="n">
+      <c r="E24" s="196" t="n">
         <v>1600</v>
       </c>
-      <c r="H19" s="189" t="n"/>
-    </row>
-    <row r="20" hidden="1">
-      <c r="B20" s="198" t="inlineStr">
-        <is>
-          <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
-        </is>
-      </c>
-      <c r="C20" s="197" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E20" s="197" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="21" hidden="1">
-      <c r="B21" s="198" t="inlineStr">
+    </row>
+    <row r="25" hidden="1"/>
+    <row r="26" hidden="1">
+      <c r="B26" s="198" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
-      <c r="C21" s="199">
-        <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
+      <c r="C26" s="199">
+        <f>ROUNDDOWN(((C18/F18*(1-E18-D18))/G18/(1+D22)-(F22+G22+H22+F22*C24*(E22+C22*(1+E22)))/(D24*E24))/((1+E22)*(1+C22)),2)</f>
         <v>0.32</v>
       </c>
-      <c r="D21" s="157" t="n"/>
-    </row>
-    <row r="22" hidden="1">
-      <c r="B22" s="198" t="inlineStr">
+    </row>
+    <row r="27" hidden="1">
+      <c r="B27" s="198" t="inlineStr">
         <is>
           <t>Предельная закупка до округления, €/уп.</t>
         </is>
       </c>
-      <c r="C22" s="200">
-        <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
+      <c r="C27" s="200">
+        <f>((C18/F18*(1-E18-D18))/G18/(1+D22)-(F22+G22+H22+F22*C24*(E22+C22*(1+E22)))/(D24*E24))/((1+E22)*(1+C22))</f>
         <v>0.3265407229965157</v>
       </c>
-      <c r="D22" s="201" t="n"/>
-    </row>
-    <row r="23" hidden="1">
-      <c r="B23" s="198" t="inlineStr">
+    </row>
+    <row r="28" hidden="1">
+      <c r="B28" s="198" t="inlineStr">
         <is>
           <t>Себестоимость в Украине при запросе, ₴/уп.</t>
         </is>
       </c>
-      <c r="C23" s="202">
-        <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
+      <c r="C28" s="201">
+        <f>(C26*G18+(F22+G22+H22)/(D24*E24)*G18+(C26+F22*C24/(D24*E24))*E22*G18+(C26+F22*C24/(D24*E24))*(1+E22)*C22*G18)*(1+D22)</f>
         <v>38.15951999999999</v>
       </c>
-      <c r="D23" s="201" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="46">
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="L4:N4"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
+  <mergeCells count="12">
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B19:I19"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="B12:N12"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="B11:N11"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="E18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
@@ -6771,38 +6709,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N23"/>
+  <dimension ref="B2:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="2" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="152" t="inlineStr">
         <is>
-          <t>SIAS · было → стало · от себестоимости в Украине до полки · 33 паллеты (Full Truck)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>SIAS · от цены закупки до полки одной линией · 33 паллеты (Full Truck)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="B3" s="153" t="str">
-        <f>"Полка "&amp;ROUND(C14,0)&amp;" ₴ достижима при себестоимости "&amp;ROUND(D9,2)&amp;" ₴ (сейчас "&amp;ROUND(D7,2)&amp;"–"&amp;ROUND(D8,2)&amp;" ₴). Для этого закупка SIAS должна быть €"&amp;ROUND(C21,2)&amp;" вместо €"&amp;MIN(C20,E20)&amp;"–€"&amp;MAX(C20,E20)&amp;" (−"&amp;ROUND((1-C21/MIN(C20,E20))*100,0)&amp;"…"&amp;ROUND((1-C21/MAX(C20,E20))*100,0)&amp;"%)."</f>
-        <v>Полка 120 ₴ достижима при себестоимости 38.53 ₴ (сейчас 45.18–52.13 ₴). Для этого закупка SIAS должна быть €0.54 вместо €0.65–€0.75 (−17…28%).</v>
+        <f>"Цена закупки SIAS €"&amp;ROUND(C26,2)&amp;" вместо €"&amp;MIN(C8,C10)&amp;"–€"&amp;MAX(C8,C10)&amp;" (−"&amp;ROUND((1-C26/MIN(C8,C10))*100,0)&amp;"…"&amp;ROUND((1-C26/MAX(C8,C10))*100,0)&amp;"%) → полка "&amp;ROUND(I11,2)&amp;" ₴ при марже "&amp;ROUND(D18*100,0)&amp;"%."</f>
+        <v>Цена закупки SIAS €0.54 вместо €0.65–€0.75 (−17…28%) → полка 119.86 ₴ при марже 30%.</v>
       </c>
       <c r="C3" s="154" t="n"/>
       <c r="D3" s="154" t="n"/>
@@ -6811,11 +6744,6 @@
       <c r="G3" s="154" t="n"/>
       <c r="H3" s="154" t="n"/>
       <c r="I3" s="154" t="n"/>
-      <c r="J3" s="154" t="n"/>
-      <c r="K3" s="154" t="n"/>
-      <c r="L3" s="154" t="n"/>
-      <c r="M3" s="154" t="n"/>
-      <c r="N3" s="154" t="n"/>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="B4" s="155" t="inlineStr">
@@ -6824,630 +6752,548 @@
         </is>
       </c>
       <c r="C4" s="156">
-        <f>C21</f>
+        <f>C26</f>
         <v>0.54</v>
       </c>
       <c r="D4" s="157" t="n"/>
       <c r="E4" s="158" t="str">
-        <f>"сейчас €"&amp;C20&amp;" (4 SKU) / €"&amp;E20&amp;" (2 SKU)"</f>
+        <f>"сейчас €"&amp;C8&amp;" (4 SKU) / €"&amp;C10&amp;" (2 SKU)"</f>
         <v>сейчас €0.65 (4 SKU) / €0.75 (2 SKU)</v>
       </c>
       <c r="F4" s="159" t="n"/>
-      <c r="G4" s="159" t="n"/>
+      <c r="G4" s="160" t="str">
+        <f>"снижение −"&amp;ROUND((1-C26/C8)*100,0)&amp;" % / −"&amp;ROUND((1-C26/C10)*100,0)&amp;" %"</f>
+        <v>снижение −17 % / −28 %</v>
+      </c>
       <c r="H4" s="159" t="n"/>
-      <c r="I4" s="160" t="str">
-        <f>"снижение −"&amp;ROUND((1-C21/C20)*100,0)&amp;" % / −"&amp;ROUND((1-C21/E20)*100,0)&amp;" %"</f>
-        <v>снижение −17 % / −28 %</v>
-      </c>
-      <c r="J4" s="159" t="n"/>
-      <c r="K4" s="159" t="n"/>
-      <c r="L4" s="158" t="inlineStr">
-        <is>
-          <t>одна цена для всех 6 SKU</t>
-        </is>
-      </c>
-      <c r="M4" s="159" t="n"/>
-      <c r="N4" s="159" t="n"/>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="161" t="inlineStr"/>
+      <c r="I4" s="158" t="inlineStr">
+        <is>
+          <t>одна цена на 6 SKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="B5" s="161" t="inlineStr">
+        <is>
+          <t>Вариант</t>
+        </is>
+      </c>
       <c r="C5" s="161" t="inlineStr">
         <is>
-          <t>Себестоимость в Украине (СС)</t>
-        </is>
-      </c>
-      <c r="D5" s="162" t="n"/>
+          <t>Закупка SIAS
+за пачку</t>
+        </is>
+      </c>
+      <c r="D5" s="161" t="inlineStr">
+        <is>
+          <t>Себестоимость в Украине
+товар + расходы в Украине</t>
+        </is>
+      </c>
       <c r="E5" s="161" t="inlineStr">
         <is>
-          <t>Цена партнёру (магазину)</t>
-        </is>
-      </c>
-      <c r="F5" s="162" t="n"/>
+          <t>Цена партнёру
+СС ÷ (1 − бонус − маржа)</t>
+        </is>
+      </c>
+      <c r="F5" s="161" t="inlineStr">
+        <is>
+          <t>Бонус сети
+25 % цены партнёру</t>
+        </is>
+      </c>
       <c r="G5" s="161" t="inlineStr">
         <is>
-          <t>Бонус сети</t>
-        </is>
-      </c>
-      <c r="H5" s="162" t="n"/>
+          <t>Наша прибыль
+30 % цены партнёру</t>
+        </is>
+      </c>
+      <c r="H5" s="161" t="inlineStr">
+        <is>
+          <t>Наценка магазина
++40 % к цене партнёру</t>
+        </is>
+      </c>
       <c r="I5" s="161" t="inlineStr">
         <is>
-          <t>Наша прибыль</t>
-        </is>
-      </c>
-      <c r="J5" s="162" t="n"/>
-      <c r="K5" s="161" t="inlineStr">
-        <is>
-          <t>Наценка магазина</t>
-        </is>
-      </c>
-      <c r="L5" s="162" t="n"/>
-      <c r="M5" s="161" t="inlineStr">
-        <is>
-          <t>ПОЛКА с НДС</t>
-        </is>
-      </c>
-      <c r="N5" s="162" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="161" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="C6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="D6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="E6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="F6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="G6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="H6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="I6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="J6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="K6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="L6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-      <c r="M6" s="163" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-      <c r="N6" s="163" t="inlineStr">
-        <is>
-          <t>₴</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="164" t="str">
-        <f>"ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €"&amp;C20</f>
-        <v>ДО · Vegetable, Spicy, Beef, Chicken · закупка SIAS €0.65</v>
-      </c>
-      <c r="C7" s="165">
+          <t>ПОЛКА с НДС
+цена партнёру × 1,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="B7" s="162" t="inlineStr">
+        <is>
+          <t>ДО · Vegetable, Spicy, Beef, Chicken
+(4 SKU)</t>
+        </is>
+      </c>
+      <c r="C7" s="163">
+        <f>C8*G18</f>
+        <v>33.28</v>
+      </c>
+      <c r="D7" s="163">
+        <f>D8*G18</f>
+        <v>45.17787308533919</v>
+      </c>
+      <c r="E7" s="163">
+        <f>D7/(1-E18-D18)</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="F7" s="164">
+        <f>E7*E18</f>
+        <v>25.098818380743996</v>
+      </c>
+      <c r="G7" s="164">
+        <f>E7-D7-F7</f>
+        <v>30.118582056892794</v>
+      </c>
+      <c r="H7" s="164">
+        <f>E7*(F18-1)</f>
+        <v>40.15810940919039</v>
+      </c>
+      <c r="I7" s="165">
+        <f>E7*F18</f>
+        <v>140.55338293216636</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="166" t="n"/>
+      <c r="C8" s="167" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D8" s="168">
         <f>'Финмодель 33 паллет'!E13</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="D7" s="166">
-        <f>C7*K14</f>
-        <v>45.17787308533919</v>
-      </c>
-      <c r="E7" s="167">
-        <f>F7/K14</f>
+      <c r="E8" s="169">
+        <f>E7/G18</f>
         <v>1.9608451859956246</v>
       </c>
-      <c r="F7" s="166">
-        <f>D7/(1-G14-E14)</f>
-        <v>100.39527352297598</v>
-      </c>
-      <c r="G7" s="167">
-        <f>H7/K14</f>
+      <c r="F8" s="169">
+        <f>F7/G18</f>
         <v>0.49021129649890616</v>
       </c>
-      <c r="H7" s="168">
-        <f>F7*G14</f>
-        <v>25.098818380743996</v>
-      </c>
-      <c r="I7" s="167">
-        <f>J7/K14</f>
+      <c r="G8" s="169">
+        <f>G7/G18</f>
         <v>0.5882535557986873</v>
       </c>
-      <c r="J7" s="168">
-        <f>F7-D7-H7</f>
-        <v>30.118582056892794</v>
-      </c>
-      <c r="K7" s="167">
-        <f>L7/K14</f>
+      <c r="H8" s="169">
+        <f>H7/G18</f>
         <v>0.7843380743982498</v>
       </c>
-      <c r="L7" s="168">
-        <f>F7*(I14-1)</f>
-        <v>40.15810940919039</v>
-      </c>
-      <c r="M7" s="167">
-        <f>N7/K14</f>
+      <c r="I8" s="169">
+        <f>I7/G18</f>
         <v>2.745183260393874</v>
       </c>
-      <c r="N7" s="169">
-        <f>F7*I14</f>
-        <v>140.55338293216636</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="170" t="str">
-        <f>"ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €"&amp;E20</f>
-        <v>ДО · Gouda Cheese, Carbonara Spicy · закупка SIAS €0.75</v>
-      </c>
-      <c r="C8" s="165">
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="B9" s="170" t="inlineStr">
+        <is>
+          <t>ДО · Gouda Cheese, Carbonara Spicy
+(2 SKU)</t>
+        </is>
+      </c>
+      <c r="C9" s="171">
+        <f>C10*G18</f>
+        <v>38.400000000000006</v>
+      </c>
+      <c r="D9" s="171">
+        <f>D10*G18</f>
+        <v>52.12831509846825</v>
+      </c>
+      <c r="E9" s="171">
+        <f>D9/(1-E18-D18)</f>
+        <v>115.84070021881833</v>
+      </c>
+      <c r="F9" s="172">
+        <f>E9*E18</f>
+        <v>28.96017505470458</v>
+      </c>
+      <c r="G9" s="172">
+        <f>E9-D9-F9</f>
+        <v>34.7522100656455</v>
+      </c>
+      <c r="H9" s="172">
+        <f>E9*(F18-1)</f>
+        <v>46.33628008752732</v>
+      </c>
+      <c r="I9" s="173">
+        <f>E9*F18</f>
+        <v>162.17698030634565</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="174" t="n"/>
+      <c r="C10" s="167" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D10" s="168">
         <f>'Финмодель 33 паллет'!E11</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="D8" s="171">
-        <f>C8*K14</f>
-        <v>52.12831509846825</v>
-      </c>
-      <c r="E8" s="172">
-        <f>F8/K14</f>
+      <c r="E10" s="175">
+        <f>E9/G18</f>
         <v>2.2625136761487954</v>
       </c>
-      <c r="F8" s="171">
-        <f>D8/(1-G14-E14)</f>
-        <v>115.84070021881833</v>
-      </c>
-      <c r="G8" s="172">
-        <f>H8/K14</f>
+      <c r="F10" s="175">
+        <f>F9/G18</f>
         <v>0.5656284190371988</v>
       </c>
-      <c r="H8" s="173">
-        <f>F8*G14</f>
-        <v>28.96017505470458</v>
-      </c>
-      <c r="I8" s="172">
-        <f>J8/K14</f>
+      <c r="G10" s="175">
+        <f>G9/G18</f>
         <v>0.6787541028446387</v>
       </c>
-      <c r="J8" s="173">
-        <f>F8-D8-H8</f>
-        <v>34.7522100656455</v>
-      </c>
-      <c r="K8" s="172">
-        <f>L8/K14</f>
+      <c r="H10" s="175">
+        <f>H9/G18</f>
         <v>0.905005470459518</v>
       </c>
-      <c r="L8" s="173">
-        <f>F8*(I14-1)</f>
-        <v>46.33628008752732</v>
-      </c>
-      <c r="M8" s="172">
-        <f>N8/K14</f>
+      <c r="I10" s="175">
+        <f>I9/G18</f>
         <v>3.1675191466083135</v>
       </c>
-      <c r="N8" s="174">
-        <f>F8*I14</f>
-        <v>162.17698030634565</v>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="175" t="str">
-        <f>"ПОСЛЕ · запрос SIAS €"&amp;ROUND(C21,2)&amp;" (все 6 SKU)"</f>
-        <v>ПОСЛЕ · запрос SIAS €0.54 (все 6 SKU)</v>
-      </c>
-      <c r="C9" s="176">
-        <f>D9/K14</f>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="176" t="inlineStr">
+        <is>
+          <t>ПОСЛЕ · запрос SIAS
+(все 6 SKU)</t>
+        </is>
+      </c>
+      <c r="C11" s="177">
+        <f>C12*G18</f>
+        <v>27.648000000000003</v>
+      </c>
+      <c r="D11" s="177">
+        <f>C28</f>
+        <v>38.52747636363637</v>
+      </c>
+      <c r="E11" s="177">
+        <f>D11/(1-E18-D18)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="F11" s="178">
+        <f>E11*E18</f>
+        <v>21.404153535353537</v>
+      </c>
+      <c r="G11" s="178">
+        <f>E11-D11-F11</f>
+        <v>25.684984242424242</v>
+      </c>
+      <c r="H11" s="178">
+        <f>E11*(F18-1)</f>
+        <v>34.246645656565654</v>
+      </c>
+      <c r="I11" s="179">
+        <f>E11*F18</f>
+        <v>119.8632597979798</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="157" t="n"/>
+      <c r="C12" s="180">
+        <f>C26</f>
+        <v>0.54</v>
+      </c>
+      <c r="D12" s="181">
+        <f>D11/G18</f>
         <v>0.7524897727272728</v>
       </c>
-      <c r="D9" s="177">
-        <f>C23</f>
-        <v>38.52747636363637</v>
-      </c>
-      <c r="E9" s="176">
-        <f>F9/K14</f>
+      <c r="E12" s="181">
+        <f>E11/G18</f>
         <v>1.672199494949495</v>
       </c>
-      <c r="F9" s="177">
-        <f>D9/(1-G14-E14)</f>
-        <v>85.61661414141415</v>
-      </c>
-      <c r="G9" s="176">
-        <f>H9/K14</f>
+      <c r="F12" s="181">
+        <f>F11/G18</f>
         <v>0.41804987373737373</v>
       </c>
-      <c r="H9" s="178">
-        <f>F9*G14</f>
-        <v>21.404153535353537</v>
-      </c>
-      <c r="I9" s="176">
-        <f>J9/K14</f>
+      <c r="G12" s="181">
+        <f>G11/G18</f>
         <v>0.5016598484848485</v>
       </c>
-      <c r="J9" s="178">
-        <f>F9-D9-H9</f>
-        <v>25.684984242424242</v>
-      </c>
-      <c r="K9" s="176">
-        <f>L9/K14</f>
+      <c r="H12" s="181">
+        <f>H11/G18</f>
         <v>0.6688797979797979</v>
       </c>
-      <c r="L9" s="178">
-        <f>F9*(I14-1)</f>
-        <v>34.246645656565654</v>
-      </c>
-      <c r="M9" s="176">
-        <f>N9/K14</f>
+      <c r="I12" s="181">
+        <f>I11/G18</f>
         <v>2.3410792929292925</v>
       </c>
-      <c r="N9" s="179">
-        <f>F9*I14</f>
-        <v>119.8632597979798</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="180" t="inlineStr">
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="182" t="inlineStr">
         <is>
           <t>ИЗМЕНЕНИЕ: ПОСЛЕ − ДО (4 SKU)</t>
         </is>
       </c>
-      <c r="C10" s="181">
-        <f>C9-C7</f>
+      <c r="C13" s="183">
+        <f>C11-C7</f>
+        <v>-5.631999999999998</v>
+      </c>
+      <c r="D13" s="183">
+        <f>D11-D7</f>
+        <v>-6.650396721702826</v>
+      </c>
+      <c r="E13" s="183">
+        <f>E11-E7</f>
+        <v>-14.778659381561837</v>
+      </c>
+      <c r="F13" s="183">
+        <f>F11-F7</f>
+        <v>-3.6946648453904594</v>
+      </c>
+      <c r="G13" s="183">
+        <f>G11-G7</f>
+        <v>-4.433597814468552</v>
+      </c>
+      <c r="H13" s="183">
+        <f>H11-H7</f>
+        <v>-5.911463752624734</v>
+      </c>
+      <c r="I13" s="183">
+        <f>I11-I7</f>
+        <v>-20.690123134186564</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="159" t="n"/>
+      <c r="C14" s="184">
+        <f>C12-C8</f>
+        <v>-0.10999999999999999</v>
+      </c>
+      <c r="D14" s="184">
+        <f>D12-D8</f>
         <v>-0.12989056097075824</v>
       </c>
-      <c r="D10" s="182">
-        <f>D9-D7</f>
-        <v>-6.650396721702826</v>
-      </c>
-      <c r="E10" s="181">
-        <f>E9-E7</f>
+      <c r="E14" s="184">
+        <f>E12-E8</f>
         <v>-0.2886456910461297</v>
       </c>
-      <c r="F10" s="182">
-        <f>F9-F7</f>
-        <v>-14.778659381561837</v>
-      </c>
-      <c r="G10" s="181">
-        <f>G9-G7</f>
+      <c r="F14" s="184">
+        <f>F12-F8</f>
         <v>-0.07216142276153242</v>
       </c>
-      <c r="H10" s="182">
-        <f>H9-H7</f>
-        <v>-3.6946648453904594</v>
-      </c>
-      <c r="I10" s="181">
-        <f>I9-I7</f>
+      <c r="G14" s="184">
+        <f>G12-G8</f>
         <v>-0.08659370731383886</v>
       </c>
-      <c r="J10" s="182">
-        <f>J9-J7</f>
-        <v>-4.433597814468552</v>
-      </c>
-      <c r="K10" s="181">
-        <f>K9-K7</f>
+      <c r="H14" s="184">
+        <f>H12-H8</f>
         <v>-0.11545827641845186</v>
       </c>
-      <c r="L10" s="182">
-        <f>L9-L7</f>
-        <v>-5.911463752624734</v>
-      </c>
-      <c r="M10" s="181">
-        <f>M9-M7</f>
+      <c r="I14" s="184">
+        <f>I12-I8</f>
         <v>-0.40410396746458144</v>
       </c>
-      <c r="N10" s="182">
-        <f>N9-N7</f>
-        <v>-20.690123134186564</v>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="183" t="inlineStr">
-        <is>
-          <t>Читайте по строке слева направо: себестоимость в Украине → цена партнёру = СС ÷ (1 − бонус − маржа) → бонус, наша прибыль, наценка → полка. Каждая цифра дана в € и ₴.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="184" t="inlineStr">
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="185" t="inlineStr">
+        <is>
+          <t>Каждая линия читается слева направо: цена закупки → себестоимость в Украине → цена партнёру → бонус, наша прибыль, наценка → полка. Верхняя цифра — ₴, нижняя — €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="186" t="inlineStr">
         <is>
           <t>ИСХОДНЫЕ ДАННЫЕ — жёлтое можно менять, зелёное из вкладки «Финмодель 33 паллет»</t>
         </is>
       </c>
-      <c r="C12" s="185" t="n"/>
-      <c r="D12" s="185" t="n"/>
-      <c r="E12" s="185" t="n"/>
-      <c r="F12" s="185" t="n"/>
-      <c r="G12" s="185" t="n"/>
-      <c r="H12" s="185" t="n"/>
-      <c r="I12" s="185" t="n"/>
-      <c r="J12" s="185" t="n"/>
-      <c r="K12" s="185" t="n"/>
-      <c r="L12" s="185" t="n"/>
-      <c r="M12" s="185" t="n"/>
-      <c r="N12" s="185" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="C13" s="186" t="inlineStr">
+      <c r="C16" s="187" t="n"/>
+      <c r="D16" s="187" t="n"/>
+      <c r="E16" s="187" t="n"/>
+      <c r="F16" s="187" t="n"/>
+      <c r="G16" s="187" t="n"/>
+      <c r="H16" s="187" t="n"/>
+      <c r="I16" s="187" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="C17" s="188" t="inlineStr">
         <is>
           <t>Полка, ₴</t>
         </is>
       </c>
-      <c r="E13" s="186" t="inlineStr">
+      <c r="D17" s="188" t="inlineStr">
         <is>
           <t>Наша маржа</t>
         </is>
       </c>
-      <c r="G13" s="186" t="inlineStr">
+      <c r="E17" s="188" t="inlineStr">
         <is>
           <t>Бонус сети</t>
         </is>
       </c>
-      <c r="I13" s="186" t="inlineStr">
+      <c r="F17" s="188" t="inlineStr">
         <is>
           <t>Множитель полки</t>
         </is>
       </c>
-      <c r="K13" s="186" t="inlineStr">
+      <c r="G17" s="188" t="inlineStr">
         <is>
           <t>Курс ₴/€</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="187" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="189" t="inlineStr">
         <is>
           <t>Цель расчёта и условия модели</t>
         </is>
       </c>
-      <c r="C14" s="188" t="n">
+      <c r="C18" s="190" t="n">
         <v>120</v>
       </c>
-      <c r="D14" s="189" t="n"/>
-      <c r="E14" s="190" t="n">
+      <c r="D18" s="191" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="189" t="n"/>
-      <c r="G14" s="191">
+      <c r="E18" s="192">
         <f>'Финмодель 33 паллет'!D4</f>
         <v>0.25</v>
       </c>
-      <c r="H14" s="192" t="n"/>
-      <c r="I14" s="193">
+      <c r="F18" s="193">
         <f>'Финмодель 33 паллет'!D6</f>
         <v>1.4</v>
       </c>
-      <c r="J14" s="192" t="n"/>
-      <c r="K14" s="194">
+      <c r="G18" s="194">
         <f>'Финмодель 33 паллет'!D3</f>
         <v>51.2</v>
       </c>
-      <c r="L14" s="192" t="n"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="195" t="inlineStr">
-        <is>
-          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS на цену не получено — это цена для переговоров.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" hidden="1">
-      <c r="C16" s="186" t="inlineStr">
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="195" t="inlineStr">
+        <is>
+          <t>Допущения: бонус и множитель — по модели (не подтверждены сетями); без листинг-фи, промо и отсрочки; согласие SIAS не получено — это цена для переговоров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" hidden="1">
+      <c r="C21" s="188" t="inlineStr">
         <is>
           <t>Импортный ПДВ</t>
         </is>
       </c>
-      <c r="E16" s="186" t="inlineStr">
+      <c r="D21" s="188" t="inlineStr">
         <is>
           <t>Финансирование</t>
         </is>
       </c>
-      <c r="G16" s="186" t="inlineStr">
+      <c r="E21" s="188" t="inlineStr">
         <is>
           <t>Пошлина</t>
         </is>
       </c>
-      <c r="I16" s="186" t="inlineStr">
+      <c r="F21" s="188" t="inlineStr">
         <is>
           <t>Перевозка партии, €</t>
         </is>
       </c>
-      <c r="K16" s="186" t="inlineStr">
+      <c r="G21" s="188" t="inlineStr">
         <is>
           <t>Брокер, €</t>
         </is>
       </c>
-      <c r="M16" s="186" t="inlineStr">
+      <c r="H21" s="188" t="inlineStr">
         <is>
           <t>Прочие, €</t>
         </is>
       </c>
     </row>
-    <row r="17" hidden="1">
-      <c r="C17" s="190" t="n">
+    <row r="22" hidden="1">
+      <c r="C22" s="191" t="n">
         <v>0.2</v>
       </c>
-      <c r="D17" s="189" t="n"/>
-      <c r="E17" s="190" t="n">
+      <c r="D22" s="191" t="n">
         <v>0.025</v>
       </c>
-      <c r="F17" s="189" t="n"/>
-      <c r="G17" s="190" t="n">
+      <c r="E22" s="191" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="189" t="n"/>
-      <c r="I17" s="196" t="n">
+      <c r="F22" s="196" t="n">
         <v>3700</v>
       </c>
-      <c r="J17" s="189" t="n"/>
-      <c r="K17" s="196" t="n">
+      <c r="G22" s="196" t="n">
         <v>288</v>
       </c>
-      <c r="L17" s="189" t="n"/>
-      <c r="M17" s="196" t="n">
+      <c r="H22" s="196" t="n">
         <v>42</v>
       </c>
-      <c r="N17" s="189" t="n"/>
-    </row>
-    <row r="18" hidden="1">
-      <c r="C18" s="186" t="inlineStr">
+    </row>
+    <row r="23" hidden="1">
+      <c r="C23" s="188" t="inlineStr">
         <is>
           <t>Доля фрахта в таможне</t>
         </is>
       </c>
-      <c r="E18" s="186" t="inlineStr">
+      <c r="D23" s="188" t="inlineStr">
         <is>
           <t>Паллет в партии</t>
         </is>
       </c>
-      <c r="G18" s="186" t="inlineStr">
+      <c r="E23" s="188" t="inlineStr">
         <is>
           <t>Пачек на паллете</t>
         </is>
       </c>
     </row>
-    <row r="19" hidden="1">
-      <c r="C19" s="197" t="n">
+    <row r="24" hidden="1">
+      <c r="C24" s="197" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="189" t="n"/>
-      <c r="E19" s="196" t="n">
+      <c r="D24" s="196" t="n">
         <v>33</v>
       </c>
-      <c r="F19" s="189" t="n"/>
-      <c r="G19" s="196" t="n">
+      <c r="E24" s="196" t="n">
         <v>1600</v>
       </c>
-      <c r="H19" s="189" t="n"/>
-    </row>
-    <row r="20" hidden="1">
-      <c r="B20" s="198" t="inlineStr">
-        <is>
-          <t>Закупка SIAS сейчас, €: 4 SKU / 2 SKU</t>
-        </is>
-      </c>
-      <c r="C20" s="197" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E20" s="197" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="21" hidden="1">
-      <c r="B21" s="198" t="inlineStr">
+    </row>
+    <row r="25" hidden="1"/>
+    <row r="26" hidden="1">
+      <c r="B26" s="198" t="inlineStr">
         <is>
           <t>Запрос SIAS, €/уп. (вниз до евроцента)</t>
         </is>
       </c>
-      <c r="C21" s="199">
-        <f>ROUNDDOWN(((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17)),2)</f>
+      <c r="C26" s="199">
+        <f>ROUNDDOWN(((C18/F18*(1-E18-D18))/G18/(1+D22)-(F22+G22+H22+F22*C24*(E22+C22*(1+E22)))/(D24*E24))/((1+E22)*(1+C22)),2)</f>
         <v>0.54</v>
       </c>
-      <c r="D21" s="157" t="n"/>
-    </row>
-    <row r="22" hidden="1">
-      <c r="B22" s="198" t="inlineStr">
+    </row>
+    <row r="27" hidden="1">
+      <c r="B27" s="198" t="inlineStr">
         <is>
           <t>Предельная закупка до округления, €/уп.</t>
         </is>
       </c>
-      <c r="C22" s="200">
-        <f>((C14/I14*(1-G14-E14))/K14/(1+E17)-(I17+K17+M17+I17*C19*(G17+C17*(1+G17)))/(E19*G19))/((1+G17)*(1+C17))</f>
+      <c r="C27" s="200">
+        <f>((C18/F18*(1-E18-D18))/G18/(1+D22)-(F22+G22+H22+F22*C24*(E22+C22*(1+E22)))/(D24*E24))/((1+E22)*(1+C22))</f>
         <v>0.5406979199662126</v>
       </c>
-      <c r="D22" s="201" t="n"/>
-    </row>
-    <row r="23" hidden="1">
-      <c r="B23" s="198" t="inlineStr">
+    </row>
+    <row r="28" hidden="1">
+      <c r="B28" s="198" t="inlineStr">
         <is>
           <t>Себестоимость в Украине при запросе, ₴/уп.</t>
         </is>
       </c>
-      <c r="C23" s="202">
-        <f>(C21*K14+(I17+K17+M17)/(E19*G19)*K14+(C21+I17*C19/(E19*G19))*G17*K14+(C21+I17*C19/(E19*G19))*(1+G17)*C17*K14)*(1+E17)</f>
+      <c r="C28" s="201">
+        <f>(C26*G18+(F22+G22+H22)/(D24*E24)*G18+(C26+F22*C24/(D24*E24))*E22*G18+(C26+F22*C24/(D24*E24))*(1+E22)*C22*G18)*(1+D22)</f>
         <v>38.52747636363637</v>
       </c>
-      <c r="D23" s="201" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="46">
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="L4:N4"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
+  <mergeCells count="12">
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B19:I19"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="B12:N12"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="B11:N11"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="E18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>

</xml_diff>